<commit_message>
FIX #115: Import client data update (new POI from 15 cities)
- zakopane.xlsx: 77 -> 83 POI, fix newline-separated tags in 7 rows, fix 'rano' -> 'morning'
- multi_city_attractions.xlsx: rebuilt all 15 cities (678 rows, 44 cols, All Cities sheet)
- tag_preferences.py: add 70+ new tags (FIX #115) to all preference groups
- excel_validator.py: add same tags to _KNOWN_TAGS (334 -> 155 validation errors)
- load_restaurants.py: update path to planer_update/Planer - restauracje.xlsx
</commit_message>
<xml_diff>
--- a/data/zakopane.xlsx
+++ b/data/zakopane.xlsx
@@ -17,18 +17,15 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,22 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -429,226 +416,226 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR78"/>
+  <dimension ref="A1:AR84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>image_key</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Description_short</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Description_long</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Why visit</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Opening hours</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>opening_hours_seasonal</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>time_min</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>time_max</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ticket_normal</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ticket_reduced</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Lat</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Lng</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Link do godzin</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Link do cennika</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Space</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Intensity</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>weather_dependency</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>popularity_score</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Must see score</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Peak hours</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>recommended_time_of_day</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t xml:space="preserve">Target group </t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t xml:space="preserve">Children's age </t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Type of attraction</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Activity_style</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>crowd_level</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t xml:space="preserve">Budget type </t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Seasonality of attractions</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>Pro_tip</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>parking_name</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>parking_address</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>parking_lat</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>parking_lng</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>parking_type</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>parking_walk_time_min</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>priority_level</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>kids_only</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
@@ -735,11 +722,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P2" t="n">
-        <v>49.2953934</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>19.9638039</v>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>49.29539340</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>19.96380390</t>
+        </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -837,11 +828,15 @@
           <t>Jagiellońska 31, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL2" t="n">
-        <v>49.29527714748905</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>19.96450238217657</v>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>49.29527714748905</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>19.96450238217657</t>
+        </is>
       </c>
       <c r="AN2" t="inlineStr">
         <is>
@@ -937,11 +932,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P3" t="n">
-        <v>49.2864315</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>19.9621711</v>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>49.28643150</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>19.96217110</t>
+        </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -1039,11 +1038,15 @@
           <t>Józefa Piłsudskiego 51, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL3" t="n">
-        <v>49.28637200796405</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>19.96220234068982</v>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>49.28637200796405</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>19.962202340689817</t>
+        </is>
       </c>
       <c r="AN3" t="inlineStr">
         <is>
@@ -1140,11 +1143,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P4" t="n">
-        <v>49.2916215</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>19.9604081</v>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>49.29162150</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>19.96040810</t>
+        </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -1242,11 +1249,15 @@
           <t>34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL4" t="n">
-        <v>49.29327022308206</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>19.95807655548775</v>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>49.29327022308206</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>19.95807655548775</t>
+        </is>
       </c>
       <c r="AN4" t="inlineStr">
         <is>
@@ -1341,11 +1352,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P5" t="n">
-        <v>49.2949039</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>19.9504388</v>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>49.29490390</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>19.95043880</t>
+        </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1443,11 +1458,15 @@
           <t>Mariusza Zaruskiego 1, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL5" t="n">
-        <v>49.29433237891199</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>19.95166160881956</v>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>49.29433237891199</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>19.951661608819556</t>
+        </is>
       </c>
       <c r="AN5" t="inlineStr">
         <is>
@@ -1543,11 +1562,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P6" t="n">
-        <v>49.2876722</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>19.9799362</v>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>49.28767220</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>19.97993620</t>
+        </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1645,11 +1668,15 @@
           <t>Droga do Olczy 11, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL6" t="n">
-        <v>49.28768470927717</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>19.97993464078015</v>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>49.28768470927717</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>19.979934640780147</t>
+        </is>
       </c>
       <c r="AN6" t="inlineStr">
         <is>
@@ -1744,11 +1771,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P7" t="n">
-        <v>49.2943257</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>19.9368506</v>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>49.29432570</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>19.93685060</t>
+        </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1846,11 +1877,15 @@
           <t>Powstańców Śląskich 11, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL7" t="n">
-        <v>49.29417049287513</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>19.93704701555601</v>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>49.29417049287513</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>19.937047015556008</t>
+        </is>
       </c>
       <c r="AN7" t="inlineStr">
         <is>
@@ -1946,11 +1981,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P8" t="n">
-        <v>49.2800904</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>19.9632539</v>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>49.28009040</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>19.96325390</t>
+        </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -2003,7 +2042,7 @@
           <t>friends, family_kids</t>
         </is>
       </c>
-      <c r="AC8" s="3" t="n">
+      <c r="AC8" s="1" t="n">
         <v>45944</v>
       </c>
       <c r="AD8" t="inlineStr">
@@ -2047,11 +2086,15 @@
           <t>Józefa Piłsudskiego 28-32, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL8" t="n">
-        <v>49.28225573159638</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>19.96448295394309</v>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>49.28225573159638</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>19.964482953943094</t>
+        </is>
       </c>
       <c r="AN8" t="inlineStr">
         <is>
@@ -2147,11 +2190,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P9" t="n">
-        <v>49.2981174</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>19.9456043</v>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>49.29811740</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>19.94560430</t>
+        </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -2251,11 +2298,15 @@
           <t>Szkolna 2a, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL9" t="n">
-        <v>49.29884500451914</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>19.9471063337796</v>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>49.29884500451914</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>19.947106333779605</t>
+        </is>
       </c>
       <c r="AN9" t="inlineStr">
         <is>
@@ -2349,11 +2400,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P10" t="n">
-        <v>49.3050438</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>19.9660141</v>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>49.30504380</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>19.96601410</t>
+        </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -2452,11 +2507,15 @@
           <t>Szymony 17B, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL10" t="n">
-        <v>49.30482967453035</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>19.96605689192144</v>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>49.30482967453035</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>19.966056891921436</t>
+        </is>
       </c>
       <c r="AN10" t="inlineStr">
         <is>
@@ -2550,11 +2609,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P11" t="n">
-        <v>49.2950159</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>19.9512991</v>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>49.29501590</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>19.95129910</t>
+        </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -2652,11 +2715,15 @@
           <t>Szkolna 2a, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL11" t="n">
-        <v>49.29884500451914</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>19.9471063337796</v>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>49.29884500451914</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>19.947106333779605</t>
+        </is>
       </c>
       <c r="AN11" t="inlineStr">
         <is>
@@ -2745,11 +2812,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P12" t="n">
-        <v>49.283815</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>19.9644304</v>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>49.28381500</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>19.96443040</t>
+        </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2848,11 +2919,15 @@
           <t>Karola Szymanowskiego k/17, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL12" t="n">
-        <v>49.28371636121852</v>
-      </c>
-      <c r="AM12" t="n">
-        <v>19.9649332003545</v>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>49.28371636121852</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>19.964933200354505</t>
+        </is>
       </c>
       <c r="AN12" t="inlineStr">
         <is>
@@ -2946,11 +3021,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P13" t="n">
-        <v>49.2957417</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>19.9528545</v>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>49.29574170</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>19.95285450</t>
+        </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -3048,11 +3127,15 @@
           <t>Tadeusza Kościuszki 3, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL13" t="n">
-        <v>49.29563664460791</v>
-      </c>
-      <c r="AM13" t="n">
-        <v>19.95302614085424</v>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>49.29563664460791</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>19.953026140854238</t>
+        </is>
       </c>
       <c r="AN13" t="inlineStr">
         <is>
@@ -3146,11 +3229,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P14" t="n">
-        <v>49.2939691</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>19.957179</v>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>49.29396910</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>19.95717900</t>
+        </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -3248,11 +3335,15 @@
           <t>Aleje 3-go Maja, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL14" t="n">
-        <v>49.29421509759925</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>19.95656167049711</v>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>49.29421509759925</t>
+        </is>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>19.956561670497106</t>
+        </is>
       </c>
       <c r="AN14" t="inlineStr">
         <is>
@@ -3341,11 +3432,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P15" t="n">
-        <v>49.2937448</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>19.9596661</v>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>49.29374480</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>19.95966610</t>
+        </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -3443,11 +3538,15 @@
           <t>Aleje 3-go Maja 9, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL15" t="n">
-        <v>49.29324569432775</v>
-      </c>
-      <c r="AM15" t="n">
-        <v>19.95822072085884</v>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>49.29324569432775</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>19.958220720858836</t>
+        </is>
       </c>
       <c r="AN15" t="inlineStr">
         <is>
@@ -3541,11 +3640,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P16" t="n">
-        <v>49.2951046</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>19.9656424</v>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>49.29510460</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>19.96564240</t>
+        </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
@@ -3643,11 +3746,15 @@
           <t>Jagiellońska 31, 34-500 Zakopane, Poland</t>
         </is>
       </c>
-      <c r="AL16" t="n">
-        <v>49.29485863239372</v>
-      </c>
-      <c r="AM16" t="n">
-        <v>19.96470030891096</v>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>49.29485863239372</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>19.964700308910963</t>
+        </is>
       </c>
       <c r="AN16" t="inlineStr">
         <is>
@@ -3742,11 +3849,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P17" t="n">
-        <v>49.3999583</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>20.0225918</v>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>49.39995830</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>20.02259180</t>
+        </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
@@ -3844,11 +3955,15 @@
           <t>os. Nowe 45, 34-424 Szaflary</t>
         </is>
       </c>
-      <c r="AL17" t="n">
-        <v>49.39962067618252</v>
-      </c>
-      <c r="AM17" t="n">
-        <v>20.02184613839256</v>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t>49.39962067618252</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>20.02184613839256</t>
+        </is>
       </c>
       <c r="AN17" t="inlineStr">
         <is>
@@ -3943,11 +4058,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P18" t="n">
-        <v>49.3518255</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>19.8231199</v>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>49.35182550</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>19.82311990</t>
+        </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
@@ -3987,7 +4106,7 @@
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>morning, midday, afternoon</t>
+          <t>midday, afternoon, evening</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
@@ -4045,11 +4164,15 @@
           <t>315, 34-513 Chochołów</t>
         </is>
       </c>
-      <c r="AL18" t="n">
-        <v>49.3520575535073</v>
-      </c>
-      <c r="AM18" t="n">
-        <v>19.82175897064164</v>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>49.3520575535073</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>19.821758970641643</t>
+        </is>
       </c>
       <c r="AN18" t="inlineStr">
         <is>
@@ -4144,11 +4267,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P19" t="n">
-        <v>49.3878209</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>20.0990954</v>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>49.38782090</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>20.09909540</t>
+        </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
@@ -4188,7 +4315,7 @@
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>morning, midday, afternoon</t>
+          <t>midday, afternoon, evening</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr">
@@ -4246,11 +4373,15 @@
           <t>Środkowa 181, 34-405 Białka Tatrzańska, Poland</t>
         </is>
       </c>
-      <c r="AL19" t="n">
-        <v>49.38778654963126</v>
-      </c>
-      <c r="AM19" t="n">
-        <v>20.10039184808332</v>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>49.38778654963126</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>20.100391848083316</t>
+        </is>
       </c>
       <c r="AN19" t="inlineStr">
         <is>
@@ -4344,11 +4475,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P20" t="n">
-        <v>49.3248339</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>20.0940415</v>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>49.32483390</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>20.09404150</t>
+        </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
@@ -4388,7 +4523,7 @@
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>morning, midday, afternoon</t>
+          <t>midday, afternoon, evening</t>
         </is>
       </c>
       <c r="AA20" t="inlineStr">
@@ -4446,11 +4581,15 @@
           <t>Sportowa 22, 34-530 Bukowina Tatrzańska, Poland</t>
         </is>
       </c>
-      <c r="AL20" t="n">
-        <v>49.32500339803969</v>
-      </c>
-      <c r="AM20" t="n">
-        <v>20.09508661679884</v>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>49.32500339803969</t>
+        </is>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>20.09508661679884</t>
+        </is>
       </c>
       <c r="AN20" t="inlineStr">
         <is>
@@ -4545,11 +4684,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P21" t="n">
-        <v>49.2794102</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>19.9639442</v>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>49.27941020</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>19.96394420</t>
+        </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
@@ -4647,11 +4790,15 @@
           <t>Józefa Piłsudskiego 28-32, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL21" t="n">
-        <v>49.28220695693889</v>
-      </c>
-      <c r="AM21" t="n">
-        <v>19.96447342331977</v>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>49.28220695693889</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>19.964473423319767</t>
+        </is>
       </c>
       <c r="AN21" t="inlineStr">
         <is>
@@ -4745,11 +4892,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P22" t="n">
-        <v>49.284941</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>19.9720608</v>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>49.28494100</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>19.97206080</t>
+        </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
@@ -4847,11 +4998,15 @@
           <t>Tytusa Chałubińskiego 42a, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL22" t="n">
-        <v>49.28526190879251</v>
-      </c>
-      <c r="AM22" t="n">
-        <v>19.9716100958812</v>
+      <c r="AL22" t="inlineStr">
+        <is>
+          <t>49.28526190879251</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>19.971610095881204</t>
+        </is>
       </c>
       <c r="AN22" t="inlineStr">
         <is>
@@ -4940,11 +5095,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P23" t="n">
-        <v>49.2912955</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>19.9604778</v>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>49.29129550</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>19.96047780</t>
+        </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
@@ -4994,7 +5153,7 @@
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>solo, couples, friends, family_kids</t>
+          <t xml:space="preserve"> friends, family_kids</t>
         </is>
       </c>
       <c r="AC23" t="inlineStr">
@@ -5042,11 +5201,15 @@
           <t>Aleje 3-go maja, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL23" t="n">
-        <v>49.29251552805412</v>
-      </c>
-      <c r="AM23" t="n">
-        <v>19.95908605418339</v>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>49.29251552805412</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>19.959086054183388</t>
+        </is>
       </c>
       <c r="AN23" t="inlineStr">
         <is>
@@ -5135,11 +5298,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P24" t="n">
-        <v>49.292904</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>19.9560636</v>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>49.29290400</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>19.95606360</t>
+        </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
@@ -5237,11 +5404,15 @@
           <t>plac Niepodległości 5, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL24" t="n">
-        <v>49.29236171073057</v>
-      </c>
-      <c r="AM24" t="n">
-        <v>19.95519221654092</v>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>49.292361710730574</t>
+        </is>
+      </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>19.955192216540915</t>
+        </is>
       </c>
       <c r="AN24" t="inlineStr">
         <is>
@@ -5331,11 +5502,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P25" t="n">
-        <v>49.2949668</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>19.9499116</v>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>49.29496680</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>19.94991160</t>
+        </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
@@ -5388,7 +5563,7 @@
           <t>solo, couples, friends, seniors</t>
         </is>
       </c>
-      <c r="AC25" s="3" t="n">
+      <c r="AC25" s="1" t="n">
         <v>45944</v>
       </c>
       <c r="AD25" t="inlineStr">
@@ -5431,11 +5606,15 @@
           <t>Mariusza Zaruskiego 1, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL25" t="n">
-        <v>49.29429371765401</v>
-      </c>
-      <c r="AM25" t="n">
-        <v>19.95164171402313</v>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>49.294293717654014</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>19.951641714023133</t>
+        </is>
       </c>
       <c r="AN25" t="inlineStr">
         <is>
@@ -5525,11 +5704,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P26" t="n">
-        <v>49.2894914</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>19.9581178</v>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>49.28949140</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>19.95811780</t>
+        </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
@@ -5582,7 +5765,7 @@
           <t>solo, couples, friends, family_kids, seniors</t>
         </is>
       </c>
-      <c r="AC26" s="3" t="n">
+      <c r="AC26" s="1" t="n">
         <v>45944</v>
       </c>
       <c r="AD26" t="inlineStr">
@@ -5625,11 +5808,15 @@
           <t>Kazimierza Przerwy-Tetmajera 17, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL26" t="n">
-        <v>49.28920668357339</v>
-      </c>
-      <c r="AM26" t="n">
-        <v>19.9578271971264</v>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>49.28920668357339</t>
+        </is>
+      </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>19.9578271971264</t>
+        </is>
       </c>
       <c r="AN26" t="inlineStr">
         <is>
@@ -5719,11 +5906,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P27" t="n">
-        <v>49.2943331</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>19.9429691</v>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>49.29433310</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>19.94296910</t>
+        </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
@@ -5776,7 +5967,7 @@
           <t>solo, couples, friends, family_kids, seniors</t>
         </is>
       </c>
-      <c r="AC27" s="3" t="n">
+      <c r="AC27" s="1" t="n">
         <v>45944</v>
       </c>
       <c r="AD27" t="inlineStr">
@@ -5819,11 +6010,15 @@
           <t>Kościeliska 18, 34-500 Zakopane, Poland</t>
         </is>
       </c>
-      <c r="AL27" t="n">
-        <v>49.29423307964222</v>
-      </c>
-      <c r="AM27" t="n">
-        <v>19.94307549195877</v>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>49.29423307964222</t>
+        </is>
+      </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>19.943075491958773</t>
+        </is>
       </c>
       <c r="AN27" t="inlineStr">
         <is>
@@ -5913,11 +6108,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P28" t="n">
-        <v>49.2886803</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>19.9663291</v>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>49.28868030</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>19.96632910</t>
+        </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
@@ -5970,7 +6169,7 @@
           <t>solo, couples, friends, family_kids, seniors</t>
         </is>
       </c>
-      <c r="AC28" s="3" t="n">
+      <c r="AC28" s="1" t="n">
         <v>45944</v>
       </c>
       <c r="AD28" t="inlineStr">
@@ -6013,11 +6212,15 @@
           <t>Hr. Władysława Zamoyskiego 25, 34-500 Zakopane, Poland</t>
         </is>
       </c>
-      <c r="AL28" t="n">
-        <v>49.28876287435649</v>
-      </c>
-      <c r="AM28" t="n">
-        <v>19.9666987218065</v>
+      <c r="AL28" t="inlineStr">
+        <is>
+          <t>49.28876287435649</t>
+        </is>
+      </c>
+      <c r="AM28" t="inlineStr">
+        <is>
+          <t>19.9666987218065</t>
+        </is>
       </c>
       <c r="AN28" t="inlineStr">
         <is>
@@ -6106,11 +6309,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P29" t="n">
-        <v>49.2924196</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>19.9484817</v>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>49.29241960</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>19.94848170</t>
+        </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
@@ -6163,7 +6370,7 @@
           <t>solo, couples, friends, family_kids, seniors</t>
         </is>
       </c>
-      <c r="AC29" s="3" t="n">
+      <c r="AC29" s="1" t="n">
         <v>45944</v>
       </c>
       <c r="AD29" t="inlineStr">
@@ -6206,11 +6413,15 @@
           <t>Ogrodowa 2, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL29" t="n">
-        <v>49.29374981765316</v>
-      </c>
-      <c r="AM29" t="n">
-        <v>19.95176421343834</v>
+      <c r="AL29" t="inlineStr">
+        <is>
+          <t>49.29374981765316</t>
+        </is>
+      </c>
+      <c r="AM29" t="inlineStr">
+        <is>
+          <t>19.95176421343834</t>
+        </is>
       </c>
       <c r="AN29" t="inlineStr">
         <is>
@@ -6300,11 +6511,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P30" t="n">
-        <v>49.2816859</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>19.9623758</v>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>49.28168590</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>19.96237580</t>
+        </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
@@ -6403,11 +6618,15 @@
           <t>Józefa Piłsudskiego 28-32, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL30" t="n">
-        <v>49.28216607253456</v>
-      </c>
-      <c r="AM30" t="n">
-        <v>19.96449449239132</v>
+      <c r="AL30" t="inlineStr">
+        <is>
+          <t>49.28216607253456</t>
+        </is>
+      </c>
+      <c r="AM30" t="inlineStr">
+        <is>
+          <t>19.964494492391324</t>
+        </is>
       </c>
       <c r="AN30" t="inlineStr">
         <is>
@@ -6496,11 +6715,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P31" t="n">
-        <v>49.2842616</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>20.0013828</v>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>49.28426160</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>20.00138280</t>
+        </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
@@ -6598,11 +6821,15 @@
           <t>Droga Oswalda Balzera, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL31" t="n">
-        <v>49.28425502719659</v>
-      </c>
-      <c r="AM31" t="n">
-        <v>20.000749330936</v>
+      <c r="AL31" t="inlineStr">
+        <is>
+          <t>49.28425502719659</t>
+        </is>
+      </c>
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>20.000749330935996</t>
+        </is>
       </c>
       <c r="AN31" t="inlineStr">
         <is>
@@ -6702,11 +6929,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P32" t="n">
-        <v>49.294211</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>19.9517825</v>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>49.29421100</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>19.95178250</t>
+        </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
@@ -6804,11 +7035,15 @@
           <t>34-512 Witów</t>
         </is>
       </c>
-      <c r="AL32" t="n">
-        <v>49.28807813151476</v>
-      </c>
-      <c r="AM32" t="n">
-        <v>19.84804736703877</v>
+      <c r="AL32" t="inlineStr">
+        <is>
+          <t>49.28807813151476</t>
+        </is>
+      </c>
+      <c r="AM32" t="inlineStr">
+        <is>
+          <t>19.848047367038767</t>
+        </is>
       </c>
       <c r="AN32" t="inlineStr">
         <is>
@@ -6918,11 +7153,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P33" t="n">
-        <v>49.2666667</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>19.8333333</v>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>49.26666670</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>19.83333330</t>
+        </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
@@ -7010,11 +7249,15 @@
           <t>34-512 Witów</t>
         </is>
       </c>
-      <c r="AL33" t="n">
-        <v>49.28807813151476</v>
-      </c>
-      <c r="AM33" t="n">
-        <v>19.84804736703877</v>
+      <c r="AL33" t="inlineStr">
+        <is>
+          <t>49.28807813151476</t>
+        </is>
+      </c>
+      <c r="AM33" t="inlineStr">
+        <is>
+          <t>19.848047367038767</t>
+        </is>
       </c>
       <c r="AN33" t="inlineStr">
         <is>
@@ -7125,11 +7368,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P34" t="n">
-        <v>49.25</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>19.8666667</v>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>49.25000000</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>19.86666670</t>
+        </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
@@ -7217,11 +7464,15 @@
           <t>Strzelców Podhalańskich 58, 34-511 Kościelisko</t>
         </is>
       </c>
-      <c r="AL34" t="n">
-        <v>49.27567766423668</v>
-      </c>
-      <c r="AM34" t="n">
-        <v>19.86923843610088</v>
+      <c r="AL34" t="inlineStr">
+        <is>
+          <t>49.275677664236675</t>
+        </is>
+      </c>
+      <c r="AM34" t="inlineStr">
+        <is>
+          <t>19.869238436100883</t>
+        </is>
       </c>
       <c r="AN34" t="inlineStr">
         <is>
@@ -7332,11 +7583,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P35" t="n">
-        <v>49.2607771</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>20.0895038</v>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>49.26077710</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>20.08950380</t>
+        </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
@@ -7424,11 +7679,15 @@
           <t>DW960, 34-532 Brzegi</t>
         </is>
       </c>
-      <c r="AL35" t="n">
-        <v>49.28495541022139</v>
-      </c>
-      <c r="AM35" t="n">
-        <v>20.11278591938301</v>
+      <c r="AL35" t="inlineStr">
+        <is>
+          <t>49.28495541022139</t>
+        </is>
+      </c>
+      <c r="AM35" t="inlineStr">
+        <is>
+          <t>20.112785919383015</t>
+        </is>
       </c>
       <c r="AN35" t="inlineStr">
         <is>
@@ -7539,11 +7798,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P36" t="n">
-        <v>49.1971411</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>20.070087</v>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>49.19714110</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>20.07008700</t>
+        </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
@@ -7631,11 +7894,15 @@
           <t>Droga Oswalda Balzera, 34-532 Brzegi</t>
         </is>
       </c>
-      <c r="AL36" t="n">
-        <v>49.25627181318524</v>
-      </c>
-      <c r="AM36" t="n">
-        <v>20.10349998425671</v>
+      <c r="AL36" t="inlineStr">
+        <is>
+          <t>49.25627181318524</t>
+        </is>
+      </c>
+      <c r="AM36" t="inlineStr">
+        <is>
+          <t>20.10349998425671</t>
+        </is>
       </c>
       <c r="AN36" t="inlineStr">
         <is>
@@ -7722,11 +7989,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P37" t="n">
-        <v>49.29866390052654</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>19.9454830120256</v>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>49.29866390052654</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>19.945483012025598</t>
+        </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
@@ -7756,7 +8027,7 @@
       </c>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>morning</t>
+          <t>morning, afternoon</t>
         </is>
       </c>
       <c r="AA37" t="inlineStr">
@@ -7814,11 +8085,15 @@
           <t>Szkolna 2a, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL37" t="n">
-        <v>49.2987097514752</v>
-      </c>
-      <c r="AM37" t="n">
-        <v>19.94708806976537</v>
+      <c r="AL37" t="inlineStr">
+        <is>
+          <t>49.298709751475194</t>
+        </is>
+      </c>
+      <c r="AM37" t="inlineStr">
+        <is>
+          <t>19.947088069765375</t>
+        </is>
       </c>
       <c r="AN37" t="inlineStr">
         <is>
@@ -7906,11 +8181,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P38" t="n">
-        <v>49.3038831</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>19.9128467</v>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>49.30388310</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>19.91284670</t>
+        </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
@@ -7998,11 +8277,15 @@
           <t>Butorów 5, 34-511 Kościelisko</t>
         </is>
       </c>
-      <c r="AL38" t="n">
-        <v>49.30389735001076</v>
-      </c>
-      <c r="AM38" t="n">
-        <v>19.91295267789988</v>
+      <c r="AL38" t="inlineStr">
+        <is>
+          <t>49.30389735001076</t>
+        </is>
+      </c>
+      <c r="AM38" t="inlineStr">
+        <is>
+          <t>19.91295267789988</t>
+        </is>
       </c>
       <c r="AN38" t="inlineStr">
         <is>
@@ -8133,11 +8416,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P39" t="n">
-        <v>49.2693317</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>19.9792181</v>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>49.26933170</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>19.97921810</t>
+        </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
@@ -8235,11 +8522,15 @@
           <t>Przewodników Tatrzańskich 3A, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL39" t="n">
-        <v>49.28096463046775</v>
-      </c>
-      <c r="AM39" t="n">
-        <v>19.97995694820392</v>
+      <c r="AL39" t="inlineStr">
+        <is>
+          <t>49.28096463046775</t>
+        </is>
+      </c>
+      <c r="AM39" t="inlineStr">
+        <is>
+          <t>19.979956948203913</t>
+        </is>
       </c>
       <c r="AN39" t="inlineStr">
         <is>
@@ -8337,11 +8628,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P40" t="n">
-        <v>49.2700957</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>19.9813526</v>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>49.27009570</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>19.98135260</t>
+        </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
@@ -8429,11 +8724,15 @@
           <t>Józefa Piłsudskiego 28-32, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL40" t="n">
-        <v>49.28223989244243</v>
-      </c>
-      <c r="AM40" t="n">
-        <v>19.96474649212863</v>
+      <c r="AL40" t="inlineStr">
+        <is>
+          <t>49.28223989244243</t>
+        </is>
+      </c>
+      <c r="AM40" t="inlineStr">
+        <is>
+          <t>19.964746492128626</t>
+        </is>
       </c>
       <c r="AN40" t="inlineStr">
         <is>
@@ -8531,11 +8830,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P41" t="n">
-        <v>49.2730783</v>
-      </c>
-      <c r="Q41" t="n">
-        <v>19.9333087</v>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>49.27307830</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>19.93330870</t>
+        </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
@@ -8623,11 +8926,15 @@
           <t>Strążyska 39a, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL41" t="n">
-        <v>49.27926359746931</v>
-      </c>
-      <c r="AM41" t="n">
-        <v>19.93880274960191</v>
+      <c r="AL41" t="inlineStr">
+        <is>
+          <t>49.27926359746931</t>
+        </is>
+      </c>
+      <c r="AM41" t="inlineStr">
+        <is>
+          <t>19.93880274960191</t>
+        </is>
       </c>
       <c r="AN41" t="inlineStr">
         <is>
@@ -8725,11 +9032,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P42" t="n">
-        <v>49.2745153</v>
-      </c>
-      <c r="Q42" t="n">
-        <v>19.9411407</v>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>49.27451530</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>19.94114070</t>
+        </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
@@ -8817,11 +9128,15 @@
           <t>Strążyska 39a, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL42" t="n">
-        <v>49.27926359746931</v>
-      </c>
-      <c r="AM42" t="n">
-        <v>19.93880274960191</v>
+      <c r="AL42" t="inlineStr">
+        <is>
+          <t>49.27926359746931</t>
+        </is>
+      </c>
+      <c r="AM42" t="inlineStr">
+        <is>
+          <t>19.93880274960191</t>
+        </is>
       </c>
       <c r="AN42" t="inlineStr">
         <is>
@@ -8919,11 +9234,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P43" t="n">
-        <v>49.2590822</v>
-      </c>
-      <c r="Q43" t="n">
-        <v>19.9683412</v>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>49.25908220</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>19.96834120</t>
+        </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
@@ -9011,11 +9330,15 @@
           <t>Karola Szymanowskiego k/17, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL43" t="n">
-        <v>49.28506314378279</v>
-      </c>
-      <c r="AM43" t="n">
-        <v>19.96497764513334</v>
+      <c r="AL43" t="inlineStr">
+        <is>
+          <t>49.285063143782786</t>
+        </is>
+      </c>
+      <c r="AM43" t="inlineStr">
+        <is>
+          <t>19.96497764513334</t>
+        </is>
       </c>
       <c r="AN43" t="inlineStr">
         <is>
@@ -9113,11 +9436,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P44" t="n">
-        <v>49.3063407</v>
-      </c>
-      <c r="Q44" t="n">
-        <v>20.0107764</v>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>49.30634070</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>20.01077640</t>
+        </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
@@ -9147,7 +9474,7 @@
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>midday</t>
+          <t>midday, afternoon</t>
         </is>
       </c>
       <c r="AA44" t="inlineStr">
@@ -9205,11 +9532,15 @@
           <t>Gawlaki, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL44" t="n">
-        <v>49.30637531505664</v>
-      </c>
-      <c r="AM44" t="n">
-        <v>20.01086836710718</v>
+      <c r="AL44" t="inlineStr">
+        <is>
+          <t>49.306375315056634</t>
+        </is>
+      </c>
+      <c r="AM44" t="inlineStr">
+        <is>
+          <t>20.010868367107186</t>
+        </is>
       </c>
       <c r="AN44" t="inlineStr">
         <is>
@@ -9307,11 +9638,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P45" t="n">
-        <v>49.2594431</v>
-      </c>
-      <c r="Q45" t="n">
-        <v>19.9302071</v>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>49.25944310</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>19.93020710</t>
+        </is>
       </c>
       <c r="T45" t="inlineStr">
         <is>
@@ -9399,11 +9734,15 @@
           <t>Strążyska 39a, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL45" t="n">
-        <v>49.27926359746931</v>
-      </c>
-      <c r="AM45" t="n">
-        <v>19.93880274960191</v>
+      <c r="AL45" t="inlineStr">
+        <is>
+          <t>49.27926359746931</t>
+        </is>
+      </c>
+      <c r="AM45" t="inlineStr">
+        <is>
+          <t>19.93880274960191</t>
+        </is>
       </c>
       <c r="AN45" t="inlineStr">
         <is>
@@ -9501,11 +9840,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P46" t="n">
-        <v>49.267381</v>
-      </c>
-      <c r="Q46" t="n">
-        <v>20.0005687</v>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>49.26738100</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>20.00056870</t>
+        </is>
       </c>
       <c r="T46" t="inlineStr">
         <is>
@@ -9593,11 +9936,15 @@
           <t>Droga Oswalda Balzera, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL46" t="n">
-        <v>49.28383703741373</v>
-      </c>
-      <c r="AM46" t="n">
-        <v>19.99889057463658</v>
+      <c r="AL46" t="inlineStr">
+        <is>
+          <t>49.283837037413726</t>
+        </is>
+      </c>
+      <c r="AM46" t="inlineStr">
+        <is>
+          <t>19.998890574636583</t>
+        </is>
       </c>
       <c r="AN46" t="inlineStr">
         <is>
@@ -9695,11 +10042,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P47" t="n">
-        <v>49.2627558</v>
-      </c>
-      <c r="Q47" t="n">
-        <v>19.9846641</v>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>49.26275580</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>19.98466410</t>
+        </is>
       </c>
       <c r="T47" t="inlineStr">
         <is>
@@ -9787,11 +10138,15 @@
           <t>Przewodników Tatrzańskich 3A, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL47" t="n">
-        <v>49.28096463046775</v>
-      </c>
-      <c r="AM47" t="n">
-        <v>19.97995694820392</v>
+      <c r="AL47" t="inlineStr">
+        <is>
+          <t>49.28096463046775</t>
+        </is>
+      </c>
+      <c r="AM47" t="inlineStr">
+        <is>
+          <t>19.979956948203913</t>
+        </is>
       </c>
       <c r="AN47" t="inlineStr">
         <is>
@@ -9889,11 +10244,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P48" t="n">
-        <v>49.2640999</v>
-      </c>
-      <c r="Q48" t="n">
-        <v>19.9544844</v>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>49.26409990</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>19.95448440</t>
+        </is>
       </c>
       <c r="T48" t="inlineStr">
         <is>
@@ -9981,11 +10340,15 @@
           <t>Przewodników Tatrzańskich 3A, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL48" t="n">
-        <v>49.28096463046775</v>
-      </c>
-      <c r="AM48" t="n">
-        <v>19.97995694820392</v>
+      <c r="AL48" t="inlineStr">
+        <is>
+          <t>49.28096463046775</t>
+        </is>
+      </c>
+      <c r="AM48" t="inlineStr">
+        <is>
+          <t>19.979956948203913</t>
+        </is>
       </c>
       <c r="AN48" t="inlineStr">
         <is>
@@ -10083,11 +10446,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P49" t="n">
-        <v>49.2597575</v>
-      </c>
-      <c r="Q49" t="n">
-        <v>19.9043787</v>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>49.25975750</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>19.90437870</t>
+        </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
@@ -10175,11 +10542,15 @@
           <t>Mała Łąka, 34-511 Kościelisko</t>
         </is>
       </c>
-      <c r="AL49" t="n">
-        <v>49.27814106285203</v>
-      </c>
-      <c r="AM49" t="n">
-        <v>19.90469034171385</v>
+      <c r="AL49" t="inlineStr">
+        <is>
+          <t>49.27814106285203</t>
+        </is>
+      </c>
+      <c r="AM49" t="inlineStr">
+        <is>
+          <t>19.90469034171385</t>
+        </is>
       </c>
       <c r="AN49" t="inlineStr">
         <is>
@@ -10277,11 +10648,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P50" t="n">
-        <v>49.270927</v>
-      </c>
-      <c r="Q50" t="n">
-        <v>19.9171668</v>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>49.27092700</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>19.91716680</t>
+        </is>
       </c>
       <c r="T50" t="inlineStr">
         <is>
@@ -10369,11 +10744,15 @@
           <t>Mała Łąka, 34-511 Kościelisko</t>
         </is>
       </c>
-      <c r="AL50" t="n">
-        <v>49.27814106285203</v>
-      </c>
-      <c r="AM50" t="n">
-        <v>19.90469034171385</v>
+      <c r="AL50" t="inlineStr">
+        <is>
+          <t>49.27814106285203</t>
+        </is>
+      </c>
+      <c r="AM50" t="inlineStr">
+        <is>
+          <t>19.90469034171385</t>
+        </is>
       </c>
       <c r="AN50" t="inlineStr">
         <is>
@@ -10471,11 +10850,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P51" t="n">
-        <v>49.283438</v>
-      </c>
-      <c r="Q51" t="n">
-        <v>20.0359096</v>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>49.28343800</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>20.03590960</t>
+        </is>
       </c>
       <c r="T51" t="inlineStr">
         <is>
@@ -10563,11 +10946,15 @@
           <t>Cyrhla 26C, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL51" t="n">
-        <v>49.28887603692906</v>
-      </c>
-      <c r="AM51" t="n">
-        <v>20.01327133489216</v>
+      <c r="AL51" t="inlineStr">
+        <is>
+          <t>49.28887603692906</t>
+        </is>
+      </c>
+      <c r="AM51" t="inlineStr">
+        <is>
+          <t>20.013271334892163</t>
+        </is>
       </c>
       <c r="AN51" t="inlineStr">
         <is>
@@ -10665,11 +11052,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P52" t="n">
-        <v>49.2454853</v>
-      </c>
-      <c r="Q52" t="n">
-        <v>20.0063853</v>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>49.24548530</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>20.00638530</t>
+        </is>
       </c>
       <c r="T52" t="inlineStr">
         <is>
@@ -10757,11 +11148,15 @@
           <t>Bronisława Czecha 1, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL52" t="n">
-        <v>49.2840161893837</v>
-      </c>
-      <c r="AM52" t="n">
-        <v>19.9727495819826</v>
+      <c r="AL52" t="inlineStr">
+        <is>
+          <t>49.2840161893837</t>
+        </is>
+      </c>
+      <c r="AM52" t="inlineStr">
+        <is>
+          <t>19.9727495819826</t>
+        </is>
       </c>
       <c r="AN52" t="inlineStr">
         <is>
@@ -10859,11 +11254,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P53" t="n">
-        <v>49.291268</v>
-      </c>
-      <c r="Q53" t="n">
-        <v>19.95507</v>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>49.29126800</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>19.95507000</t>
+        </is>
       </c>
       <c r="T53" t="inlineStr">
         <is>
@@ -10893,7 +11292,7 @@
       </c>
       <c r="Z53" t="inlineStr">
         <is>
-          <t>midday</t>
+          <t>midday, afternoon, evening</t>
         </is>
       </c>
       <c r="AA53" t="inlineStr">
@@ -10951,11 +11350,15 @@
           <t>plac Niepodległości 5, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL53" t="n">
-        <v>49.29235931950797</v>
-      </c>
-      <c r="AM53" t="n">
-        <v>19.95539991222302</v>
+      <c r="AL53" t="inlineStr">
+        <is>
+          <t>49.292359319507966</t>
+        </is>
+      </c>
+      <c r="AM53" t="inlineStr">
+        <is>
+          <t>19.955399912223026</t>
+        </is>
       </c>
       <c r="AN53" t="inlineStr">
         <is>
@@ -11042,11 +11445,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P54" t="n">
-        <v>49.2796428</v>
-      </c>
-      <c r="Q54" t="n">
-        <v>19.9193173</v>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>49.27964280</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>19.91931730</t>
+        </is>
       </c>
       <c r="T54" t="inlineStr">
         <is>
@@ -11134,11 +11541,15 @@
           <t>Osiedle Krzeptówki 17, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL54" t="n">
-        <v>49.27966870849051</v>
-      </c>
-      <c r="AM54" t="n">
-        <v>19.91938420791758</v>
+      <c r="AL54" t="inlineStr">
+        <is>
+          <t>49.27966870849051</t>
+        </is>
+      </c>
+      <c r="AM54" t="inlineStr">
+        <is>
+          <t>19.91938420791758</t>
+        </is>
       </c>
       <c r="AN54" t="inlineStr">
         <is>
@@ -11225,11 +11636,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P55" t="n">
-        <v>49.3213574</v>
-      </c>
-      <c r="Q55" t="n">
-        <v>19.9937334</v>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>49.32135740</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>19.99373340</t>
+        </is>
       </c>
       <c r="T55" t="inlineStr">
         <is>
@@ -11317,11 +11732,15 @@
           <t>Tadeusza Kościuszki 60, 34-520 Poronin</t>
         </is>
       </c>
-      <c r="AL55" t="n">
-        <v>49.32138166487979</v>
-      </c>
-      <c r="AM55" t="n">
-        <v>19.99388002584367</v>
+      <c r="AL55" t="inlineStr">
+        <is>
+          <t>49.321381664879794</t>
+        </is>
+      </c>
+      <c r="AM55" t="inlineStr">
+        <is>
+          <t>19.99388002584367</t>
+        </is>
       </c>
       <c r="AN55" t="inlineStr">
         <is>
@@ -11414,11 +11833,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P56" t="n">
-        <v>49.263544</v>
-      </c>
-      <c r="Q56" t="n">
-        <v>19.8693207</v>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>49.26354400</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>19.86932070</t>
+        </is>
       </c>
       <c r="T56" t="inlineStr">
         <is>
@@ -11506,11 +11929,15 @@
           <t>Strzelców Podhalańskich 58, 43-229 Kościelisko</t>
         </is>
       </c>
-      <c r="AL56" t="n">
-        <v>49.27569585477032</v>
-      </c>
-      <c r="AM56" t="n">
-        <v>19.86924254127315</v>
+      <c r="AL56" t="inlineStr">
+        <is>
+          <t>49.27569585477032</t>
+        </is>
+      </c>
+      <c r="AM56" t="inlineStr">
+        <is>
+          <t>19.86924254127315</t>
+        </is>
       </c>
       <c r="AN56" t="inlineStr">
         <is>
@@ -11597,11 +12024,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P57" t="n">
-        <v>49.2900847</v>
-      </c>
-      <c r="Q57" t="n">
-        <v>19.9623495</v>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>49.29008470</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>19.96234950</t>
+        </is>
       </c>
       <c r="T57" t="inlineStr">
         <is>
@@ -11689,11 +12120,15 @@
           <t>Kazimierza Przerwy-Tetmajera 17, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL57" t="n">
-        <v>49.28921018246771</v>
-      </c>
-      <c r="AM57" t="n">
-        <v>19.95777058756633</v>
+      <c r="AL57" t="inlineStr">
+        <is>
+          <t>49.289210182467706</t>
+        </is>
+      </c>
+      <c r="AM57" t="inlineStr">
+        <is>
+          <t>19.95777058756633</t>
+        </is>
       </c>
       <c r="AN57" t="inlineStr">
         <is>
@@ -11780,11 +12215,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P58" t="n">
-        <v>49.2851264</v>
-      </c>
-      <c r="Q58" t="n">
-        <v>19.9563019</v>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>49.28512640</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>19.95630190</t>
+        </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
@@ -11882,11 +12321,15 @@
           <t>Droga Do Białego 3, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL58" t="n">
-        <v>49.28516713534483</v>
-      </c>
-      <c r="AM58" t="n">
-        <v>19.95627984758001</v>
+      <c r="AL58" t="inlineStr">
+        <is>
+          <t>49.28516713534483</t>
+        </is>
+      </c>
+      <c r="AM58" t="inlineStr">
+        <is>
+          <t>19.95627984758001</t>
+        </is>
       </c>
       <c r="AN58" t="inlineStr">
         <is>
@@ -11984,11 +12427,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P59" t="n">
-        <v>49.3027368</v>
-      </c>
-      <c r="Q59" t="n">
-        <v>20.1174987</v>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>49.30273680</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>20.11749870</t>
+        </is>
       </c>
       <c r="T59" t="inlineStr">
         <is>
@@ -12076,11 +12523,15 @@
           <t>Głodówka 10a, 34-532 Brzegi</t>
         </is>
       </c>
-      <c r="AL59" t="n">
-        <v>49.3022252254619</v>
-      </c>
-      <c r="AM59" t="n">
-        <v>20.11448030212592</v>
+      <c r="AL59" t="inlineStr">
+        <is>
+          <t>49.302225225461896</t>
+        </is>
+      </c>
+      <c r="AM59" t="inlineStr">
+        <is>
+          <t>20.11448030212592</t>
+        </is>
       </c>
       <c r="AN59" t="inlineStr">
         <is>
@@ -12167,11 +12618,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P60" t="n">
-        <v>49.3057976</v>
-      </c>
-      <c r="Q60" t="n">
-        <v>19.9310972</v>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>49.30579760</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>19.93109720</t>
+        </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
@@ -12264,11 +12719,15 @@
           <t>34-511 Kościelisko</t>
         </is>
       </c>
-      <c r="AL60" t="n">
-        <v>49.30376356582092</v>
-      </c>
-      <c r="AM60" t="n">
-        <v>19.91163754360958</v>
+      <c r="AL60" t="inlineStr">
+        <is>
+          <t>49.303763565820915</t>
+        </is>
+      </c>
+      <c r="AM60" t="inlineStr">
+        <is>
+          <t>19.911637543609586</t>
+        </is>
       </c>
       <c r="AN60" t="inlineStr">
         <is>
@@ -12355,11 +12814,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P61" t="n">
-        <v>49.2965934</v>
-      </c>
-      <c r="Q61" t="n">
-        <v>19.9470409</v>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>49.29659340</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>19.94704090</t>
+        </is>
       </c>
       <c r="T61" t="inlineStr">
         <is>
@@ -12389,7 +12852,7 @@
       </c>
       <c r="Z61" t="inlineStr">
         <is>
-          <t>midday</t>
+          <t>midday, afternoon</t>
         </is>
       </c>
       <c r="AA61" t="inlineStr">
@@ -12447,11 +12910,15 @@
           <t>Kościeliska 3, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL61" t="n">
-        <v>49.29603655458883</v>
-      </c>
-      <c r="AM61" t="n">
-        <v>19.94723204904453</v>
+      <c r="AL61" t="inlineStr">
+        <is>
+          <t>49.29603655458883</t>
+        </is>
+      </c>
+      <c r="AM61" t="inlineStr">
+        <is>
+          <t>19.94723204904453</t>
+        </is>
       </c>
       <c r="AN61" t="inlineStr">
         <is>
@@ -12538,11 +13005,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P62" t="n">
-        <v>49.4739253</v>
-      </c>
-      <c r="Q62" t="n">
-        <v>20.1277911</v>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>49.47392530</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>20.12779110</t>
+        </is>
       </c>
       <c r="T62" t="inlineStr">
         <is>
@@ -12630,11 +13101,15 @@
           <t>Gorczańska 2, 34-432 Łopuszna</t>
         </is>
       </c>
-      <c r="AL62" t="n">
-        <v>49.4739885406501</v>
-      </c>
-      <c r="AM62" t="n">
-        <v>20.12820359660578</v>
+      <c r="AL62" t="inlineStr">
+        <is>
+          <t>49.4739885406501</t>
+        </is>
+      </c>
+      <c r="AM62" t="inlineStr">
+        <is>
+          <t>20.12820359660578</t>
+        </is>
       </c>
       <c r="AN62" t="inlineStr">
         <is>
@@ -12721,11 +13196,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P63" t="n">
-        <v>49.2652077</v>
-      </c>
-      <c r="Q63" t="n">
-        <v>20.086447</v>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>49.26520770</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>20.08644700</t>
+        </is>
       </c>
       <c r="T63" t="inlineStr">
         <is>
@@ -12813,11 +13292,15 @@
           <t>DW960, 34-532 Brzegi</t>
         </is>
       </c>
-      <c r="AL63" t="n">
-        <v>49.28487689876398</v>
-      </c>
-      <c r="AM63" t="n">
-        <v>20.11278195551806</v>
+      <c r="AL63" t="inlineStr">
+        <is>
+          <t>49.284876898763976</t>
+        </is>
+      </c>
+      <c r="AM63" t="inlineStr">
+        <is>
+          <t>20.112781955518063</t>
+        </is>
       </c>
       <c r="AN63" t="inlineStr">
         <is>
@@ -12900,11 +13383,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P64" t="n">
-        <v>49.3054734</v>
-      </c>
-      <c r="Q64" t="n">
-        <v>19.9045138</v>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>49.30547340</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>19.90451380</t>
+        </is>
       </c>
       <c r="T64" t="inlineStr">
         <is>
@@ -12992,11 +13479,15 @@
           <t>Droga Zubka, 34-511 Kościelisko</t>
         </is>
       </c>
-      <c r="AL64" t="n">
-        <v>49.30355974561837</v>
-      </c>
-      <c r="AM64" t="n">
-        <v>19.91181090231959</v>
+      <c r="AL64" t="inlineStr">
+        <is>
+          <t>49.303559745618365</t>
+        </is>
+      </c>
+      <c r="AM64" t="inlineStr">
+        <is>
+          <t>19.91181090231959</t>
+        </is>
       </c>
       <c r="AN64" t="inlineStr">
         <is>
@@ -13083,11 +13574,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P65" t="n">
-        <v>49.2938545</v>
-      </c>
-      <c r="Q65" t="n">
-        <v>19.9538936</v>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>49.29385450</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>19.95389360</t>
+        </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
@@ -13127,7 +13622,7 @@
       </c>
       <c r="Z65" t="inlineStr">
         <is>
-          <t>evening</t>
+          <t>afternoon, evening</t>
         </is>
       </c>
       <c r="AA65" t="inlineStr">
@@ -13185,11 +13680,15 @@
           <t>plac Niepodległości 5, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL65" t="n">
-        <v>49.29250342378384</v>
-      </c>
-      <c r="AM65" t="n">
-        <v>19.95545798391481</v>
+      <c r="AL65" t="inlineStr">
+        <is>
+          <t>49.292503423783835</t>
+        </is>
+      </c>
+      <c r="AM65" t="inlineStr">
+        <is>
+          <t>19.955457983914812</t>
+        </is>
       </c>
       <c r="AN65" t="inlineStr">
         <is>
@@ -13209,7 +13708,7 @@
       </c>
       <c r="AR65" t="inlineStr">
         <is>
-          <t>street_food,food_market,lively_atmosphere,central_location</t>
+          <t>street_food,food_market,lively_atmosphere,central_location, evening_activity, walking, local_food_experience, shopping, relaxation</t>
         </is>
       </c>
     </row>
@@ -13287,11 +13786,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P66" t="n">
-        <v>49.2958592</v>
-      </c>
-      <c r="Q66" t="n">
-        <v>19.9559261</v>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>49.29585920</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>19.95592610</t>
+        </is>
       </c>
       <c r="T66" t="inlineStr">
         <is>
@@ -13321,7 +13824,7 @@
       </c>
       <c r="Z66" t="inlineStr">
         <is>
-          <t>evening</t>
+          <t>afternoon, evening</t>
         </is>
       </c>
       <c r="AA66" t="inlineStr">
@@ -13379,11 +13882,15 @@
           <t>Tadeusza Kościuszki 3, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL66" t="n">
-        <v>49.2955352233874</v>
-      </c>
-      <c r="AM66" t="n">
-        <v>19.95316800109384</v>
+      <c r="AL66" t="inlineStr">
+        <is>
+          <t>49.2955352233874</t>
+        </is>
+      </c>
+      <c r="AM66" t="inlineStr">
+        <is>
+          <t>19.953168001093836</t>
+        </is>
       </c>
       <c r="AN66" t="inlineStr">
         <is>
@@ -13403,7 +13910,7 @@
       </c>
       <c r="AR66" t="inlineStr">
         <is>
-          <t>meadows_fields,scenic_walk,quiet_relax_spot</t>
+          <t>meadows_fields,scenic_walk,quiet_relax_spot, walking, relaxation, seniors, family_friendly, evening_activity</t>
         </is>
       </c>
     </row>
@@ -13470,11 +13977,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P67" t="n">
-        <v>49.3178921</v>
-      </c>
-      <c r="Q67" t="n">
-        <v>19.9797066</v>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>49.31789210</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>19.97970660</t>
+        </is>
       </c>
       <c r="R67" t="inlineStr">
         <is>
@@ -13572,11 +14083,15 @@
           <t>Harenda 12A, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL67" t="n">
-        <v>49.31811586981819</v>
-      </c>
-      <c r="AM67" t="n">
-        <v>19.97979242737103</v>
+      <c r="AL67" t="inlineStr">
+        <is>
+          <t>49.318115869818186</t>
+        </is>
+      </c>
+      <c r="AM67" t="inlineStr">
+        <is>
+          <t>19.979792427371027</t>
+        </is>
       </c>
       <c r="AN67" t="inlineStr">
         <is>
@@ -13663,11 +14178,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P68" t="n">
-        <v>49.2942647</v>
-      </c>
-      <c r="Q68" t="n">
-        <v>19.9428375</v>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>49.29426470</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>19.94283750</t>
+        </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
@@ -13765,11 +14284,15 @@
           <t>Kościeliska 3, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL68" t="n">
-        <v>49.29613380235063</v>
-      </c>
-      <c r="AM68" t="n">
-        <v>19.94727608705408</v>
+      <c r="AL68" t="inlineStr">
+        <is>
+          <t>49.29613380235063</t>
+        </is>
+      </c>
+      <c r="AM68" t="inlineStr">
+        <is>
+          <t>19.94727608705408</t>
+        </is>
       </c>
       <c r="AN68" t="inlineStr">
         <is>
@@ -13867,11 +14390,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P69" t="n">
-        <v>49.2961476</v>
-      </c>
-      <c r="Q69" t="n">
-        <v>19.9464968</v>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>49.29614760</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>19.94649680</t>
+        </is>
       </c>
       <c r="T69" t="inlineStr">
         <is>
@@ -13959,11 +14486,15 @@
           <t>Kościeliska 3, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL69" t="n">
-        <v>49.29613380235063</v>
-      </c>
-      <c r="AM69" t="n">
-        <v>19.94727608705408</v>
+      <c r="AL69" t="inlineStr">
+        <is>
+          <t>49.29613380235063</t>
+        </is>
+      </c>
+      <c r="AM69" t="inlineStr">
+        <is>
+          <t>19.94727608705408</t>
+        </is>
       </c>
       <c r="AN69" t="inlineStr">
         <is>
@@ -14050,11 +14581,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P70" t="n">
-        <v>49.2968874</v>
-      </c>
-      <c r="Q70" t="n">
-        <v>19.9618881</v>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>49.29688740</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>19.96188810</t>
+        </is>
       </c>
       <c r="R70" t="inlineStr">
         <is>
@@ -14152,11 +14687,15 @@
           <t>Jagiellońska 18b, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL70" t="n">
-        <v>49.29690569316998</v>
-      </c>
-      <c r="AM70" t="n">
-        <v>19.96194098437152</v>
+      <c r="AL70" t="inlineStr">
+        <is>
+          <t>49.296905693169975</t>
+        </is>
+      </c>
+      <c r="AM70" t="inlineStr">
+        <is>
+          <t>19.961940984371523</t>
+        </is>
       </c>
       <c r="AN70" t="inlineStr">
         <is>
@@ -14276,11 +14815,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P71" t="n">
-        <v>49.3070021</v>
-      </c>
-      <c r="Q71" t="n">
-        <v>20.0890354</v>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>49.30700210</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>20.08903540</t>
+        </is>
       </c>
       <c r="R71" t="inlineStr">
         <is>
@@ -14378,11 +14921,15 @@
           <t>34-531 Małe Ciche</t>
         </is>
       </c>
-      <c r="AL71" t="n">
-        <v>49.30638175276096</v>
-      </c>
-      <c r="AM71" t="n">
-        <v>20.09014884289007</v>
+      <c r="AL71" t="inlineStr">
+        <is>
+          <t>49.306381752760956</t>
+        </is>
+      </c>
+      <c r="AM71" t="inlineStr">
+        <is>
+          <t>20.09014884289007</t>
+        </is>
       </c>
       <c r="AN71" t="inlineStr">
         <is>
@@ -14469,11 +15016,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P72" t="n">
-        <v>49.2923889</v>
-      </c>
-      <c r="Q72" t="n">
-        <v>19.9596746</v>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>49.29238890</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>19.95967460</t>
+        </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
@@ -14571,11 +15122,15 @@
           <t>Al. 3-go Maja 9, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL72" t="n">
-        <v>49.29314453205548</v>
-      </c>
-      <c r="AM72" t="n">
-        <v>19.95805058231904</v>
+      <c r="AL72" t="inlineStr">
+        <is>
+          <t>49.29314453205548</t>
+        </is>
+      </c>
+      <c r="AM72" t="inlineStr">
+        <is>
+          <t>19.95805058231904</t>
+        </is>
       </c>
       <c r="AN72" t="inlineStr">
         <is>
@@ -14673,11 +15228,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P73" t="n">
-        <v>49.292889</v>
-      </c>
-      <c r="Q73" t="n">
-        <v>19.9296709</v>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>49.29288900</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>19.92967090</t>
+        </is>
       </c>
       <c r="S73" t="inlineStr">
         <is>
@@ -14770,11 +15329,15 @@
           <t>Szymaszkowa 2, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL73" t="n">
-        <v>49.29344366273254</v>
-      </c>
-      <c r="AM73" t="n">
-        <v>19.92925550244357</v>
+      <c r="AL73" t="inlineStr">
+        <is>
+          <t>49.29344366273254</t>
+        </is>
+      </c>
+      <c r="AM73" t="inlineStr">
+        <is>
+          <t>19.929255502443567</t>
+        </is>
       </c>
       <c r="AN73" t="inlineStr">
         <is>
@@ -14861,11 +15424,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P74" t="n">
-        <v>49.2945548</v>
-      </c>
-      <c r="Q74" t="n">
-        <v>19.9532834</v>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>49.29455480</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>19.95328340</t>
+        </is>
       </c>
       <c r="T74" t="inlineStr">
         <is>
@@ -14953,11 +15520,15 @@
           <t>Mariusza Zaruskiego 1, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL74" t="n">
-        <v>49.29429468832737</v>
-      </c>
-      <c r="AM74" t="n">
-        <v>19.95162138420485</v>
+      <c r="AL74" t="inlineStr">
+        <is>
+          <t>49.29429468832737</t>
+        </is>
+      </c>
+      <c r="AM74" t="inlineStr">
+        <is>
+          <t>19.95162138420485</t>
+        </is>
       </c>
       <c r="AN74" t="inlineStr">
         <is>
@@ -15044,11 +15615,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P75" t="n">
-        <v>49.2937321</v>
-      </c>
-      <c r="Q75" t="n">
-        <v>19.9324219</v>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>49.29373210</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>19.93242190</t>
+        </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
@@ -15141,11 +15716,15 @@
           <t>Szymaszkowa 2, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL75" t="n">
-        <v>49.29344366273254</v>
-      </c>
-      <c r="AM75" t="n">
-        <v>19.92925550244357</v>
+      <c r="AL75" t="inlineStr">
+        <is>
+          <t>49.29344366273254</t>
+        </is>
+      </c>
+      <c r="AM75" t="inlineStr">
+        <is>
+          <t>19.929255502443567</t>
+        </is>
       </c>
       <c r="AN75" t="inlineStr">
         <is>
@@ -15232,11 +15811,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P76" t="n">
-        <v>49.3058551</v>
-      </c>
-      <c r="Q76" t="n">
-        <v>19.958669</v>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>49.30585510</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>19.95866900</t>
+        </is>
       </c>
       <c r="T76" t="inlineStr">
         <is>
@@ -15276,7 +15859,7 @@
       </c>
       <c r="AB76" t="inlineStr">
         <is>
-          <t>couples, seniors, friends</t>
+          <t>couples, seniors friends</t>
         </is>
       </c>
       <c r="AD76" t="inlineStr">
@@ -15319,11 +15902,15 @@
           <t>Jana Kasprowicza 1, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL76" t="n">
-        <v>49.30587450712098</v>
-      </c>
-      <c r="AM76" t="n">
-        <v>19.95876895628176</v>
+      <c r="AL76" t="inlineStr">
+        <is>
+          <t>49.30587450712098</t>
+        </is>
+      </c>
+      <c r="AM76" t="inlineStr">
+        <is>
+          <t>19.958768956281755</t>
+        </is>
       </c>
       <c r="AN76" t="inlineStr">
         <is>
@@ -15338,8 +15925,10 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ76" t="b">
-        <v>0</v>
+      <c r="AQ76" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="AR76" t="inlineStr">
         <is>
@@ -15410,11 +15999,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P77" t="n">
-        <v>49.293009</v>
-      </c>
-      <c r="Q77" t="n">
-        <v>19.9549909</v>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>49.29300900</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>19.95499090</t>
+        </is>
       </c>
       <c r="T77" t="inlineStr">
         <is>
@@ -15502,11 +16095,15 @@
           <t>plac Niepodległości 5, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL77" t="n">
-        <v>49.29239844675728</v>
-      </c>
-      <c r="AM77" t="n">
-        <v>19.9551733112919</v>
+      <c r="AL77" t="inlineStr">
+        <is>
+          <t>49.29239844675728</t>
+        </is>
+      </c>
+      <c r="AM77" t="inlineStr">
+        <is>
+          <t>19.955173311291897</t>
+        </is>
       </c>
       <c r="AN77" t="inlineStr">
         <is>
@@ -15521,8 +16118,10 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ77" t="b">
-        <v>0</v>
+      <c r="AQ77" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="AR77" t="inlineStr">
         <is>
@@ -15553,17 +16152,17 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Godziny: 
-sobota 09:00–19:00
-niedziela
-(Zesłanie Ducha Świętego)
-09:00–19:00
-Godziny otwarcia mogą być inne
-poniedziałek 09:00–19:00
-wtorek 09:00–19:00
-środa 09:00–19:00
-czwartek 09:00–19:00
-piątek 09:00–19:00</t>
+          <t>{
+  "date_from": "01-01",
+  "date_to": "12-31",
+  "mon": "09:00-19:00",
+  "tue": "09:00-19:00",
+  "wed": "09:00-19:00",
+  "thu": "09:00-19:00",
+  "fri": "09:00-19:00",
+  "sat": "09:00-19:00",
+  "sun": "09:00-19:00"
+}</t>
         </is>
       </c>
       <c r="I78" t="n">
@@ -15593,11 +16192,15 @@
           <t>Małopolska</t>
         </is>
       </c>
-      <c r="P78" t="n">
-        <v>49.2977911</v>
-      </c>
-      <c r="Q78" t="n">
-        <v>19.9464494</v>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>49.29779110</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>19.94644940</t>
+        </is>
       </c>
       <c r="T78" t="inlineStr">
         <is>
@@ -15680,11 +16283,15 @@
           <t>Szkolna 2a, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="AL78" t="n">
-        <v>49.29880556365436</v>
-      </c>
-      <c r="AM78" t="n">
-        <v>19.94711458413337</v>
+      <c r="AL78" t="inlineStr">
+        <is>
+          <t>49.298805563654355</t>
+        </is>
+      </c>
+      <c r="AM78" t="inlineStr">
+        <is>
+          <t>19.947114584133367</t>
+        </is>
       </c>
       <c r="AN78" t="inlineStr">
         <is>
@@ -15699,12 +16306,1175 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ78" t="b">
+      <c r="AQ78" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AR78" t="inlineStr">
+        <is>
+          <t>food_market, street_food, local_products, souvenirs, regional_food, oscypek, market, local_experience</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Bachledówka</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Bachledówka to malownicze wzniesienie niedaleko Zakopanego. Na szczycie znajduje się sanktuarium, a z okolicy można podziwiać piękne panoramy Tatr i Podhala.</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bachledówka to malownicze wzniesienie na Pogórzu Gubałowskim, położone między Czerwiennem a Ratułowem, zaledwie kilka kilometrów od Zakopanego. Na szczycie znajduje się Sanktuarium na Bachledówce, a z okolicznych polan rozciągają się zachwycające panoramy Tatr, Podhala i Beskidów. </t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>To idealne miejsce na chwilę odpoczynku i podziwianie górskich krajobrazów.</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>{
+  "date_from": "01-01",
+  "date_to": "12-31",
+  "mon": "08:00-22:00",
+  "tue": "08:00-22:00",
+  "wed": "08:00-22:00",
+  "thu": "08:00-22:00",
+  "fri": "08:00-22:00",
+  "sat": "08:00-22:00",
+  "sun": "08:00-22:00"
+}</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>30</v>
+      </c>
+      <c r="J79" t="n">
+        <v>90</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Wstęp bezpłatny</t>
+        </is>
+      </c>
+      <c r="L79" t="n">
         <v>0</v>
       </c>
-      <c r="AR78" t="inlineStr">
-        <is>
-          <t>food_market, street_food, local_products, souvenirs, regional_food, oscypek, market, local_experience</t>
+      <c r="M79" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>Czerwienne 341, 34-407 Czerwienne</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>Małopolska</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>49.374645514748195</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>19.919203962070593</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>outdoor</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>good_weather_only</t>
+        </is>
+      </c>
+      <c r="W79" t="n">
+        <v>5</v>
+      </c>
+      <c r="X79" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>13:00-15:00</t>
+        </is>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>afternoon, evening</t>
+        </is>
+      </c>
+      <c r="AA79" t="inlineStr">
+        <is>
+          <t>Czerwienne</t>
+        </is>
+      </c>
+      <c r="AB79" t="inlineStr">
+        <is>
+          <t>seniors, couples</t>
+        </is>
+      </c>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>nature_landscape</t>
+        </is>
+      </c>
+      <c r="AE79" t="inlineStr">
+        <is>
+          <t>recreational</t>
+        </is>
+      </c>
+      <c r="AF79" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="AG79" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
+      <c r="AH79" t="inlineStr">
+        <is>
+          <t>all_year</t>
+        </is>
+      </c>
+      <c r="AI79" t="inlineStr">
+        <is>
+          <t>Przyjedź tu o wschodzie lub zachodzie słońca. To właśnie wtedy panoramy Tatr i Podhala prezentują się najpiękniej, a na miejscu jest znacznie spokojniej niż w popularnych punktach widokowych wokół Zakopanego.</t>
+        </is>
+      </c>
+      <c r="AJ79" t="inlineStr">
+        <is>
+          <t>Parking na miejscu</t>
+        </is>
+      </c>
+      <c r="AK79" t="inlineStr">
+        <is>
+          <t>Czerwienne 343A, 34-407 Czerwienne</t>
+        </is>
+      </c>
+      <c r="AL79" t="inlineStr">
+        <is>
+          <t>49.37478396691881</t>
+        </is>
+      </c>
+      <c r="AM79" t="inlineStr">
+        <is>
+          <t>19.920829460366576</t>
+        </is>
+      </c>
+      <c r="AN79" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="AO79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP79" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="AQ79" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AR79" t="inlineStr">
+        <is>
+          <t>nature_landscape, viewpoint, relaxation, history_mystery, museum_heritage, panoramic_view, scenic_view</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Toporowa Cyrhla</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Malownicza, spokojna dzielnica Zakopanego położona na wschodnich krańcach miasta, u podnóża Tatr.</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Toporowa Cyrhla to jedna z najwyżej położonych dzielnic Zakopanego, słynąca z pięknych widoków na Tatry i kameralnej atmosfery. Obszar ten jest popularny wśród turystów szukających ciszy oraz miejsc do pieszych wędrówek, oddalonych od zatłoczonego centrum. Znajdują się tu liczne pensjonaty, szlaki piesze oraz przystanek na trasie do Morskiego Oka. To idealne miejsce dla osób ceniących spokój i kontakt z naturą.</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Warto odwiedzić Toporową Cyrhlę ze względu na zapierające dech w piersiach widoki, łatwy dostęp do szlaków oraz spokojną, górską atmosferę z dala od miejskiego zgiełku.</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>{
+  "date_from": "01-01",
+  "date_to": "12-31",
+  "mon": "08:00-22:00",
+  "tue": "08:00-22:00",
+  "wed": "08:00-22:00",
+  "thu": "08:00-22:00",
+  "fri": "08:00-22:00",
+  "sat": "08:00-22:00",
+  "sun": "08:00-22:00"
+}</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>30</v>
+      </c>
+      <c r="J80" t="n">
+        <v>180</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Wstęp bezpłatny</t>
+        </is>
+      </c>
+      <c r="L80" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>Toporowa Cyrhla, 34-531, Poland</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>Małopolska</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>49.29500900</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>20.03824900</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>outdoor</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>good_weather_only</t>
+        </is>
+      </c>
+      <c r="W80" t="n">
+        <v>4</v>
+      </c>
+      <c r="X80" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>12:00-14:00</t>
+        </is>
+      </c>
+      <c r="Z80" t="inlineStr">
+        <is>
+          <t>morning, afternoon, evening</t>
+        </is>
+      </c>
+      <c r="AA80" t="inlineStr">
+        <is>
+          <t>Zakopane</t>
+        </is>
+      </c>
+      <c r="AB80" t="inlineStr">
+        <is>
+          <t>couples, seniors, friends, family_kids, solo</t>
+        </is>
+      </c>
+      <c r="AC80" t="inlineStr">
+        <is>
+          <t>6-10, 10-14</t>
+        </is>
+      </c>
+      <c r="AD80" t="inlineStr">
+        <is>
+          <t>nature_landscape</t>
+        </is>
+      </c>
+      <c r="AE80" t="inlineStr">
+        <is>
+          <t>recreational</t>
+        </is>
+      </c>
+      <c r="AF80" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="AG80" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
+      <c r="AH80" t="inlineStr">
+        <is>
+          <t>all_year</t>
+        </is>
+      </c>
+      <c r="AI80" t="inlineStr">
+        <is>
+          <t>Warto wybrać się na spacer szlakiem prowadzącym na Polanę Kopieniec lub ku Dolinie Suchej Wody – to mniej uczęszczane, malownicze trasy.</t>
+        </is>
+      </c>
+      <c r="AJ80" t="inlineStr">
+        <is>
+          <t>Parking przy bacówce</t>
+        </is>
+      </c>
+      <c r="AK80" t="inlineStr">
+        <is>
+          <t>Sądelska, 34-531 Murzasichle</t>
+        </is>
+      </c>
+      <c r="AL80" t="inlineStr">
+        <is>
+          <t>49.29133520761806</t>
+        </is>
+      </c>
+      <c r="AM80" t="inlineStr">
+        <is>
+          <t>20.03523067578938</t>
+        </is>
+      </c>
+      <c r="AN80" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="AO80" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP80" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="AQ80" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AR80" t="inlineStr">
+        <is>
+          <t>viewpoint, nature_landscape, panoramic_view, scenic_view, relaxation, seniors, couples</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Punkt widokowy na Antałówce</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Punkt widokowy na Antałówce to spokojne miejsce w centrum Zakopanego z piękną panoramą Tatr. Idealne na krótki odpoczynek, zdjęcia lub piknik przy zachodzie słońca.</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Punkt widokowy na Antałówce to jedna z mniej znanych perełek Zakopanego. Z polany rozciąga się piękna panorama Tatr, a dzięki kameralnemu charakterowi można tu odpocząć z dala od tłumów. To doskonałe miejsce na spokojny spacer, chwilę relaksu lub piknik przy zachodzie słońca. Antałówka zachwyca widokami i pozwala odkryć spokojniejsze oblicze stolicy Tatr.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Warto odwiedzić Antałówkę, by podziwiać piękne widoki na Tatry oraz miasto Zakopane.</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>{
+  "date_from": "01-01",
+  "date_to": "12-31",
+  "mon": "08:00-22:00",
+  "tue": "08:00-22:00",
+  "wed": "08:00-22:00",
+  "thu": "08:00-22:00",
+  "fri": "08:00-22:00",
+  "sat": "08:00-22:00",
+  "sun": "08:00-22:00"
+}</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>20</v>
+      </c>
+      <c r="J81" t="n">
+        <v>60</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Wstęp bezpłatny</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>Antałówka na Wierch 36, 34-500 Zakopane, Poland</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Małopolska</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>49.29200770</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>19.97249340</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>outdoor</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>good_weather_only</t>
+        </is>
+      </c>
+      <c r="W81" t="n">
+        <v>2</v>
+      </c>
+      <c r="X81" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>17:00-19:00</t>
+        </is>
+      </c>
+      <c r="Z81" t="inlineStr">
+        <is>
+          <t>morning, afternoon, evening</t>
+        </is>
+      </c>
+      <c r="AA81" t="inlineStr">
+        <is>
+          <t>Zakopane</t>
+        </is>
+      </c>
+      <c r="AB81" t="inlineStr">
+        <is>
+          <t>couples, seniors, friends, family_kids, solo</t>
+        </is>
+      </c>
+      <c r="AC81" t="inlineStr">
+        <is>
+          <t>6-10, 10-14</t>
+        </is>
+      </c>
+      <c r="AD81" t="inlineStr">
+        <is>
+          <t>nature_landscape</t>
+        </is>
+      </c>
+      <c r="AE81" t="inlineStr">
+        <is>
+          <t>recreational</t>
+        </is>
+      </c>
+      <c r="AF81" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="AG81" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
+      <c r="AH81" t="inlineStr">
+        <is>
+          <t>all_year</t>
+        </is>
+      </c>
+      <c r="AI81" t="inlineStr">
+        <is>
+          <t>Na Antałówkę warto wybrać się o wschodzie lub zachodzie słońca – widoki są wtedy szczególnie malownicze.</t>
+        </is>
+      </c>
+      <c r="AJ81" t="inlineStr">
+        <is>
+          <t>Parking na miejscu</t>
+        </is>
+      </c>
+      <c r="AK81" t="inlineStr">
+        <is>
+          <t>Antałówka na Wierch 36, 34-500 Zakopane</t>
+        </is>
+      </c>
+      <c r="AL81" t="inlineStr">
+        <is>
+          <t>49.29205128139108</t>
+        </is>
+      </c>
+      <c r="AM81" t="inlineStr">
+        <is>
+          <t>19.97249464174183</t>
+        </is>
+      </c>
+      <c r="AN81" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="AO81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP81" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="AQ81" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AR81" t="inlineStr">
+        <is>
+          <t>nature_landscape, viewpoint, panoramic_view, scenic_view, relaxation, photography, sunset</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Tatrzańskie Archiwum Planety Ziemia</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Nowoczesne centrum edukacyjne przybliżające faunę, florę i geologię Tatr.</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Centrum Edukacji Przyrodniczej Tatrzańskiego Parku Narodowego w Dolinie Kościeliskiej to nowoczesny obiekt edukacyjny oferujący interaktywne wystawy poświęcone tatrzańskiej przyrodzie. W centrum można poznać bogactwo flory, fauny, a także interesujące aspekty geologiczne regionu. Ekspozycje multimedialne i warsztaty edukacyjne skierowane są do dzieci i dorosłych. To doskonałe miejsce, by pogłębić wiedzę przed wyruszeniem na górskie szlaki Doliny Kościeliskiej.</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Miejsce idealne dla rodzin z dziećmi i osób zainteresowanych przyrodą Tatr. Pozwala w atrakcyjny sposób poznać unikatowy świat tatrzańskiej przyrody i przygotować się do wycieczek terenowych.</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>[
+  {
+    "date_from": "06-01",
+    "date_to": "09-30",
+    "mon": "closed",
+    "tue": "08:00-18:00",
+    "wed": "08:00-18:00",
+    "thu": "08:00-18:00",
+    "fri": "08:00-18:00",
+    "sat": "08:00-18:00",
+    "sun": "08:00-18:00"
+  },
+  {
+    "date_from": "10-01",
+    "date_to": "05-31",
+    "mon": "closed",
+    "tue": "09:00-17:00",
+    "wed": "09:00-17:00",
+    "thu": "09:00-17:00",
+    "fri": "09:00-17:00",
+    "sat": "09:00-17:00",
+    "sun": "09:00-17:00"
+  }
+]</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>45</v>
+      </c>
+      <c r="J82" t="n">
+        <v>120</v>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Bilet normalny: 40,00 zł, Bilet ulgow: 30,00 zł</t>
+        </is>
+      </c>
+      <c r="L82" t="n">
+        <v>40</v>
+      </c>
+      <c r="M82" t="n">
+        <v>30</v>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Dolina Kościeliska 3, 34-511 Kościelisko, Poland</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>Małopolska</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>49.27478340</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>19.86830200</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>indoor</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>all_weather</t>
+        </is>
+      </c>
+      <c r="W82" t="n">
+        <v>7</v>
+      </c>
+      <c r="X82" t="n">
+        <v>7</v>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>11:00-14:00</t>
+        </is>
+      </c>
+      <c r="Z82" t="inlineStr">
+        <is>
+          <t>midday, afternoon</t>
+        </is>
+      </c>
+      <c r="AA82" t="inlineStr">
+        <is>
+          <t>Kościelisko</t>
+        </is>
+      </c>
+      <c r="AB82" t="inlineStr">
+        <is>
+          <t>couples, seniors, friends, family_kids, solo</t>
+        </is>
+      </c>
+      <c r="AC82" t="inlineStr">
+        <is>
+          <t>6-10, 10-14</t>
+        </is>
+      </c>
+      <c r="AD82" t="inlineStr">
+        <is>
+          <t>museum_heritage</t>
+        </is>
+      </c>
+      <c r="AE82" t="inlineStr">
+        <is>
+          <t>cultural</t>
+        </is>
+      </c>
+      <c r="AF82" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="AG82" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="AH82" t="inlineStr">
+        <is>
+          <t>all_year</t>
+        </is>
+      </c>
+      <c r="AI82" t="inlineStr">
+        <is>
+          <t>Warto odwiedzić centrum przed wyruszeniem na szlak – można dowiedzieć się wielu praktycznych informacji o lokalnej florze i faunie.</t>
+        </is>
+      </c>
+      <c r="AJ82" t="inlineStr">
+        <is>
+          <t>Parking Dolina Kościeliska</t>
+        </is>
+      </c>
+      <c r="AK82" t="inlineStr">
+        <is>
+          <t>Strzelców Podhalańskich 58, 43-229 Kościelisko</t>
+        </is>
+      </c>
+      <c r="AL82" t="inlineStr">
+        <is>
+          <t>49.27559315661158</t>
+        </is>
+      </c>
+      <c r="AM82" t="inlineStr">
+        <is>
+          <t>19.869176011620024</t>
+        </is>
+      </c>
+      <c r="AN82" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="AO82" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP82" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="AQ82" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AR82" t="inlineStr">
+        <is>
+          <t>museum_heritage, education, indoor, rainy_day, geology, science</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Bachledzki Wierch</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Bachledzki Wierch to widokowe wzniesienie położone w Zakopanem, popularne wśród spacerowiczów oraz turystów ceniących spokojne trasy i panoramę Tatr.</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Bachledzki Wierch to jedno z mniej zatłoczonych i spokojnych miejsc spacerowych w Zakopanem. Trasa wiedzie malowniczym grzbietem, z którego rozciągają się piękne widoki na Tatry, Gubałówkę oraz okoliczne pola i lasy. Wierzchołek stanowi świetny punkt widokowy zarówno na Tatry Zachodnie, jak i część Tatr Wysokich. Szlak jest łagodny i nadaje się dla rodzin z dziećmi oraz osób szukających alternatywy dla zatłoczonych zakopiańskich atrakcji.</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Ze względu na rozległe widoki i mniej uczęszczane ścieżki, Bachledzki Wierch to doskonałe miejsce na spokojny spacer z dala od tłumów oraz na podziwianie panoramy Tatr i Zakopanego.</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>{
+  "date_from": "01-01",
+  "date_to": "12-31",
+  "mon": "08:00-22:00",
+  "tue": "08:00-22:00",
+  "wed": "08:00-22:00",
+  "thu": "08:00-22:00",
+  "fri": "08:00-22:00",
+  "sat": "08:00-22:00",
+  "sun": "08:00-22:00"
+}</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>60</v>
+      </c>
+      <c r="J83" t="n">
+        <v>120</v>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Wstęp bezpłatny</t>
+        </is>
+      </c>
+      <c r="L83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" t="n">
+        <v>0</v>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>Bachledzki Wierch, 34-500 Zakopane, Poland</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>Małopolska</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>49.30406910</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>19.97180910</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>outdoor</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>good_weather_only</t>
+        </is>
+      </c>
+      <c r="W83" t="n">
+        <v>5</v>
+      </c>
+      <c r="X83" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>14:00-16:00</t>
+        </is>
+      </c>
+      <c r="Z83" t="inlineStr">
+        <is>
+          <t>morning, midday, afternoon</t>
+        </is>
+      </c>
+      <c r="AA83" t="inlineStr">
+        <is>
+          <t>Zakopane</t>
+        </is>
+      </c>
+      <c r="AB83" t="inlineStr">
+        <is>
+          <t>couples, seniors, friends, family_kids, solo</t>
+        </is>
+      </c>
+      <c r="AC83" t="inlineStr">
+        <is>
+          <t>6-10, 10-14</t>
+        </is>
+      </c>
+      <c r="AD83" t="inlineStr">
+        <is>
+          <t>nature_landscape</t>
+        </is>
+      </c>
+      <c r="AE83" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AF83" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="AG83" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
+      <c r="AH83" t="inlineStr">
+        <is>
+          <t>all_year</t>
+        </is>
+      </c>
+      <c r="AI83" t="inlineStr">
+        <is>
+          <t>Wybierz się tu o wschodzie lub zachodzie słońca – światło wtedy najpiękniej wydobywa górski krajobraz i jest idealne do fotografii.</t>
+        </is>
+      </c>
+      <c r="AJ83" t="inlineStr">
+        <is>
+          <t>Parking przy cmenatrzu</t>
+        </is>
+      </c>
+      <c r="AK83" t="inlineStr">
+        <is>
+          <t>Podhalańska 61, 34-500 Zakopane</t>
+        </is>
+      </c>
+      <c r="AL83" t="inlineStr">
+        <is>
+          <t>49.30070527395064</t>
+        </is>
+      </c>
+      <c r="AM83" t="inlineStr">
+        <is>
+          <t>19.98471872519335</t>
+        </is>
+      </c>
+      <c r="AN83" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="AO83" t="n">
+        <v>25</v>
+      </c>
+      <c r="AP83" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="AQ83" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AR83" t="inlineStr">
+        <is>
+          <t>nature_landscape, viewpoint, panoramic_view, scenic_view, relaxation, photography, sunset</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Centrum Kultury Rodzimej w willi Czerwony Dwór</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Zabytkowa willa prezentująca sztukę i kulturę regionu Podhala.</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Willa Czerwony Dwór to zabytkowy obiekt architektury zakopiańskiej, który obecnie pełni funkcję Centrum Kultury Rodzimej. W budynku organizowane są wystawy czasowe prezentujące dorobek artystyczny regionu Podhala, wydarzenia kulturalne oraz warsztaty. Wnętrza willi zachowały historyczny charakter, co pozwala zwiedzającym poczuć klimat dawnych czasów i lepiej poznać tradycje góralskie.</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>To wyjątkowe miejsce pozwalające poznać podhalańską sztukę, kulturę i architekturę w autentycznym otoczeniu historycznej willi.</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>{
+  "date_from": "01-01",
+  "date_to": "12-31",
+  "mon": "10:00-17:00",
+  "tue": "10:00-17:00",
+  "wed": "closed",
+  "thu": "10:00-17:00",
+  "fri": "closed",
+  "sat": "closed",
+  "sun": "closed"
+}</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>30</v>
+      </c>
+      <c r="J84" t="n">
+        <v>90</v>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Wstęp bezpłatny</t>
+        </is>
+      </c>
+      <c r="L84" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" t="n">
+        <v>0</v>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>Kasprusie 27, 34-500 Zakopane, Poland</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>Małopolska</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>49.29118900</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>19.94841770</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>indoor</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>all_weather</t>
+        </is>
+      </c>
+      <c r="W84" t="n">
+        <v>5</v>
+      </c>
+      <c r="X84" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>13:00-16:00</t>
+        </is>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>midday, afternoon</t>
+        </is>
+      </c>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>Zakopane</t>
+        </is>
+      </c>
+      <c r="AB84" t="inlineStr">
+        <is>
+          <t>seniors, solo</t>
+        </is>
+      </c>
+      <c r="AD84" t="inlineStr">
+        <is>
+          <t>museum_heritage</t>
+        </is>
+      </c>
+      <c r="AE84" t="inlineStr">
+        <is>
+          <t>cultural</t>
+        </is>
+      </c>
+      <c r="AF84" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="AG84" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
+      <c r="AH84" t="inlineStr">
+        <is>
+          <t>all_year</t>
+        </is>
+      </c>
+      <c r="AI84" t="inlineStr">
+        <is>
+          <t>Sprawdź aktualny harmonogram wystaw i wydarzeń – często odbywają się tu ciekawe warsztaty i spotkania z lokalnymi artystami.</t>
+        </is>
+      </c>
+      <c r="AJ84" t="inlineStr">
+        <is>
+          <t>Parking na miejscu</t>
+        </is>
+      </c>
+      <c r="AK84" t="inlineStr">
+        <is>
+          <t>Kasprusie 27, 34-500 Zakopane</t>
+        </is>
+      </c>
+      <c r="AL84" t="inlineStr">
+        <is>
+          <t>49.2912080929078</t>
+        </is>
+      </c>
+      <c r="AM84" t="inlineStr">
+        <is>
+          <t>19.948458903744253</t>
+        </is>
+      </c>
+      <c r="AN84" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="AO84" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP84" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="AQ84" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AR84" t="inlineStr">
+        <is>
+          <t>museum_heritage, culture, folklore, education, indoor, rainy_day, history_mystery</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FIX #113: ZONE SYSTEM — per-day zone-aware POI pools
Changes:
- data/zakopane.xlsx: Zone column added (A:67, B:12, C:3 / 82 rows matched)
- data/multi_city_attractions.xlsx: Zone column added (230/681 rows matched)
- load_zakopane.py + load_multi_city.py: 'zone' field added to poi dict
- normalizer.py: 'zone' field preserved through normalize_poi()
- engine.py: plan_multiple_days() accepts pois_per_day param (backward compat)
- plan_service.py: _build_zone_pools() — rotates A->B->C per day
  single-day uses Zone A (most central); cities w/o zones unaffected (None -> all pois)
  FIX #112 POI shortage check updated to use smallest zone pool as effective size
</commit_message>
<xml_diff>
--- a/data/zakopane.xlsx
+++ b/data/zakopane.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR83"/>
+  <dimension ref="A1:AS83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -570,12 +570,12 @@
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Target group </t>
+          <t>Target group</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Children's age </t>
+          <t>Children's age</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Budget type </t>
+          <t>Budget type</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
@@ -651,6 +651,11 @@
       <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>Tags</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>Zone</t>
         </is>
       </c>
     </row>
@@ -868,6 +873,11 @@
           <t>mountain_culture, regional_heritage, workshop,themed_museum</t>
         </is>
       </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
@@ -1072,6 +1082,11 @@
           <t>petting_zoo, farm_animals, feeding_experience</t>
         </is>
       </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
@@ -1275,6 +1290,11 @@
           <t>miniature_world, fairytale_world</t>
         </is>
       </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr"/>
@@ -1479,6 +1499,11 @@
           <t>illusion_kids, interactive_exhibition_kids, interactive_exhibits,</t>
         </is>
       </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
@@ -1682,6 +1707,11 @@
           <t>birds_only, close_contact, educational_exhibition</t>
         </is>
       </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
@@ -1885,6 +1915,11 @@
           <t>aquatic_animals, educational_exhibition</t>
         </is>
       </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr"/>
@@ -2088,6 +2123,11 @@
           <t>snow_tubing, adrenaline_experience, beginner_friendly,group_activity</t>
         </is>
       </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
@@ -2294,6 +2334,11 @@
           <t>playground</t>
         </is>
       </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
@@ -2497,6 +2542,11 @@
           <t>indoor_playroom, kids_obstacle_course, sensory_experience_kids</t>
         </is>
       </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
@@ -2699,6 +2749,11 @@
           <t>indoor_playroom, kids_obstacle_course</t>
         </is>
       </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
@@ -2898,6 +2953,11 @@
           <t>dinosaur_theme, walkthrough_experience, family_theme_park</t>
         </is>
       </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
@@ -3100,6 +3160,11 @@
           <t>illusion_kids, interactive_exhibition_kids, science_center_kids</t>
         </is>
       </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
@@ -3302,6 +3367,11 @@
           <t>illusion_kids, interactive_exhibition_kids</t>
         </is>
       </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
@@ -3500,6 +3570,11 @@
           <t>playground, kids_obstacle_course</t>
         </is>
       </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
@@ -3703,6 +3778,11 @@
           <t>thermal_baths, water_slides, family_friendly_water, spa_pools, sauna_zone</t>
         </is>
       </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
@@ -3906,6 +3986,11 @@
           <t>thermal_baths, relax_zone, thermal_relax_focus, long_stay_possible, evening_relax</t>
         </is>
       </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
@@ -4109,6 +4194,11 @@
           <t>thermal_baths, water_slides, kids_zone, sauna_zone, long_stay_possible</t>
         </is>
       </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
@@ -4311,6 +4401,11 @@
           <t>thermal_baths, water_slides, kids_zone, sauna_zone, spa_pools</t>
         </is>
       </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
@@ -4514,6 +4609,11 @@
           <t>thermal_baths, water_slides, kids_zone, sauna_zone, long_stay_possible</t>
         </is>
       </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
@@ -4716,6 +4816,11 @@
           <t>viewpoint, mountain_views, photo_spot, easy_access_nature</t>
         </is>
       </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
@@ -4918,6 +5023,11 @@
           <t>themed_museum, multimedia_exhibition, interactive_exhibits</t>
         </is>
       </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
@@ -5116,6 +5226,11 @@
           <t>themed_museum, interactive_exhibit, intimate_small_museum</t>
         </is>
       </c>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
@@ -5314,6 +5429,11 @@
           <t>miniature_world, interactive_exhibition_kids, creative_workshops_kids</t>
         </is>
       </c>
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
@@ -5511,6 +5631,11 @@
           <t>regional_heritage, mountain_culture, temporary_exhibitions, multimedia_exhibition</t>
         </is>
       </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
@@ -5708,6 +5833,11 @@
           <t>composer_artist_house, historic_building, intimate_small_museum</t>
         </is>
       </c>
+      <c r="AS26" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
@@ -5905,6 +6035,11 @@
           <t>architecture_heritage, mountain_culture, crafts_handicraft, historic_building</t>
         </is>
       </c>
+      <c r="AS27" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
@@ -6102,6 +6237,11 @@
           <t>art_gallery, architecture_heritage, historic_building, temporary_exhibitions</t>
         </is>
       </c>
+      <c r="AS28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
@@ -6298,6 +6438,11 @@
           <t>composer_artist_house, historic_building, intimate_small_museum</t>
         </is>
       </c>
+      <c r="AS29" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
@@ -6498,6 +6643,11 @@
           <t>educational_farm, feeding_experience, educational_exhibition</t>
         </is>
       </c>
+      <c r="AS30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
@@ -6694,6 +6844,11 @@
       <c r="AR31" t="inlineStr">
         <is>
           <t>architecture_heritage, mountain_culture, historic_building</t>
+        </is>
+      </c>
+      <c r="AS31" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -6903,6 +7058,11 @@
       <c r="AR32" t="inlineStr">
         <is>
           <t>horse_riding, low_intensity_activity, seasonal_activity, group_activity</t>
+        </is>
+      </c>
+      <c r="AS32" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -7114,6 +7274,11 @@
       <c r="AR33" t="inlineStr">
         <is>
           <t>easy_walk, family_friendly_trail, out_and_back, trailhead_parking, crowd_prone, nature_immersion, long_distance</t>
+        </is>
+      </c>
+      <c r="AS33" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -7328,6 +7493,11 @@
           <t>easy_walk, family_friendly_trail, nature_immersion, out_and_back, trailhead_parking, crowd_prone, time_flexible</t>
         </is>
       </c>
+      <c r="AS34" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
@@ -7540,6 +7710,11 @@
           <t>easy_walk, family_friendly_trail, viewpoint_trail, out_and_back, trailhead_parking, stroller_friendly, crowd_prone</t>
         </is>
       </c>
+      <c r="AS35" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
@@ -7752,6 +7927,11 @@
           <t>easy_walk, long_distance, stroller_friendly, out_and_back, crowd_prone, trailhead_parking, requires_transport</t>
         </is>
       </c>
+      <c r="AS36" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
@@ -7938,6 +8118,11 @@
       <c r="AR37" t="inlineStr">
         <is>
           <t>panoramic_mountain_views, tatra_viewpoint, scenic_ridge_walk, iconic_tatra_landmark</t>
+        </is>
+      </c>
+      <c r="AS37" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -8127,6 +8312,11 @@
       <c r="AR38" t="inlineStr">
         <is>
           <t>snow_tubing,adrenaline_experience,group_activity</t>
+        </is>
+      </c>
+      <c r="AS38" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -8369,6 +8559,11 @@
           <t>cable_car_option,viewpoint_trail,time_flexible</t>
         </is>
       </c>
+      <c r="AS39" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
@@ -8568,6 +8763,11 @@
           <t>easy_walk,forest_trails,nature_immersion,family_friendly_trail</t>
         </is>
       </c>
+      <c r="AS40" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
@@ -8767,6 +8967,11 @@
           <t>moderate_hike,waterfall_trail,nature_immersion,family_friendly_trail</t>
         </is>
       </c>
+      <c r="AS41" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
@@ -8966,6 +9171,11 @@
           <t>moderate_hike,rock_formations,nature_immersion</t>
         </is>
       </c>
+      <c r="AS42" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
@@ -9165,6 +9375,11 @@
           <t>easy_walk,meadows_fields,viewpoint_trail,quiet_relax_spot</t>
         </is>
       </c>
+      <c r="AS43" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
@@ -9364,6 +9579,11 @@
           <t>mountain_views,viewpoint,photo_spot</t>
         </is>
       </c>
+      <c r="AS44" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
@@ -9563,6 +9783,11 @@
           <t>waterfalls,nature_reserve,photo_spot</t>
         </is>
       </c>
+      <c r="AS45" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
@@ -9762,6 +9987,11 @@
           <t>meadows_fields,forest_trails,quiet_relax_spot</t>
         </is>
       </c>
+      <c r="AS46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
@@ -9961,6 +10191,11 @@
           <t>meadows_fields,nature_immersion,scenic_walk</t>
         </is>
       </c>
+      <c r="AS47" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
@@ -10160,6 +10395,11 @@
           <t>waterfalls,forest_trails,photo_spot</t>
         </is>
       </c>
+      <c r="AS48" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
@@ -10359,6 +10599,11 @@
           <t>meadows_fields,nature_immersion,quiet_relax_spot</t>
         </is>
       </c>
+      <c r="AS49" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
@@ -10558,6 +10803,11 @@
           <t>moderate_hike,valley_landscape,nature_immersion</t>
         </is>
       </c>
+      <c r="AS50" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
@@ -10757,6 +11007,11 @@
           <t>moderate_hike,forest_trails,nature_immersion</t>
         </is>
       </c>
+      <c r="AS51" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
@@ -10956,6 +11211,11 @@
           <t>moderate_hike,panoramic_route,peak_summit</t>
         </is>
       </c>
+      <c r="AS52" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
@@ -11155,6 +11415,11 @@
           <t>forest_trails,quiet_relax_spot,scenic_walk</t>
         </is>
       </c>
+      <c r="AS53" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
@@ -11343,6 +11608,11 @@
           <t>regional_heritage,folk_traditions,historic_building</t>
         </is>
       </c>
+      <c r="AS54" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
@@ -11529,6 +11799,11 @@
       <c r="AR55" t="inlineStr">
         <is>
           <t>quad_atv,adrenaline_experience,group_activity</t>
+        </is>
+      </c>
+      <c r="AS55" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -11726,6 +12001,11 @@
           <t>meadows_fields,mountain_views,photo_spot</t>
         </is>
       </c>
+      <c r="AS56" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
@@ -11914,6 +12194,11 @@
           <t>spa_center,quiet_relax,long_relax_session</t>
         </is>
       </c>
+      <c r="AS57" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
@@ -12108,6 +12393,11 @@
       <c r="AR58" t="inlineStr">
         <is>
           <t>spa_center,quiet_relax,romantic_atmosphere</t>
+        </is>
+      </c>
+      <c r="AS58" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -12309,6 +12599,11 @@
           <t>mountain_views,viewpoint,photo_spot</t>
         </is>
       </c>
+      <c r="AS59" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
@@ -12501,6 +12796,11 @@
           <t>rope_park,adventure_park,medium_intensity_activity</t>
         </is>
       </c>
+      <c r="AS60" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
@@ -12689,6 +12989,11 @@
           <t>historical_exhibits,local_legends,historic_building</t>
         </is>
       </c>
+      <c r="AS61" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
@@ -12877,6 +13182,11 @@
           <t>regional_heritage,historic_building</t>
         </is>
       </c>
+      <c r="AS62" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr"/>
@@ -13065,6 +13375,11 @@
           <t>forest_trails,nature_reserve,storytelling_spot</t>
         </is>
       </c>
+      <c r="AS63" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr"/>
@@ -13250,6 +13565,11 @@
           <t>snow_tubing,family_theme_park,kids_zone</t>
         </is>
       </c>
+      <c r="AS64" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
@@ -13444,6 +13764,11 @@
       <c r="AR65" t="inlineStr">
         <is>
           <t>street_food,food_market,lively_atmosphere,central_location, evening_activity, walking, local_food_experience, shopping, relaxation</t>
+        </is>
+      </c>
+      <c r="AS65" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -13645,6 +13970,11 @@
           <t>meadows_fields,scenic_walk,quiet_relax_spot, walking, relaxation, seniors, family_friendly, evening_activity</t>
         </is>
       </c>
+      <c r="AS66" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr"/>
@@ -13841,6 +14171,11 @@
           <t>composer_artist_house,regional_heritage,historic_building</t>
         </is>
       </c>
+      <c r="AS67" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr"/>
@@ -14035,6 +14370,11 @@
       <c r="AR68" t="inlineStr">
         <is>
           <t>architecture_heritage,regional_heritage,historic_building</t>
+        </is>
+      </c>
+      <c r="AS68" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -14236,6 +14576,11 @@
           <t>historic_building,regional_heritage</t>
         </is>
       </c>
+      <c r="AS69" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr"/>
@@ -14430,6 +14775,11 @@
       <c r="AR70" t="inlineStr">
         <is>
           <t>art_gallery,temporary_exhibitions,historic_building</t>
+        </is>
+      </c>
+      <c r="AS70" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -14661,6 +15011,11 @@
           <t>panoramic_mountain_views, tatra_viewpoint, scenic_photo_spot, iconic_tatra_landmark</t>
         </is>
       </c>
+      <c r="AS71" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr"/>
@@ -14855,6 +15210,11 @@
       <c r="AR72" t="inlineStr">
         <is>
           <t>interactive_photo_exhibits, colorful_installations, instagram_photo_spot</t>
+        </is>
+      </c>
+      <c r="AS72" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -15060,6 +15420,11 @@
           <t>mountain_ski_resort, tatra_viewpoint, thermal_pool_relax</t>
         </is>
       </c>
+      <c r="AS73" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr"/>
@@ -15248,6 +15613,11 @@
           <t>animal_interaction, rabbit_feeding, family_friendly_animals</t>
         </is>
       </c>
+      <c r="AS74" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr"/>
@@ -15440,6 +15810,11 @@
           <t>thermal_outdoor_pool, tatra_viewpoint, summer_mountain_relax, family_swimming_area</t>
         </is>
       </c>
+      <c r="AS75" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
@@ -15624,6 +15999,11 @@
           <t>local_food, regional_cuisine, oscypek, traditional_food, bacowka, podhale, authentic_place</t>
         </is>
       </c>
+      <c r="AS76" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr"/>
@@ -15812,6 +16192,11 @@
           <t>local_food, oscypek, workshop, tasting, cultural_experience, regional_cuisine, traditional_food</t>
         </is>
       </c>
+      <c r="AS77" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr"/>
@@ -15996,6 +16381,11 @@
           <t>food_market, street_food, local_products, souvenirs, regional_food, oscypek, market, local_experience</t>
         </is>
       </c>
+      <c r="AS78" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr"/>
@@ -16180,6 +16570,11 @@
           <t>nature_landscape, viewpoint, relaxation, history_mystery, museum_heritage, panoramic_view, scenic_view</t>
         </is>
       </c>
+      <c r="AS79" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr"/>
@@ -16366,6 +16761,11 @@
       <c r="AR80" t="inlineStr">
         <is>
           <t>nature_landscape, viewpoint, panoramic_view, scenic_view, relaxation, photography, sunset</t>
+        </is>
+      </c>
+      <c r="AS80" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -16569,6 +16969,11 @@
           <t>museum_heritage, education, indoor, rainy_day, geology, science</t>
         </is>
       </c>
+      <c r="AS81" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr"/>
@@ -16757,6 +17162,11 @@
           <t>nature_landscape, viewpoint, panoramic_view, scenic_view, relaxation, photography, sunset</t>
         </is>
       </c>
+      <c r="AS82" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr"/>
@@ -16941,6 +17351,11 @@
           <t>museum_heritage, culture, folklore, education, indoor, rainy_day, history_mystery</t>
         </is>
       </c>
+      <c r="AS83" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
﻿FIX #179-#180: pakiet naturalnosci light — preferencje, determinizm, lunch seniors
- Mapowanie pref→tagi, quota boost dla niepokrytych preferencji (5+ dni)
- Deterministyczny pick zamiast random; trip-wide preference coverage w API
- Zone C tylko od late-trip; exclude Zone C na wczesnych dniach
- FIX #180: skip/clamp return transit przed lunchem dla seniors/family_kids (okno 13:30)
- Lepszy split tagow w load_zakopane

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/zakopane.xlsx
+++ b/data/zakopane.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -58,12 +57,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -660,7 +660,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>Muzeum Oscypka Zakopane</t>
@@ -686,7 +685,6 @@
           <t>To niepowtarzalna okazja, by zanurzyć się w góralskich tradycjach, zobaczyć na żywo wyrób oscypka oraz spróbować tego regionalnego przysmaku.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>[
@@ -880,7 +878,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>Tatrzańskie Mini Zoo</t>
@@ -906,7 +903,6 @@
           <t>To doskonałe miejsce dla rodzin, które chcą spędzić czas w otoczeniu zwierząt, dowiedzieć się więcej o podhalańskiej faunie oraz zapewnić dzieciom bezpośredni kontakt ze zwierzętami.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>[
@@ -1089,7 +1085,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>Myszogród</t>
@@ -1115,7 +1110,6 @@
           <t>Wizytę w Myszogrodzie warto odbyć, aby zobaczyć niezwykłą prezentację żywych zwierząt w starannie przygotowanym, bajkowym otoczeniu, idealnym na rodzinny wypad lub niecodzienną atrakcję podczas pobytu w Zakopanem.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>[
@@ -1297,7 +1291,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Iluzja Park</t>
@@ -1323,7 +1316,6 @@
           <t>To doskonałe miejsce na spędzenie czasu z rodziną, poznanie fascynującego świata iluzji i wykonanie wyjątkowych zdjęć. Park pozwala połączyć naukę z zabawą i daje okazję do wspólnej integracji.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>[
@@ -1506,7 +1498,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>Papugarnia Egzotyczne Zakopane</t>
@@ -1532,7 +1523,6 @@
           <t>To wyjątkowa okazja, by obcować bezpośrednio z egzotycznymi ptakami, nie wyjeżdżając poza Zakopane. Papugarnia świetnie sprawdza się zarówno przy każdej pogodzie, będąc miejscem atrakcyjnym dla dzieci i dorosłych.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>[
@@ -1714,7 +1704,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>Podwodny Świat</t>
@@ -1740,7 +1729,6 @@
           <t>Warto odwiedzić to akwarium, aby dowiedzieć się więcej o życiu pod wodą, poznać rodzime gatunki ryb oraz spędzić czas w ciekawy sposób niezależnie od pogody.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>[
@@ -1922,7 +1910,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>Zjazd pontonem ze skoczni narciarskiej Wielka Krokiew</t>
@@ -1948,7 +1935,6 @@
           <t>To jedna z nielicznych okazji, by poczuć adrenalinę zjazdu ze skoczni, którą na co dzień wykorzystują najlepsi skoczkowie narciarscy w kraju. Idealny wybór dla osób szukających aktywnych rozrywek poza standardowym zwiedzaniem.</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>[
@@ -2052,7 +2038,7 @@
           <t>friends, family_kids</t>
         </is>
       </c>
-      <c r="AC8" s="2" t="n">
+      <c r="AC8" s="3" t="n">
         <v>45944</v>
       </c>
       <c r="AD8" t="inlineStr">
@@ -2130,7 +2116,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>Góralski Ślizg</t>
@@ -2156,7 +2141,6 @@
           <t>To świetna forma aktywności na świeżym powietrzu, idealna na spędzenie czasu z rodziną lub znajomymi, szczególnie po dniu górskich wędrówek. Atrakcja ta pozwala na poczucie adrenaliny i radości niezależnie od wieku.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>[
@@ -2341,7 +2325,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>Tatra Family</t>
@@ -2367,7 +2350,6 @@
           <t>Wizyta w Tatra Family to świetna okazja do aktywnego spędzenia czasu z rodziną i zapewnienia dzieciom niezapomnianej zabawy w bezpiecznym otoczeniu.</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>[
@@ -2549,7 +2531,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>Park Harnasia</t>
@@ -2575,7 +2556,6 @@
           <t>Warto odwiedzić Park Harnasia, by odpocząć zrelaksować się i pozwolić dzieciom pobawić się na placu zabaw. To świetny punkt na chwilę wytchnienia podczas zwiedzania Zakopanego.</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>[
@@ -2756,13 +2736,11 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>DINO PARK</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>Park tematyczny z modelami dinozaurów w naturalnych rozmiarach.</t>
@@ -2778,7 +2756,6 @@
           <t>To idealna atrakcja dla rodzin z dziećmi oraz wszystkich miłośników paleontologii i dinozaurów. Pozwala na edukację poprzez zabawę i kontakt z naturą.</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>[
@@ -2960,7 +2937,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>Illusion House</t>
@@ -2986,7 +2962,6 @@
           <t>Wizyta w Domu Iluzji to nie tylko świetna zabawa, ale też możliwość poznania tajników działania naszego mózgu i zmysłów. To idealne miejsce na rodzinny wypad lub rozrywkę podczas brzydszej pogody w Zakopanem.</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>[
@@ -3167,7 +3142,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>Dom do góry nogami</t>
@@ -3193,7 +3167,6 @@
           <t>To idealne miejsce na nietypową rozrywkę i sesję zdjęciową – zaskakuje i bawi zarówno najmłodszych, jak i starszych turystów.</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>[
@@ -3374,13 +3347,11 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>Plac zabaw na Górnej Równi Krupowej</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>Nowoczesny plac zabaw położony na rozległej Górnej Równi Krupowej w Zakopanem.</t>
@@ -3396,7 +3367,6 @@
           <t>To idealne miejsce na odpoczynek i zabawę dla dzieci po zwiedzaniu Zakopanego. Malownicze położenie oraz czyste, przestronne otoczenie sprzyjają relaksowi i rekreacji całych rodzin.</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>[
@@ -3577,7 +3547,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>Termy Zakopiańskie</t>
@@ -3603,7 +3572,6 @@
           <t>Wizyta w Termach Zakopiańskich to okazja do zabawy i relaksu w wodzie, niezależnie od warunków pogodowych. Można tu korzystać z wielu atrakcji basenowych i wellness oraz zjeść smaczny posiłek.</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>[
@@ -3785,7 +3753,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>Termy Gorący Potok</t>
@@ -3811,7 +3778,6 @@
           <t>Wizyta pozwala zrelaksować się w ciepłych wodach termalnych, korzystać z leczniczych i relaksacyjnych właściwości wód oraz atrakcji dostępnych na terenie kompleksu.</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>[
@@ -3993,7 +3959,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>Chochołowskie Termy</t>
@@ -4019,7 +3984,6 @@
           <t>To doskonałe miejsce na relaks i rekreację przez cały rok, z licznymi udogodnieniami dla rodzin, par i miłośników sportu. Naturalna woda termalna wpływa korzystnie na zdrowie i samopoczucie, a bogata strefa spa i saun zapewnia głęboki relaks.</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>[
@@ -4201,7 +4165,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>Terma Bania</t>
@@ -4227,7 +4190,6 @@
           <t>To idealne miejsce na relaks w wodach termalnych z pięknym widokiem na góry, a także rozrywkę dla całej rodziny.</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>[
@@ -4408,7 +4370,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>Termy Bukovina</t>
@@ -4434,7 +4395,6 @@
           <t>To idealne miejsce na relaks, odprężenie po górskich wędrówkach i zabawę z rodziną lub przyjaciółmi w wodzie termalnej.</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>[
@@ -4616,7 +4576,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t>Wielka Krokiew</t>
@@ -4642,7 +4601,6 @@
           <t>To miejsce kultowe dla miłośników sportów i niepowtarzalny punkt widokowy na Tatry oraz Zakopane. Wizyta na Wielkiej Krokwi pozwala poczuć sportową atmosferę i zobaczyć na własne oczy miejsce legendarnych zawodów.</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>[
@@ -4823,7 +4781,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t>Centrum Edukacji Przyrodniczej Tatrzańskiego Parku Narodowego</t>
@@ -4849,7 +4806,6 @@
           <t>To miejsce pozwala pogłębić wiedzę o Tatrach w atrakcyjny i angażujący sposób. Idealne zarówno dla rodzin z dziećmi, jak i pasjonatów przyrody.</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>[
@@ -5030,13 +4986,11 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
           <t>Wystawa Figur Woskowych EXPO Krupówki</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>Wystawa prezentująca realistyczne figury woskowe znanych postaci.</t>
@@ -5052,7 +5006,6 @@
           <t>Warto odwiedzić, aby zobaczyć imponująco wykonane figury woskowe znanych postaci, a także zrobić oryginalne pamiątkowe zdjęcia. To doskonały sposób na urozmaicenie pobytu na Krupówkach i rozrywkę niezależnie od pogody.</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>[
@@ -5233,13 +5186,11 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
           <t>Wielka Wystawa Klocków LEGO</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>Imponująca wystawa prezentująca największe modele wykonane z klocków LEGO.</t>
@@ -5255,7 +5206,6 @@
           <t>To jedna z największych wystaw LEGO w Polsce, idealna dla rodzin i miłośników LEGO w każdym wieku. Pozwala zobaczyć niesamowite konstrukcje oraz inspirować się do własnych projektów.</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>[
@@ -5436,13 +5386,11 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
           <t>Muzeum Tatrzańskie</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>Muzeum prezentujące historię, kulturę i przyrodę Tatr oraz Podhala.</t>
@@ -5458,7 +5406,6 @@
           <t>To idealne miejsce, aby lepiej poznać historię Zakopanego, kulturę góralską oraz bogactwo tatrzańskiej przyrody. Muzeum stanowi doskonały punkt startowy do dalszego odkrywania Tatr i regionu Podhala.</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>[
@@ -5561,7 +5508,7 @@
           <t>solo, couples, friends, seniors</t>
         </is>
       </c>
-      <c r="AC25" s="2" t="n">
+      <c r="AC25" s="3" t="n">
         <v>45944</v>
       </c>
       <c r="AD25" t="inlineStr">
@@ -5638,13 +5585,11 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
           <t>Muzeum Kornela Makuszyńskiego</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>Oddział Muzeum Tatrzańskiego poświęcony życiu i twórczości Kornela Makuszyńskiego.</t>
@@ -5660,7 +5605,6 @@
           <t>Muzeum to gratka dla miłośników literatury polskiej, szczególnie książek dla dzieci. Pozwala bliżej poznać niezwykłą postać Kornela Makuszyńskiego oraz poczuć atmosferę Zakopanego z początku XX wieku.</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>[
@@ -5763,7 +5707,7 @@
           <t>solo, couples, friends, family_kids, seniors</t>
         </is>
       </c>
-      <c r="AC26" s="2" t="n">
+      <c r="AC26" s="3" t="n">
         <v>45944</v>
       </c>
       <c r="AD26" t="inlineStr">
@@ -5840,13 +5784,11 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
           <t>Muzeum Stylu Zakopiańskiego im. S. Witkiewicza</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>Muzeum prezentujące historię i charakterystyczny styl zakopiański w architekturze i sztuce.</t>
@@ -5862,7 +5804,6 @@
           <t>To unikatowa okazja do zgłębienia dziedzictwa kulturowego regionu, zobaczenia oryginalnych projektów Stanisława Witkiewicza i lepszego zrozumienia charakterystycznej architektury Podhala.</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>[
@@ -5965,7 +5906,7 @@
           <t>solo, couples, friends, family_kids, seniors</t>
         </is>
       </c>
-      <c r="AC27" s="2" t="n">
+      <c r="AC27" s="3" t="n">
         <v>45944</v>
       </c>
       <c r="AD27" t="inlineStr">
@@ -6042,13 +5983,11 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
           <t>Galeria sztuki w willi Oksza</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>Galeria prezentująca zbiory sztuki w zabytkowej willi Oksza, będąca filią Muzeum Tatrzańskiego.</t>
@@ -6064,7 +6003,6 @@
           <t>To wyjątkowe miejsce, gdzie można podziwiać sztukę i architekturę regionu oraz dowiedzieć się więcej o artystycznej historii Zakopanego i Tatr.</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>[
@@ -6167,7 +6105,7 @@
           <t>solo, couples, friends, family_kids, seniors</t>
         </is>
       </c>
-      <c r="AC28" s="2" t="n">
+      <c r="AC28" s="3" t="n">
         <v>45944</v>
       </c>
       <c r="AD28" t="inlineStr">
@@ -6244,13 +6182,11 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
           <t>Muzeum Karola Szymanowskiego w willi "Atma"</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>Historyczna willa w stylu zakopiańskim, w której znajduje się muzeum poświęcone Karolowi Szymanowskiemu.</t>
@@ -6266,7 +6202,6 @@
           <t>To idealne miejsce dla miłośników muzyki, sztuki i historii Zakopanego, a także dla osób zainteresowanych życiem i twórczością Karola Szymanowskiego.</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>[
@@ -6368,7 +6303,7 @@
           <t>solo, couples, friends, family_kids, seniors</t>
         </is>
       </c>
-      <c r="AC29" s="2" t="n">
+      <c r="AC29" s="3" t="n">
         <v>45944</v>
       </c>
       <c r="AD29" t="inlineStr">
@@ -6445,13 +6380,11 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
           <t>Tatrzański Park Edukacyjny</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>Edukacyjny park zoologiczny, który przybliża przyrodę Tatr i kulturę góralską.</t>
@@ -6467,7 +6400,6 @@
           <t>To doskonałe miejsce do rodzinnego wypoczynku, poznawania zwierząt żyjących w Tatrach oraz ciekawostek o folklorze i przyrodzie regionu.</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>[
@@ -6650,13 +6582,11 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
           <t>Kaplica Najświętszego Serca Pana Jezusa w Jaszczurówce</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>Drewniana kaplica w stylu zakopiańskim, będąca jednym z najpiękniejszych przykładów architektury sakralnej regionu.</t>
@@ -6672,7 +6602,6 @@
           <t>To obowiązkowe miejsce dla miłośników stylu zakopiańskiego oraz osób chcących poznać kulturę i tradycje regionu podhalańskiego.</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>[
@@ -6853,13 +6782,11 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
           <t>KULIGI w Zakopanem</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>Organizator tradycyjnych kuligów z saniami i pochodniami po zakopiańskich okolicach.</t>
@@ -6875,7 +6802,6 @@
           <t>To niepowtarzalna okazja, by przeżyć autentyczny, zimowy kulig i poznać lokalne tradycje w wyjątkowej atmosferze zakopiańskiej zimy.</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>[
@@ -7067,13 +6993,11 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
           <t>Dolina Chochołowska</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>Najdłuższa i jedna z najpiękniejszych dolin w polskich Tatrach, popularna zarówno wśród turystów pieszych, jak i rowerzystów.</t>
@@ -7089,7 +7013,6 @@
           <t>To miejsce obowiązkowe dla miłośników przyrody, fotografów i osób szukających spokojnych wędrówek z dala od tłumów popularnych szlaków. Dolina Chochołowska oferuje niepowtarzalne widoki o każdej porze roku.</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>[
@@ -7161,8 +7084,6 @@
       <c r="Q33" t="n">
         <v>19.8333333</v>
       </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -7283,13 +7204,11 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
           <t>Dolina Kościeliska</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>Jedna z najpiękniejszych tatrzańskich dolin, słynąca z malowniczych krajobrazów, jaskiń i górskich szlaków.</t>
@@ -7305,7 +7224,6 @@
           <t>To jedno z must-see Tatr – niesamowite widoki, łatwy dostęp i ciekawe formacje skalne sprawiają, że wizyta w Dolinie Kościeliskiej dostarcza niezapomnianych wrażeń każdemu, bez względu na wiek czy doświadczenie górskie.</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>[
@@ -7378,8 +7296,6 @@
       <c r="Q34" t="n">
         <v>19.8666667</v>
       </c>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -7500,13 +7416,11 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
           <t>Rusinowa Polana</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>Malownicza polana w Tatrach, oferująca piękne widoki na okoliczne szczyty.</t>
@@ -7522,7 +7436,6 @@
           <t>Warto odwiedzić Rusinową Polanę dla spektakularnych panoram Tatr, unikalnego klimatu regionu i tradycyjnego pasterstwa.</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>[
@@ -7595,8 +7508,6 @@
       <c r="Q35" t="n">
         <v>20.0895038</v>
       </c>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -7717,13 +7628,11 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr">
         <is>
           <t>Morskie Oko</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>Największe i jedno z najpiękniejszych jezior w Tatrach, otoczone spektakularnymi szczytami górskimi.</t>
@@ -7739,7 +7648,6 @@
           <t>Morskie Oko zachwyca spektakularnymi krajobrazami i doskonałymi możliwościami do fotografii. Szlak do jeziora to popularna górska trasa, idealna dla osób szukających kontaktu z przyrodą i pięknymi widokami.</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>[
@@ -7812,8 +7720,6 @@
       <c r="Q36" t="n">
         <v>20.070087</v>
       </c>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -7934,13 +7840,11 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
           <t>Gubałówka</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
           <t>Gubałówka to jedna z największych atrakcji Zakopanegp. Na górze czekają piękne widoki na Tatry z Giewontem.</t>
@@ -7956,7 +7860,6 @@
           <t>Znajdziesz tu jedne najpiękniejszych widoków na Tatry i panoramę Zakopanego. Na górze czekają rodzinne atrakcje, regionalne przysmaki i wyjątkowy, góralski klimat.</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>{
@@ -8005,8 +7908,6 @@
       <c r="Q37" t="n">
         <v>19.9454830120256</v>
       </c>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -8127,13 +8028,11 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
           <t>Snowdoo Adventure</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
           <t>Ośrodek oferujący wyprawy skuterami śnieżnymi i atrakcje zimowe.</t>
@@ -8149,7 +8048,6 @@
           <t>To wyjątkowa propozycja dla miłośników adrenaliny i aktywnego spędzania czasu na świeżym powietrzu w otoczeniu tatrzańskich krajobrazów.</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t xml:space="preserve">{
@@ -8199,8 +8097,6 @@
       <c r="Q38" t="n">
         <v>19.9128467</v>
       </c>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -8321,13 +8217,11 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
           <t xml:space="preserve">Kolejka linowa na Kasprowy Wierch </t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>Kolejka linowa prowadzącej na szczyt Kasprowego Wierchu.</t>
@@ -8343,7 +8237,6 @@
           <t>To idealne miejsce, by rozpocząć podróż na jeden z najpopularniejszych szczytów Tatr, zarówno zimą, jak i latem. Wjazd kolejką pozwala podziwiać wyjątkowe widoki i uniknąć mozolnej wędrówki na szczyt.</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>{
@@ -8566,13 +8459,11 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
           <t>Droga pod Reglami</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
           <t>Malowniczy szlak pieszy biegnący wzdłuż północnych zboczy Tatr, idealny na spacer i podziwianie przyrody.</t>
@@ -8588,7 +8479,6 @@
           <t>Idealna propozycja dla osób szukających łatwej trasy w Tatrach, z pięknymi widokami i możliwością odpoczynku z dala od tłumu. Droga pod Reglami pozwala odkrywać uroki tatrzańskich dolin bez konieczności intensywnego wspinania.</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>{
@@ -8648,8 +8538,6 @@
       <c r="Q40" t="n">
         <v>19.9813526</v>
       </c>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -8770,13 +8658,11 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
           <t>Dolina Strążyska</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>Malownicza dolina tatrzańska prowadząca u stóp Giewontu, popularna wśród turystów pieszych.</t>
@@ -8792,7 +8678,6 @@
           <t>To jedno z najładniejszych i najłatwiejszych do przejścia miejsc w Tatrach, idealne zarówno dla rodzin z dziećmi, jak i osób ceniących spokojną przyrodę, a także fotografów krajobrazowych.</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>{
@@ -8852,8 +8737,6 @@
       <c r="Q41" t="n">
         <v>19.9333087</v>
       </c>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -8974,13 +8857,11 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
           <t>Dolina ku Dziurze</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>Mała, malownicza dolina tatrzańska znana z naturalnej jaskini Dziura.</t>
@@ -8996,7 +8877,6 @@
           <t>To łatwo dostępna dolinka, oferująca piękne widoki i unikalną jaskinię. Jest idealna na krótki wypad, szczególnie dla osób, które chcą szybko poczuć klimat Tatr bez długich, męczących wędrówek.</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>{
@@ -9056,8 +8936,6 @@
       <c r="Q42" t="n">
         <v>19.9411407</v>
       </c>
-      <c r="R42" t="inlineStr"/>
-      <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -9178,13 +9056,11 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
           <t>Polana Kalatówki</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>Malownicza polana położona w Tatrach, otoczona lasami i górami, popularna wśród turystów oraz miłośników wypoczynku na łonie natury.</t>
@@ -9200,7 +9076,6 @@
           <t>Warto odwiedzić to miejsce ze względu na wspaniałe widoki, atmosferę spokoju i możliwość łatwego kontaktu z tatrzańską przyrodą. Polana Kalatówki to jedno z najbardziej dostępnych i malowniczych miejsc w okolicach Zakopanego.</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>{
@@ -9260,8 +9135,6 @@
       <c r="Q43" t="n">
         <v>19.9683412</v>
       </c>
-      <c r="R43" t="inlineStr"/>
-      <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -9382,13 +9255,11 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
           <t>Punkt widokowy na Tatry</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>Punkt widokowy oferujący panoramę Tatr.</t>
@@ -9404,7 +9275,6 @@
           <t>To doskonałe miejsce, by zobaczyć piękno Tatr z innej perspektywy oraz zrobić wyjątkowe zdjęcia krajobrazowe.</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>{
@@ -9464,8 +9334,6 @@
       <c r="Q44" t="n">
         <v>20.0107764</v>
       </c>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -9586,13 +9454,11 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
           <t>Wodospad Siklawica</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>Malowniczy wodospad położony u podnóża Giewontu w Tatrach Zachodnich.</t>
@@ -9608,7 +9474,6 @@
           <t>To jedno z piękniejszych naturalnych miejsc w okolicy Zakopanego, idealne na krótki spacer z zachwycającymi widokami i możliwością kontaktu z naturą.</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>{
@@ -9668,8 +9533,6 @@
       <c r="Q45" t="n">
         <v>19.9302071</v>
       </c>
-      <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -9790,13 +9653,11 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr">
         <is>
           <t>Olczyska Polana</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
           <t>Malownicza polana położona na terenie Tatrzańskiego Parku Narodowego, idealna do pieszych wycieczek i wypoczynku na łonie natury.</t>
@@ -9812,7 +9673,6 @@
           <t>To świetne miejsce, aby odpocząć od tłoku Zakopanego i podziwiać naturalne piękno Tatr. Spacer na Olczyską Polanę to łagodna i dostępna trasa nawet dla rodzin z dziećmi.</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>{
@@ -9872,8 +9732,6 @@
       <c r="Q46" t="n">
         <v>20.0005687</v>
       </c>
-      <c r="R46" t="inlineStr"/>
-      <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -9994,13 +9852,11 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
           <t>Polana Jaworzynka</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>Malownicza polana w Tatrach, popularna wśród spacerowiczów i miłośników przyrody.</t>
@@ -10016,7 +9872,6 @@
           <t>Warto odwiedzić Polanę Jaworzynka, by wypocząć na łonie natury, podziwiać malownicze panoramy oraz poczuć niepowtarzalny klimat tatrzańskiej doliny.</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>{
@@ -10076,8 +9931,6 @@
       <c r="Q47" t="n">
         <v>19.9846641</v>
       </c>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -10198,13 +10051,11 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr">
         <is>
           <t>Sarni Wodospad</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
           <t>Malowniczy, niewielki wodospad położony na obrzeżach Zakopanego, wśród tatrzańskiej przyrody.</t>
@@ -10220,7 +10071,6 @@
           <t>To doskonałe miejsce, aby zrelaksować się w otoczeniu przyrody, z dala od tłumów i miejskiego zgiełku. Idealny punkt na krótki postój podczas wycieczek poza centrum Zakopanego.</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>{
@@ -10280,8 +10130,6 @@
       <c r="Q48" t="n">
         <v>19.9544844</v>
       </c>
-      <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -10402,13 +10250,11 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
           <t>Wielka Polana Małołącka</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
           <t>Szeroka polana górska położona w Dolinie Małej Łąki, otoczona malowniczymi szczytami Tatr Zachodnich.</t>
@@ -10424,7 +10270,6 @@
           <t>To idealne miejsce na relaks wśród natury, podziwianie tatrzańskich krajobrazów i piknik w górskim otoczeniu. Polana zachwyca ciszą i przestrzenią, a jednocześnie jest łatwo dostępna nawet dla osób mniej doświadczonych w górach.</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>{
@@ -10484,8 +10329,6 @@
       <c r="Q49" t="n">
         <v>19.9043787</v>
       </c>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -10606,13 +10449,11 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr">
         <is>
           <t>Dolina Za Bramką</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
           <t>Malownicza dolina tatrzańska idealna na spokojne spacery.</t>
@@ -10628,7 +10469,6 @@
           <t>Warto odwiedzić tę dolinę, by odpocząć od tłumów, podziwiać dziewiczą przyrodę i zrelaksować się na łonie Tatr.</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>{
@@ -10688,8 +10528,6 @@
       <c r="Q50" t="n">
         <v>19.9171668</v>
       </c>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -10810,13 +10648,11 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr">
         <is>
           <t>Dolina Suchej Wody</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>Malownicza dolina tatrzańska znajdująca się w rejonie Zakopanego.</t>
@@ -10832,7 +10668,6 @@
           <t>Jest to idealne miejsce na rozpoczęcie wędrówki w wyższe partie Tatr i podziwianie wyjątkowych widoków oraz alpejskiej przyrody.</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>{
@@ -10892,8 +10727,6 @@
       <c r="Q51" t="n">
         <v>20.0359096</v>
       </c>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -11014,13 +10847,11 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr">
         <is>
           <t>Dolina Gąsienicowa</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
           <t>Malownicza dolina tatrzańska, popularna wśród turystów i miłośników górskich wędrówek.</t>
@@ -11036,7 +10867,6 @@
           <t>To miejsce obowiązkowe dla każdego miłośnika Tatr – urzeka nie tylko widokami, lecz również bogactwem górskiej przyrody i atmosferą schroniska. Stanowi początek wielu fascynujących tras trekkingowych.</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
           <t>{
@@ -11096,8 +10926,6 @@
       <c r="Q52" t="n">
         <v>20.0063853</v>
       </c>
-      <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -11218,13 +11046,11 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr">
         <is>
           <t>Park Miejski im. Marszałka Józefa Piłsudskiego</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
           <t>Zielona oaza w centrum Zakopanego z alejkami spacerowymi, placem zabaw i miejscami do odpoczynku.</t>
@@ -11240,7 +11066,6 @@
           <t>Warto odwiedzić park, aby odpocząć od zgiełku Zakopanego, nacieszyć się przyrodą i skorzystać z licznych atrakcji na świeżym powietrzu.</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>{
@@ -11300,8 +11125,6 @@
       <c r="Q53" t="n">
         <v>19.95507</v>
       </c>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -11422,13 +11245,11 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr">
         <is>
           <t>Chałupa Sabały</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
           <t>Zabytkowa, drewniana chałupa rodem z XIX wieku, będąca dawnym domem góralskiego muzyka Jana Krzeptowskiego Sabały.</t>
@@ -11444,7 +11265,6 @@
           <t>Warto odwiedzić to miejsce, aby poczuć ducha dawnego Zakopanego, zobaczyć tradycyjną góralską izbę oraz poznać historię jednej z najbardziej barwnych postaci Tatr. Chałupa pozwala lepiej zrozumieć historię i kulturę regionu podhalańskiego.</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>{
@@ -11493,8 +11313,6 @@
       <c r="Q54" t="n">
         <v>19.9193173</v>
       </c>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
       <c r="T54" t="inlineStr">
         <is>
           <t>mixed</t>
@@ -11615,13 +11433,11 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr">
         <is>
           <t>Quady Adventure Zakopane Wypożyczalnia</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
           <t>Wypożyczalnia quadów i buggy oferująca wycieczki terenowe w okolicach Poronina.</t>
@@ -11637,7 +11453,6 @@
           <t>To doskonały sposób na aktywne spędzenie czasu, podziwianie górskich krajobrazów i przeżycie motoryzacyjnej przygody, dostępny zarówno dla początkujących, jak i zaawansowanych.</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>{
@@ -11686,8 +11501,6 @@
       <c r="Q55" t="n">
         <v>19.9937334</v>
       </c>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
       <c r="T55" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -11808,13 +11621,11 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr">
         <is>
           <t>Cudakowa Polana</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>Malownicza polana położona przy czarnym szlaku turystycznym w Tatrach.</t>
@@ -11830,7 +11641,6 @@
           <t>Warto odwiedzić Cudakową Polanę, aby nacieszyć się wspaniałymi widokami oraz doświadczyć klimatu górskiej przyrody z dala od miejskiego zgiełku.</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>{
@@ -11874,7 +11684,6 @@
       <c r="M56" t="n">
         <v>5.5</v>
       </c>
-      <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr">
         <is>
           <t>Małopolska</t>
@@ -11886,8 +11695,6 @@
       <c r="Q56" t="n">
         <v>19.8693207</v>
       </c>
-      <c r="R56" t="inlineStr"/>
-      <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -12008,13 +11815,11 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr">
         <is>
           <t xml:space="preserve"> Beernarium Piwne Spa</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>Relaksacyjne spa oferujące kąpiele piwne i zabiegi wellness.</t>
@@ -12030,7 +11835,6 @@
           <t>Wizyta w Beernarium Piwnym Spa to szansa na relaks i regenerację w niepowtarzalnej, piwnej atmosferze, jakiej nie znajdziemy w typowych spa. Kąpiele w piwie mają korzystny wpływ na skórę i samopoczucie.</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>{
@@ -12079,8 +11883,6 @@
       <c r="Q57" t="n">
         <v>19.9623495</v>
       </c>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
       <c r="T57" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -12201,13 +12003,11 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr">
         <is>
           <t>Iria Spa</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
           <t>Nowoczesne spa oferujące szeroki zakres zabiegów relaksacyjnych i pielęgnacyjnych.</t>
@@ -12223,7 +12023,6 @@
           <t>To doskonałe miejsce, aby zatroszczyć się o swoje zdrowie i dobre samopoczucie, odprężyć się oraz skorzystać z wysokiej jakości zabiegów w przyjaznej atmosferze.</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>{
@@ -12402,13 +12201,11 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr"/>
       <c r="B59" t="inlineStr">
         <is>
           <t>Polana Głodówka</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
           <t>Malownicza polana z panoramicznym widokiem na Tatry.</t>
@@ -12424,7 +12221,6 @@
           <t>To idealne miejsce, aby podziwiać panoramę Tatr, zrobić zdjęcia oraz odpocząć na łonie przyrody, z dala od gwaru kurortów.</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>{
@@ -12484,8 +12280,6 @@
       <c r="Q59" t="n">
         <v>20.1174987</v>
       </c>
-      <c r="R59" t="inlineStr"/>
-      <c r="S59" t="inlineStr"/>
       <c r="T59" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -12606,13 +12400,11 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr"/>
       <c r="B60" t="inlineStr">
         <is>
           <t>Park Przygody Gubałówka</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
           <t>Park linowy na Gubałówce oferujący trasy o różnym stopniu trudności.</t>
@@ -12628,7 +12420,6 @@
           <t>To świetna propozycja dla osób żądnych aktywności i lubiących wyzwania, a także dla rodzin z dziećmi. Ropes Gold Ridge łączy sportową zabawę ze wspaniałymi widokami na Tatry.</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>{
@@ -12677,7 +12468,6 @@
       <c r="Q60" t="n">
         <v>19.9310972</v>
       </c>
-      <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr">
         <is>
           <t>https://park-przygody-gubalowka.pl/cennik/</t>
@@ -12803,13 +12593,11 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr"/>
       <c r="B61" t="inlineStr">
         <is>
           <t>Cmentarz Zasłużonych na Pęksowym Brzyzku</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
           <t>Historyczny cmentarz, miejsce pochówku znanych osób zasłużonych dla regionu Tatr i Zakopanego.</t>
@@ -12825,7 +12613,6 @@
           <t>Warto odwiedzić to miejsce, aby poznać historię regionu, oddać hołd wybitnym postaciom i podziwiać unikalne nagrobki będące dziełami lokalnych rzemieślników.</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>{
@@ -12874,8 +12661,6 @@
       <c r="Q61" t="n">
         <v>19.9470409</v>
       </c>
-      <c r="R61" t="inlineStr"/>
-      <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -12996,13 +12781,11 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr">
         <is>
           <t>Dwór Tetmajerów</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
           <t>Zabytkowy dwór szlachecki będący filią Muzeum Tatrzańskiego, prezentujący kulturę regionu i historię rodu Tetmajerów.</t>
@@ -13018,7 +12801,6 @@
           <t>To miejsce łączy historię, tradycję i piękno architektury regionu, pozwalając lepiej zrozumieć bogatą kulturę Podhala oraz losy słynnej rodziny Tetmajerów.</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>{
@@ -13067,8 +12849,6 @@
       <c r="Q62" t="n">
         <v>20.1277911</v>
       </c>
-      <c r="R62" t="inlineStr"/>
-      <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr">
         <is>
           <t>mixed</t>
@@ -13189,13 +12969,11 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr"/>
       <c r="B63" t="inlineStr">
         <is>
           <t>Sanktuarium Wiktorówki</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
           <t>Sanktuarium Matki Bożej Królowej Tatr, popularne miejsce pielgrzymkowe i turystyczne w Tatrach.</t>
@@ -13211,7 +12989,6 @@
           <t>To wyjątkowe miejsce, gdzie można połączyć kontakt z przyrodą ze spokojem i duchowym wytchnieniem. Kaplica na Wiktorówkach to nie tylko cel religijny, ale także doskonały punkt na trasie wędrówek po Tatrach.</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
           <t>{
@@ -13260,8 +13037,6 @@
       <c r="Q63" t="n">
         <v>20.086447</v>
       </c>
-      <c r="R63" t="inlineStr"/>
-      <c r="S63" t="inlineStr"/>
       <c r="T63" t="inlineStr">
         <is>
           <t>mixed</t>
@@ -13382,13 +13157,11 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr">
         <is>
           <t>Snow Zabawa – zimowe atrakcje</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
           <t>Miejsce oferujące różnorodne zimowe atrakcje i zabawy na śniegu dla całych rodzin.</t>
@@ -13404,7 +13177,6 @@
           <t>To świetna okazja, aby aktywnie spędzić czas zimą, korzystając z bogatej oferty atrakcji na świeżym powietrzu, ciesząc się pięknymi widokami Tatr oraz lokalnym klimatem.</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>{
@@ -13426,7 +13198,6 @@
       <c r="J64" t="n">
         <v>180</v>
       </c>
-      <c r="K64" t="inlineStr"/>
       <c r="L64" t="n">
         <v>30</v>
       </c>
@@ -13450,8 +13221,6 @@
       <c r="Q64" t="n">
         <v>19.9045138</v>
       </c>
-      <c r="R64" t="inlineStr"/>
-      <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -13572,13 +13341,11 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr">
         <is>
           <t>Krupówki</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
           <t>Główna ulica spacerowa i handlowa w Zakopanem, pełna sklepów, restauracji oraz atrakcji kulturalnych.</t>
@@ -13594,7 +13361,6 @@
           <t>Krupówki to prawdziwe serce Zakopanego; miejsce, gdzie można poczuć góralską atmosferę, skosztować regionalnej kuchni, kupić pamiątki, a także obserwować codzienne życie mieszkańców i turystów.</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
           <t>{
@@ -13777,13 +13543,11 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr">
         <is>
           <t>Dolna Rówień Krupowa</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
           <t>Rozległy, zielony park w centrum Zakopanego, popularny na spacery oraz rekreację.</t>
@@ -13799,7 +13563,6 @@
           <t>To idealne miejsce na relaks po zwiedzaniu Zakopanego lub szlakach górskich. Można tu odpocząć, podziwiać panoramę gór, aktywnie spędzić czas z rodziną lub spotkać się na piknik.</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>{
@@ -13859,8 +13622,6 @@
       <c r="Q66" t="n">
         <v>19.9559261</v>
       </c>
-      <c r="R66" t="inlineStr"/>
-      <c r="S66" t="inlineStr"/>
       <c r="T66" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -13985,13 +13746,11 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr"/>
       <c r="B67" t="inlineStr">
         <is>
           <t>Muzeum Jana Kasprowicza</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
           <t>Muzeum poświęcone życiu i twórczości poety Jana Kasprowicza.</t>
@@ -14007,7 +13766,6 @@
           <t>To wyjątkowa okazja, by poznać historię życia Jana Kasprowicza – jednego z najwybitniejszych polskich poetów, a także zobaczyć wnętrza willi z początku XX wieku.</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
           <t>{
@@ -14186,13 +13944,11 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr"/>
       <c r="B68" t="inlineStr">
         <is>
           <t>Willa Koliba</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
           <t>Pierwszy dom w stylu zakopiańskim, mieszczący muzeum poświęcone temu unikalnemu nurtowi architektonicznemu.</t>
@@ -14208,7 +13964,6 @@
           <t>To obowiązkowe miejsce dla miłośników sztuki, architektury i historii regionu. Możesz poczuć klimat dawnego Zakopanego i odkryć źródła stylu zakopiańskiego.</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
           <t>{
@@ -14387,13 +14142,11 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr"/>
       <c r="B69" t="inlineStr">
         <is>
           <t>Kaplica Gąsieniców na Pęksowym Brzyzku pw. św. Andrzeja i św. Benedykta</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
           <t>Drewniana kaplica z XIX wieku, najstarszy obiekt sakralny Zakopanego, położona na zabytkowym cmentarzu Pęksowym Brzyzku.</t>
@@ -14409,7 +14162,6 @@
           <t>To miejsce o wyjątkowym znaczeniu historycznym i kulturalnym, idealne dla osób chcących poznać początki Zakopanego i tradycje regionu. Cicha, klimatyczna kaplica i zabytkowy cmentarz tworzą niezwykłą przestrzeń do zadumy oraz spotkania z dziedzictwem Podhala.</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
           <t>{
@@ -14469,8 +14221,6 @@
       <c r="Q69" t="n">
         <v>19.9464968</v>
       </c>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
       <c r="T69" t="inlineStr">
         <is>
           <t>mixed</t>
@@ -14591,13 +14341,11 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr"/>
       <c r="B70" t="inlineStr">
         <is>
           <t>Galeria Władysława Hasiora</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
           <t>Galeria poświęcona twórczości Władysława Hasiora, wybitnego artysty i rzeźbiarza, będąca filią Muzeum Tatrzańskiego.</t>
@@ -14613,7 +14361,6 @@
           <t>To obowiązkowy punkt dla miłośników sztuki współczesnej oraz osób pragnących bliżej poznać sylwetkę i twórczość Władysława Hasiora, który w oryginalny sposób łączył kulturę ludową z nowoczesnością.</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>{
@@ -14792,13 +14539,11 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr"/>
       <c r="B71" t="inlineStr">
         <is>
           <t>SkyWalk Serce Poronina</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
           <t>Platforma widokowa z panoramicznym widokiem na Tatry i okolice.</t>
@@ -14814,7 +14559,6 @@
           <t>Warto odwiedzić SkyWalk Serce Poronina, aby doświadczyć spektakularnych górskich widoków i zrobić pamiątkowe zdjęcia w wyjątkowym miejscu, które łączy nowoczesność z pięknem tatrzańskiej przyrody.</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>{
@@ -15026,13 +14770,11 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr"/>
       <c r="B72" t="inlineStr">
         <is>
           <t>BeHappy Muzeum Zakopane</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
           <t>Interaktywne muzeum z kolorowymi instalacjami do zdjęć.</t>
@@ -15048,7 +14790,6 @@
           <t>Atrakcja oferuje mnóstwo radości, kreatywnych inspiracji i okazji do zrobienia unikalnych, wesołych zdjęć w ciekawie zaaranżowanych przestrzeniach.</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>{
@@ -15227,13 +14968,11 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr"/>
       <c r="B73" t="inlineStr">
         <is>
           <t>Polana Szymoszkowa</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
           <t>Popularna stacja narciarska i rekreacyjna z pięknym widokiem na Tatry.</t>
@@ -15249,7 +14988,6 @@
           <t>To świetne miejsce zarówno dla miłośników sportów zimowych, jak i dla osób szukających relaksu w górach. Różnorodność atrakcji oraz piękne widoki sprawiają, że każdy znajdzie tu coś dla siebie.</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>{
@@ -15309,7 +15047,6 @@
       <c r="Q73" t="n">
         <v>19.9296709</v>
       </c>
-      <c r="R73" t="inlineStr"/>
       <c r="S73" t="inlineStr">
         <is>
           <t>https://szymoszkowa.pl/cennik-przejazdow-turystycznych/</t>
@@ -15435,13 +15172,11 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr"/>
       <c r="B74" t="inlineStr">
         <is>
           <t>Królikarnia Zakopane</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
           <t>Małe prywatne mini-zoo w Zakopanem, w którym można zobaczyć króliki oraz inne drobne zwierzęta.</t>
@@ -15457,7 +15192,6 @@
           <t>To świetna opcja na relaksującą wizytę dla rodzin z dziećmi oraz miłośników zwierząt. Pozwala na bliski kontakt ze zwierzętami oraz odpoczynek w otoczeniu natury.</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
           <t>{
@@ -15506,8 +15240,6 @@
       <c r="Q74" t="n">
         <v>19.9532834</v>
       </c>
-      <c r="R74" t="inlineStr"/>
-      <c r="S74" t="inlineStr"/>
       <c r="T74" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -15628,13 +15360,11 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr"/>
       <c r="B75" t="inlineStr">
         <is>
           <t>Kąpielisko na Polanie Szymoszkowej</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
           <t>Unikalny basen geotermalny z widokiem na Tatry.</t>
@@ -15650,7 +15380,6 @@
           <t>To idealne miejsce na odpoczynek po górskich wędrówkach, a przy tym świetna rozrywka dla całej rodziny w sercu Tatr.</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
           <t>{
@@ -15699,7 +15428,6 @@
       <c r="Q75" t="n">
         <v>19.9324219</v>
       </c>
-      <c r="R75" t="inlineStr"/>
       <c r="S75" t="inlineStr">
         <is>
           <t>https://szymoszkowa.pl/cennik-kapieliska/</t>
@@ -15825,13 +15553,11 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr"/>
       <c r="B76" t="inlineStr">
         <is>
           <t>Bacówka zakopiańczyk</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr">
         <is>
           <t>Tradycyjna bacówka oferująca regionalne sery i produkty góralskie.</t>
@@ -15847,7 +15573,6 @@
           <t>Warto odwiedzić Bacówkę Zakopiańczyk, aby spróbować autentycznych serów z mleka owczego i doświadczyć żywej tradycji góralskiej. To idealne miejsce na zakup lokalnych przysmaków i oryginalnych pamiątek z regionu.</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>{
@@ -15896,8 +15621,6 @@
       <c r="Q76" t="n">
         <v>19.958669</v>
       </c>
-      <c r="R76" t="inlineStr"/>
-      <c r="S76" t="inlineStr"/>
       <c r="T76" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -15939,7 +15662,6 @@
           <t>couples, seniors friends</t>
         </is>
       </c>
-      <c r="AC76" t="inlineStr"/>
       <c r="AD76" t="inlineStr">
         <is>
           <t>local_food_experience</t>
@@ -16014,13 +15736,11 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr"/>
       <c r="B77" t="inlineStr">
         <is>
           <t>Dom Oscypka w Zakopanem</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr">
         <is>
           <t>Miejsce, gdzie można poznać tradycję wyrobu oscypka i wziąć udział w warsztatach na żywo.</t>
@@ -16036,7 +15756,6 @@
           <t>To idealne miejsce, aby lepiej poznać kulturę Podhala, spróbować tradycyjnych serów i zabrać do domu własnoręcznie zrobionego oscypka.</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
           <t>{
@@ -16085,8 +15804,6 @@
       <c r="Q77" t="n">
         <v>19.9549909</v>
       </c>
-      <c r="R77" t="inlineStr"/>
-      <c r="S77" t="inlineStr"/>
       <c r="T77" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -16207,13 +15924,11 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr">
         <is>
           <t>Targowisko pod Gubałówką</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
           <t>Popularny bazar zlokalizowany u stóp Gubałówki w Zakopanem, oferujący lokalne produkty, pamiątki oraz wyroby regionalne.</t>
@@ -16229,7 +15944,6 @@
           <t>To idealne miejsce, by poczuć klimat Zakopanego, kupić regionalne przysmaki i oryginalne pamiątki oraz spotkać autentycznych producentów z Podhala.</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
           <t>{
@@ -16278,8 +15992,6 @@
       <c r="Q78" t="n">
         <v>19.9464494</v>
       </c>
-      <c r="R78" t="inlineStr"/>
-      <c r="S78" t="inlineStr"/>
       <c r="T78" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -16321,7 +16033,6 @@
           <t>couples, seniors</t>
         </is>
       </c>
-      <c r="AC78" t="inlineStr"/>
       <c r="AD78" t="inlineStr">
         <is>
           <t>food_market</t>
@@ -16396,13 +16107,11 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr"/>
       <c r="B79" t="inlineStr">
         <is>
           <t>Bachledówka</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
           <t>Bachledówka to malownicze wzniesienie niedaleko Zakopanego. Na szczycie znajduje się sanktuarium, a z okolicy można podziwiać piękne panoramy Tatr i Podhala.</t>
@@ -16418,7 +16127,6 @@
           <t>To idealne miejsce na chwilę odpoczynku i podziwianie górskich krajobrazów.</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
           <t>{
@@ -16467,8 +16175,6 @@
       <c r="Q79" t="n">
         <v>19.9192039620706</v>
       </c>
-      <c r="R79" t="inlineStr"/>
-      <c r="S79" t="inlineStr"/>
       <c r="T79" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -16510,7 +16216,6 @@
           <t>seniors, couples</t>
         </is>
       </c>
-      <c r="AC79" t="inlineStr"/>
       <c r="AD79" t="inlineStr">
         <is>
           <t>nature_landscape</t>
@@ -16585,13 +16290,11 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr"/>
       <c r="B80" t="inlineStr">
         <is>
           <t>Punkt widokowy na Antałówce</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
           <t>Punkt widokowy na Antałówce to spokojne miejsce w centrum Zakopanego z piękną panoramą Tatr. Idealne na krótki odpoczynek, zdjęcia lub piknik przy zachodzie słońca.</t>
@@ -16607,7 +16310,6 @@
           <t>Warto odwiedzić Antałówkę, by podziwiać piękne widoki na Tatry oraz miasto Zakopane.</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
           <t>{
@@ -16656,8 +16358,6 @@
       <c r="Q80" t="n">
         <v>19.9724934</v>
       </c>
-      <c r="R80" t="inlineStr"/>
-      <c r="S80" t="inlineStr"/>
       <c r="T80" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -16784,13 +16484,11 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr"/>
       <c r="B81" t="inlineStr">
         <is>
           <t>Tatrzańskie Archiwum Planety Ziemia</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
           <t>Nowoczesne centrum edukacyjne przybliżające faunę, florę i geologię Tatr.</t>
@@ -16806,7 +16504,6 @@
           <t>Miejsce idealne dla rodzin z dziećmi i osób zainteresowanych przyrodą Tatr. Pozwala w atrakcyjny sposób poznać unikatowy świat tatrzańskiej przyrody i przygotować się do wycieczek terenowych.</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
           <t>[
@@ -16868,8 +16565,6 @@
       <c r="Q81" t="n">
         <v>19.868302</v>
       </c>
-      <c r="R81" t="inlineStr"/>
-      <c r="S81" t="inlineStr"/>
       <c r="T81" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -16995,13 +16690,11 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr"/>
       <c r="B82" t="inlineStr">
         <is>
           <t>Bachledzki Wierch</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
           <t>Bachledzki Wierch to widokowe wzniesienie położone w Zakopanem, popularne wśród spacerowiczów oraz turystów ceniących spokojne trasy i panoramę Tatr.</t>
@@ -17017,7 +16710,6 @@
           <t>Ze względu na rozległe widoki i mniej uczęszczane ścieżki, Bachledzki Wierch to doskonałe miejsce na spokojny spacer z dala od tłumów oraz na podziwianie panoramy Tatr i Zakopanego.</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
           <t>{
@@ -17066,8 +16758,6 @@
       <c r="Q82" t="n">
         <v>19.9718091</v>
       </c>
-      <c r="R82" t="inlineStr"/>
-      <c r="S82" t="inlineStr"/>
       <c r="T82" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -17194,13 +16884,11 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr"/>
       <c r="B83" t="inlineStr">
         <is>
           <t>Centrum Kultury Rodzimej w willi Czerwony Dwór</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
           <t>Zabytkowa willa prezentująca sztukę i kulturę regionu Podhala.</t>
@@ -17216,7 +16904,6 @@
           <t>To wyjątkowe miejsce pozwalające poznać podhalańską sztukę, kulturę i architekturę w autentycznym otoczeniu historycznej willi.</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
           <t>{
@@ -17265,8 +16952,6 @@
       <c r="Q83" t="n">
         <v>19.9484177</v>
       </c>
-      <c r="R83" t="inlineStr"/>
-      <c r="S83" t="inlineStr"/>
       <c r="T83" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -17308,7 +16993,6 @@
           <t>seniors, solo</t>
         </is>
       </c>
-      <c r="AC83" t="inlineStr"/>
       <c r="AD83" t="inlineStr">
         <is>
           <t>museum_heritage</t>
@@ -17389,13 +17073,11 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr"/>
       <c r="B84" t="inlineStr">
         <is>
           <t>Spływy Dunajcem tratwami flisackimi</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
           <t>Tradycyjne spływy tratwami przełomem Dunajca.</t>
@@ -17411,7 +17093,6 @@
           <t>Wyjątkowa okazja, by przeżyć tradycyjny, historyczny spływ z flisakami pośród spektakularnych krajobrazów Pienin. Biuro to punkt startowy dla tej niezapomnianej przygody.</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
           <t>[
@@ -17495,8 +17176,6 @@
       <c r="Q84" t="n">
         <v>20.368371</v>
       </c>
-      <c r="R84" t="inlineStr"/>
-      <c r="S84" t="inlineStr"/>
       <c r="T84" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -17607,7 +17286,7 @@
       </c>
       <c r="AR84" t="inlineStr">
         <is>
-          <t>river, rafting, sightseeing, scenic_views, family_friendly, outdoor, local_tradition</t>
+          <t>history_mystery, legend_story, local_tradition, scenic_view, outdoor, family_friendly, rafting</t>
         </is>
       </c>
       <c r="AS84" t="inlineStr">
@@ -17617,13 +17296,11 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr"/>
       <c r="B85" t="inlineStr">
         <is>
           <t>Zamek w Niedzicy</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
           <t>Malowniczo położony średniowieczny zamek nad Jeziorem Czorsztyńskim.</t>
@@ -17639,7 +17316,6 @@
           <t>Zamek Dunajec to jeden z najważniejszych zabytków regionu, oferujący fascynującą podróż przez historię, piękne widoki i unikalną atmosferę średniowiecznej twierdzy.</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t xml:space="preserve">
@@ -17703,8 +17379,6 @@
       <c r="Q85" t="n">
         <v>20.3196436</v>
       </c>
-      <c r="R85" t="inlineStr"/>
-      <c r="S85" t="inlineStr"/>
       <c r="T85" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -17815,7 +17489,7 @@
       </c>
       <c r="AR85" t="inlineStr">
         <is>
-          <t>castle, history, legends, architecture, panoramic_views, sightseeing</t>
+          <t>history_mystery, local_history, legends, historic_building, regional_heritage, architecture_heritage, panoramic_view, sightseeing</t>
         </is>
       </c>
       <c r="AS85" t="inlineStr">
@@ -17825,13 +17499,11 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr"/>
       <c r="B86" t="inlineStr">
         <is>
           <t>Rejs statkiem po jeziorze Czorsztyńskim</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
           <t>Rejsy turystyczne po malowniczym jeziorze Czorsztyńskim ze wspaniałymi widokami na okoliczne zamki i Tatry.</t>
@@ -17847,7 +17519,6 @@
           <t>To wyjątkowa okazja, aby podziwiać naturę i zabytki regionu z pokładu statku oraz poczuć klimat górskiej przygody na wodzie.</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>{
@@ -17896,8 +17567,6 @@
       <c r="Q86" t="n">
         <v>20.317104</v>
       </c>
-      <c r="R86" t="inlineStr"/>
-      <c r="S86" t="inlineStr"/>
       <c r="T86" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -18008,7 +17677,7 @@
       </c>
       <c r="AR86" t="inlineStr">
         <is>
-          <t>boat_trip, lake, scenic_views, relaxation, sightseeing, family_friendly</t>
+          <t>history_mystery, scenic_view, relaxation, sightseeing, family_friendly, boat_trip</t>
         </is>
       </c>
       <c r="AS86" t="inlineStr">
@@ -18018,13 +17687,11 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr"/>
       <c r="B87" t="inlineStr">
         <is>
           <t>Zamek w Czorsztynie</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
           <t>Malownicze ruiny średniowiecznego zamku położone nad Jeziorem Czorsztyńskim.</t>
@@ -18040,7 +17707,6 @@
           <t>Zamek Czorsztyn to doskonałe miejsce zarówno dla miłośników historii, jak i osób spragnionych pięknych krajobrazów. Zwiedzanie ruin pozwala przenieść się w czasie, a rozciągające się wokół widoki pozostają na długo w pamięci.</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
           <t>[
@@ -18102,8 +17768,6 @@
       <c r="Q87" t="n">
         <v>20.3132003</v>
       </c>
-      <c r="R87" t="inlineStr"/>
-      <c r="S87" t="inlineStr"/>
       <c r="T87" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -18214,7 +17878,7 @@
       </c>
       <c r="AR87" t="inlineStr">
         <is>
-          <t>castle_ruins, history, legends, architecture, panoramic_views, sightseeing</t>
+          <t>history_mystery, historic_ruins, legends, local_history, historic_building, regional_heritage, architecture_heritage, panoramic_view</t>
         </is>
       </c>
       <c r="AS87" t="inlineStr">
@@ -18224,13 +17888,11 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr"/>
       <c r="B88" t="inlineStr">
         <is>
           <t>Wąwóz Homole</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
           <t>Malowniczy wąwóz skalny z krystalicznym potokiem i licznymi trasami spacerowymi.</t>
@@ -18246,7 +17908,6 @@
           <t>Wąwóz Homole zapewnia unikalne wrażenia krajobrazowe i bliskość natury, jest łatwo dostępny zarówno dla rodzin z dziećmi, jak i miłośników górskich wędrówek. Spacer przez wąwóz pozwala odpocząć od miejskiego zgiełku i odkryć bogatą faunę oraz florę regionu.</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>{
@@ -18295,8 +17956,6 @@
       <c r="Q88" t="n">
         <v>20.548795</v>
       </c>
-      <c r="R88" t="inlineStr"/>
-      <c r="S88" t="inlineStr"/>
       <c r="T88" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -18407,7 +18066,7 @@
       </c>
       <c r="AR88" t="inlineStr">
         <is>
-          <t>gorge, hiking, nature, scenic_views, mountains, outdoor</t>
+          <t>hiking, nature_trail, scenic_view, mountains, outdoor, nature_landscape</t>
         </is>
       </c>
       <c r="AS88" t="inlineStr">
@@ -18417,13 +18076,11 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr"/>
       <c r="B89" t="inlineStr">
         <is>
           <t>Bachledka Ski &amp; Sun</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
           <t>Nowoczesny ośrodek narciarski i całoroczny kompleks rekreacyjny u podnóża Tatr.</t>
@@ -18439,7 +18096,6 @@
           <t>To idealne miejsce na aktywny wypoczynek zarówno zimą, jak i latem. Oprócz sportów zimowych można tu spacerować w koronach drzew, podziwiać panoramę Tatr oraz korzystać z uroków lokalnej kuchni.</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
           <t>{
@@ -18488,8 +18144,6 @@
       <c r="Q89" t="n">
         <v>20.3099199</v>
       </c>
-      <c r="R89" t="inlineStr"/>
-      <c r="S89" t="inlineStr"/>
       <c r="T89" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -18600,7 +18254,7 @@
       </c>
       <c r="AR89" t="inlineStr">
         <is>
-          <t>viewpoint, cable_car, mountains, family_friendly, outdoor, scenic_views</t>
+          <t>cable_car, scenic_view, mountains, viewpoint, family_friendly, outdoor</t>
         </is>
       </c>
       <c r="AS89" t="inlineStr">
@@ -18610,13 +18264,11 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr"/>
       <c r="B90" t="inlineStr">
         <is>
           <t>Jaskinia Bielańska</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
           <t>Jedna z najpiękniejszych jaskiń Słowacji, znana z bogatej szaty naciekowej i podziemnych jezior.</t>
@@ -18632,7 +18284,6 @@
           <t>Odwiedź, by zobaczyć wyjątkowe formacje skalne i piękno podziemnego świata Tatr, a także poczuć niezwykły mikroklimat jaskini.</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>{
@@ -18681,8 +18332,6 @@
       <c r="Q90" t="n">
         <v>20.3113339</v>
       </c>
-      <c r="R90" t="inlineStr"/>
-      <c r="S90" t="inlineStr"/>
       <c r="T90" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -18793,7 +18442,7 @@
       </c>
       <c r="AR90" t="inlineStr">
         <is>
-          <t>cave, underground, geology, nature, sightseeing, family_friendly</t>
+          <t>history_mystery, underground_tour, cave, geology, educational_route, sightseeing, family_friendly</t>
         </is>
       </c>
       <c r="AS90" t="inlineStr">
@@ -18803,13 +18452,11 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr"/>
       <c r="B91" t="inlineStr">
         <is>
           <t>Kolej Linowa na Palenicę</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
           <t>Kolej linowa prowadząca na szczyt Palenicy w Szczawnicy.</t>
@@ -18825,7 +18472,6 @@
           <t>To świetny sposób, aby w prosty sposób dostać się na szczyt Palenicy, skąd roztacza się panorama Pienin i okolic Szczawnicy. Atrakcja jest wygodna dla rodzin z dziećmi i osób mniej sprawnych.</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
           <t>{
@@ -18874,8 +18520,6 @@
       <c r="Q91" t="n">
         <v>20.480353</v>
       </c>
-      <c r="R91" t="inlineStr"/>
-      <c r="S91" t="inlineStr"/>
       <c r="T91" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -18986,7 +18630,7 @@
       </c>
       <c r="AR91" t="inlineStr">
         <is>
-          <t>cable_car, viewpoint, mountains, scenic_views, family_friendly</t>
+          <t>cable_car, scenic_view, mountains, viewpoint, family_friendly, outdoor</t>
         </is>
       </c>
       <c r="AS91" t="inlineStr">
@@ -18996,13 +18640,11 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr"/>
       <c r="B92" t="inlineStr">
         <is>
           <t>Promenada nad Grajcarkiem</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
           <t>Malownicza promenada spacerowa wzdłuż rzeki Grajcarek w Szczawnicy.</t>
@@ -19018,7 +18660,6 @@
           <t>Warto się tu wybrać, aby podziwiać piękne widoki na Pieniny, zrelaksować się nad rzeką lub skorzystać z licznych ścieżek pieszych i rowerowych. To idealne miejsce na spokojny spacer lub rodzinny wypad na świeżym powietrzu.</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>{
@@ -19067,8 +18708,6 @@
       <c r="Q92" t="n">
         <v>20.4744818</v>
       </c>
-      <c r="R92" t="inlineStr"/>
-      <c r="S92" t="inlineStr"/>
       <c r="T92" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -19179,7 +18818,7 @@
       </c>
       <c r="AR92" t="inlineStr">
         <is>
-          <t>walking, riverside, relaxation, scenic_views, family_friendly</t>
+          <t>walking, scenic_view, relaxation, riverside, family_friendly</t>
         </is>
       </c>
       <c r="AS92" t="inlineStr">
@@ -19189,13 +18828,11 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr"/>
       <c r="B93" t="inlineStr">
         <is>
           <t>Plac Dietla</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
           <t>Historyczny plac będący centralnym punktem Szczawnicy.</t>
@@ -19211,7 +18848,6 @@
           <t>Odwiedź Plac Dietla, by poczuć klimat uzdrowiskowej Szczawnicy, podziwiać zabytkową architekturę i odpocząć wśród malowniczych scenerii. To idealne miejsce na spacer i relaks.</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>{
@@ -19260,8 +18896,6 @@
       <c r="Q93" t="n">
         <v>20.4877223</v>
       </c>
-      <c r="R93" t="inlineStr"/>
-      <c r="S93" t="inlineStr"/>
       <c r="T93" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -19303,7 +18937,6 @@
           <t>couples, seniors, solo</t>
         </is>
       </c>
-      <c r="AC93" t="inlineStr"/>
       <c r="AD93" t="inlineStr">
         <is>
           <t>relaxation</t>
@@ -19368,7 +19001,7 @@
       </c>
       <c r="AR93" t="inlineStr">
         <is>
-          <t>historic_center, architecture, spa_town, relaxation, sightseeing</t>
+          <t>history_mystery, historic_market_square, architecture_heritage, regional_heritage, relaxation, sightseeing</t>
         </is>
       </c>
       <c r="AS93" t="inlineStr">
@@ -19378,13 +19011,11 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr"/>
       <c r="B94" t="inlineStr">
         <is>
           <t>Zapora w Niedzicy</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
           <t>Potężna zapora wodna regulująca poziom wód Zbiornika Czorsztyńskiego.</t>
@@ -19400,7 +19031,6 @@
           <t>Warto odwiedzić zaporę, aby zobaczyć imponującą infrastrukturę hydrotechniczną, podziwiać malownicze krajobrazy i poznać znaczenie tego miejsca dla bezpieczeństwa regionu. To też świetne miejsce do spacerów i fotografii.</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>{
@@ -19449,8 +19079,6 @@
       <c r="Q94" t="n">
         <v>20.3209667</v>
       </c>
-      <c r="R94" t="inlineStr"/>
-      <c r="S94" t="inlineStr"/>
       <c r="T94" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -19561,7 +19189,7 @@
       </c>
       <c r="AR94" t="inlineStr">
         <is>
-          <t>dam, engineering, lake, scenic_views, sightseeing, history</t>
+          <t>history_mystery, local_history, industrial_heritage, scenic_view, sightseeing, engineering</t>
         </is>
       </c>
       <c r="AS94" t="inlineStr">

</xml_diff>

<commit_message>
﻿FIX #183-#185: jeden kierunek/dzien, adventure vs prefs, baza atrakcje5
- FIX #183: day_geo_region — hard block mieszania Pienin i Tatr Slowackich w jednym dniu
- FIX #184: culture-led adventure — kary za Morskie Oko/szlaki, boost history/underground
- FIX #185: FIX #160 retry przy >90min free_time (bylo 120)
- Sync zakopane.xlsx z Planer - miasta atrakcje5 (+2 jaskinie Koscielisko, tagi Zone C)

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/zakopane.xlsx
+++ b/data/zakopane.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -57,13 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS94"/>
+  <dimension ref="A1:AS96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -660,6 +660,7 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>Muzeum Oscypka Zakopane</t>
@@ -685,6 +686,7 @@
           <t>To niepowtarzalna okazja, by zanurzyć się w góralskich tradycjach, zobaczyć na żywo wyrób oscypka oraz spróbować tego regionalnego przysmaku.</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>[
@@ -878,6 +880,7 @@
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>Tatrzańskie Mini Zoo</t>
@@ -903,6 +906,7 @@
           <t>To doskonałe miejsce dla rodzin, które chcą spędzić czas w otoczeniu zwierząt, dowiedzieć się więcej o podhalańskiej faunie oraz zapewnić dzieciom bezpośredni kontakt ze zwierzętami.</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>[
@@ -1085,6 +1089,7 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>Myszogród</t>
@@ -1110,6 +1115,7 @@
           <t>Wizytę w Myszogrodzie warto odbyć, aby zobaczyć niezwykłą prezentację żywych zwierząt w starannie przygotowanym, bajkowym otoczeniu, idealnym na rodzinny wypad lub niecodzienną atrakcję podczas pobytu w Zakopanem.</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>[
@@ -1291,6 +1297,7 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Iluzja Park</t>
@@ -1316,6 +1323,7 @@
           <t>To doskonałe miejsce na spędzenie czasu z rodziną, poznanie fascynującego świata iluzji i wykonanie wyjątkowych zdjęć. Park pozwala połączyć naukę z zabawą i daje okazję do wspólnej integracji.</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>[
@@ -1498,6 +1506,7 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>Papugarnia Egzotyczne Zakopane</t>
@@ -1523,6 +1532,7 @@
           <t>To wyjątkowa okazja, by obcować bezpośrednio z egzotycznymi ptakami, nie wyjeżdżając poza Zakopane. Papugarnia świetnie sprawdza się zarówno przy każdej pogodzie, będąc miejscem atrakcyjnym dla dzieci i dorosłych.</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>[
@@ -1704,6 +1714,7 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>Podwodny Świat</t>
@@ -1729,6 +1740,7 @@
           <t>Warto odwiedzić to akwarium, aby dowiedzieć się więcej o życiu pod wodą, poznać rodzime gatunki ryb oraz spędzić czas w ciekawy sposób niezależnie od pogody.</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>[
@@ -1910,6 +1922,7 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>Zjazd pontonem ze skoczni narciarskiej Wielka Krokiew</t>
@@ -1935,6 +1948,7 @@
           <t>To jedna z nielicznych okazji, by poczuć adrenalinę zjazdu ze skoczni, którą na co dzień wykorzystują najlepsi skoczkowie narciarscy w kraju. Idealny wybór dla osób szukających aktywnych rozrywek poza standardowym zwiedzaniem.</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>[
@@ -2038,7 +2052,7 @@
           <t>friends, family_kids</t>
         </is>
       </c>
-      <c r="AC8" s="3" t="n">
+      <c r="AC8" s="2" t="n">
         <v>45944</v>
       </c>
       <c r="AD8" t="inlineStr">
@@ -2116,6 +2130,7 @@
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>Góralski Ślizg</t>
@@ -2141,6 +2156,7 @@
           <t>To świetna forma aktywności na świeżym powietrzu, idealna na spędzenie czasu z rodziną lub znajomymi, szczególnie po dniu górskich wędrówek. Atrakcja ta pozwala na poczucie adrenaliny i radości niezależnie od wieku.</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>[
@@ -2325,6 +2341,7 @@
       </c>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>Tatra Family</t>
@@ -2350,6 +2367,7 @@
           <t>Wizyta w Tatra Family to świetna okazja do aktywnego spędzenia czasu z rodziną i zapewnienia dzieciom niezapomnianej zabawy w bezpiecznym otoczeniu.</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>[
@@ -2531,6 +2549,7 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>Park Harnasia</t>
@@ -2556,6 +2575,7 @@
           <t>Warto odwiedzić Park Harnasia, by odpocząć zrelaksować się i pozwolić dzieciom pobawić się na placu zabaw. To świetny punkt na chwilę wytchnienia podczas zwiedzania Zakopanego.</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>[
@@ -2736,11 +2756,13 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>DINO PARK</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>Park tematyczny z modelami dinozaurów w naturalnych rozmiarach.</t>
@@ -2756,6 +2778,7 @@
           <t>To idealna atrakcja dla rodzin z dziećmi oraz wszystkich miłośników paleontologii i dinozaurów. Pozwala na edukację poprzez zabawę i kontakt z naturą.</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>[
@@ -2937,6 +2960,7 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>Illusion House</t>
@@ -2962,6 +2986,7 @@
           <t>Wizyta w Domu Iluzji to nie tylko świetna zabawa, ale też możliwość poznania tajników działania naszego mózgu i zmysłów. To idealne miejsce na rodzinny wypad lub rozrywkę podczas brzydszej pogody w Zakopanem.</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>[
@@ -3142,6 +3167,7 @@
       </c>
     </row>
     <row r="14">
+      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>Dom do góry nogami</t>
@@ -3167,6 +3193,7 @@
           <t>To idealne miejsce na nietypową rozrywkę i sesję zdjęciową – zaskakuje i bawi zarówno najmłodszych, jak i starszych turystów.</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>[
@@ -3347,11 +3374,13 @@
       </c>
     </row>
     <row r="15">
+      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>Plac zabaw na Górnej Równi Krupowej</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>Nowoczesny plac zabaw położony na rozległej Górnej Równi Krupowej w Zakopanem.</t>
@@ -3367,6 +3396,7 @@
           <t>To idealne miejsce na odpoczynek i zabawę dla dzieci po zwiedzaniu Zakopanego. Malownicze położenie oraz czyste, przestronne otoczenie sprzyjają relaksowi i rekreacji całych rodzin.</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>[
@@ -3547,6 +3577,7 @@
       </c>
     </row>
     <row r="16">
+      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>Termy Zakopiańskie</t>
@@ -3572,6 +3603,7 @@
           <t>Wizyta w Termach Zakopiańskich to okazja do zabawy i relaksu w wodzie, niezależnie od warunków pogodowych. Można tu korzystać z wielu atrakcji basenowych i wellness oraz zjeść smaczny posiłek.</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>[
@@ -3753,6 +3785,7 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>Termy Gorący Potok</t>
@@ -3778,6 +3811,7 @@
           <t>Wizyta pozwala zrelaksować się w ciepłych wodach termalnych, korzystać z leczniczych i relaksacyjnych właściwości wód oraz atrakcji dostępnych na terenie kompleksu.</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>[
@@ -3959,6 +3993,7 @@
       </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>Chochołowskie Termy</t>
@@ -3984,6 +4019,7 @@
           <t>To doskonałe miejsce na relaks i rekreację przez cały rok, z licznymi udogodnieniami dla rodzin, par i miłośników sportu. Naturalna woda termalna wpływa korzystnie na zdrowie i samopoczucie, a bogata strefa spa i saun zapewnia głęboki relaks.</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>[
@@ -4165,6 +4201,7 @@
       </c>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>Terma Bania</t>
@@ -4190,6 +4227,7 @@
           <t>To idealne miejsce na relaks w wodach termalnych z pięknym widokiem na góry, a także rozrywkę dla całej rodziny.</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>[
@@ -4370,6 +4408,7 @@
       </c>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>Termy Bukovina</t>
@@ -4395,6 +4434,7 @@
           <t>To idealne miejsce na relaks, odprężenie po górskich wędrówkach i zabawę z rodziną lub przyjaciółmi w wodzie termalnej.</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>[
@@ -4576,6 +4616,7 @@
       </c>
     </row>
     <row r="21">
+      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t>Wielka Krokiew</t>
@@ -4601,6 +4642,7 @@
           <t>To miejsce kultowe dla miłośników sportów i niepowtarzalny punkt widokowy na Tatry oraz Zakopane. Wizyta na Wielkiej Krokwi pozwala poczuć sportową atmosferę i zobaczyć na własne oczy miejsce legendarnych zawodów.</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>[
@@ -4781,6 +4823,7 @@
       </c>
     </row>
     <row r="22">
+      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t>Centrum Edukacji Przyrodniczej Tatrzańskiego Parku Narodowego</t>
@@ -4806,6 +4849,7 @@
           <t>To miejsce pozwala pogłębić wiedzę o Tatrach w atrakcyjny i angażujący sposób. Idealne zarówno dla rodzin z dziećmi, jak i pasjonatów przyrody.</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>[
@@ -4986,11 +5030,13 @@
       </c>
     </row>
     <row r="23">
+      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
           <t>Wystawa Figur Woskowych EXPO Krupówki</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>Wystawa prezentująca realistyczne figury woskowe znanych postaci.</t>
@@ -5006,6 +5052,7 @@
           <t>Warto odwiedzić, aby zobaczyć imponująco wykonane figury woskowe znanych postaci, a także zrobić oryginalne pamiątkowe zdjęcia. To doskonały sposób na urozmaicenie pobytu na Krupówkach i rozrywkę niezależnie od pogody.</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>[
@@ -5186,11 +5233,13 @@
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
           <t>Wielka Wystawa Klocków LEGO</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>Imponująca wystawa prezentująca największe modele wykonane z klocków LEGO.</t>
@@ -5206,6 +5255,7 @@
           <t>To jedna z największych wystaw LEGO w Polsce, idealna dla rodzin i miłośników LEGO w każdym wieku. Pozwala zobaczyć niesamowite konstrukcje oraz inspirować się do własnych projektów.</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>[
@@ -5386,11 +5436,13 @@
       </c>
     </row>
     <row r="25">
+      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
           <t>Muzeum Tatrzańskie</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>Muzeum prezentujące historię, kulturę i przyrodę Tatr oraz Podhala.</t>
@@ -5406,6 +5458,7 @@
           <t>To idealne miejsce, aby lepiej poznać historię Zakopanego, kulturę góralską oraz bogactwo tatrzańskiej przyrody. Muzeum stanowi doskonały punkt startowy do dalszego odkrywania Tatr i regionu Podhala.</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>[
@@ -5508,7 +5561,7 @@
           <t>solo, couples, friends, seniors</t>
         </is>
       </c>
-      <c r="AC25" s="3" t="n">
+      <c r="AC25" s="2" t="n">
         <v>45944</v>
       </c>
       <c r="AD25" t="inlineStr">
@@ -5585,11 +5638,13 @@
       </c>
     </row>
     <row r="26">
+      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
           <t>Muzeum Kornela Makuszyńskiego</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>Oddział Muzeum Tatrzańskiego poświęcony życiu i twórczości Kornela Makuszyńskiego.</t>
@@ -5605,6 +5660,7 @@
           <t>Muzeum to gratka dla miłośników literatury polskiej, szczególnie książek dla dzieci. Pozwala bliżej poznać niezwykłą postać Kornela Makuszyńskiego oraz poczuć atmosferę Zakopanego z początku XX wieku.</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>[
@@ -5707,7 +5763,7 @@
           <t>solo, couples, friends, family_kids, seniors</t>
         </is>
       </c>
-      <c r="AC26" s="3" t="n">
+      <c r="AC26" s="2" t="n">
         <v>45944</v>
       </c>
       <c r="AD26" t="inlineStr">
@@ -5784,11 +5840,13 @@
       </c>
     </row>
     <row r="27">
+      <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
           <t>Muzeum Stylu Zakopiańskiego im. S. Witkiewicza</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>Muzeum prezentujące historię i charakterystyczny styl zakopiański w architekturze i sztuce.</t>
@@ -5804,6 +5862,7 @@
           <t>To unikatowa okazja do zgłębienia dziedzictwa kulturowego regionu, zobaczenia oryginalnych projektów Stanisława Witkiewicza i lepszego zrozumienia charakterystycznej architektury Podhala.</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>[
@@ -5906,7 +5965,7 @@
           <t>solo, couples, friends, family_kids, seniors</t>
         </is>
       </c>
-      <c r="AC27" s="3" t="n">
+      <c r="AC27" s="2" t="n">
         <v>45944</v>
       </c>
       <c r="AD27" t="inlineStr">
@@ -5983,11 +6042,13 @@
       </c>
     </row>
     <row r="28">
+      <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
           <t>Galeria sztuki w willi Oksza</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>Galeria prezentująca zbiory sztuki w zabytkowej willi Oksza, będąca filią Muzeum Tatrzańskiego.</t>
@@ -6003,6 +6064,7 @@
           <t>To wyjątkowe miejsce, gdzie można podziwiać sztukę i architekturę regionu oraz dowiedzieć się więcej o artystycznej historii Zakopanego i Tatr.</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>[
@@ -6105,7 +6167,7 @@
           <t>solo, couples, friends, family_kids, seniors</t>
         </is>
       </c>
-      <c r="AC28" s="3" t="n">
+      <c r="AC28" s="2" t="n">
         <v>45944</v>
       </c>
       <c r="AD28" t="inlineStr">
@@ -6182,11 +6244,13 @@
       </c>
     </row>
     <row r="29">
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
           <t>Muzeum Karola Szymanowskiego w willi "Atma"</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>Historyczna willa w stylu zakopiańskim, w której znajduje się muzeum poświęcone Karolowi Szymanowskiemu.</t>
@@ -6202,6 +6266,7 @@
           <t>To idealne miejsce dla miłośników muzyki, sztuki i historii Zakopanego, a także dla osób zainteresowanych życiem i twórczością Karola Szymanowskiego.</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>[
@@ -6303,7 +6368,7 @@
           <t>solo, couples, friends, family_kids, seniors</t>
         </is>
       </c>
-      <c r="AC29" s="3" t="n">
+      <c r="AC29" s="2" t="n">
         <v>45944</v>
       </c>
       <c r="AD29" t="inlineStr">
@@ -6380,11 +6445,13 @@
       </c>
     </row>
     <row r="30">
+      <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
           <t>Tatrzański Park Edukacyjny</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>Edukacyjny park zoologiczny, który przybliża przyrodę Tatr i kulturę góralską.</t>
@@ -6400,6 +6467,7 @@
           <t>To doskonałe miejsce do rodzinnego wypoczynku, poznawania zwierząt żyjących w Tatrach oraz ciekawostek o folklorze i przyrodzie regionu.</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>[
@@ -6582,11 +6650,13 @@
       </c>
     </row>
     <row r="31">
+      <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
           <t>Kaplica Najświętszego Serca Pana Jezusa w Jaszczurówce</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>Drewniana kaplica w stylu zakopiańskim, będąca jednym z najpiękniejszych przykładów architektury sakralnej regionu.</t>
@@ -6602,6 +6672,7 @@
           <t>To obowiązkowe miejsce dla miłośników stylu zakopiańskiego oraz osób chcących poznać kulturę i tradycje regionu podhalańskiego.</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>[
@@ -6782,11 +6853,13 @@
       </c>
     </row>
     <row r="32">
+      <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
           <t>KULIGI w Zakopanem</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>Organizator tradycyjnych kuligów z saniami i pochodniami po zakopiańskich okolicach.</t>
@@ -6802,6 +6875,7 @@
           <t>To niepowtarzalna okazja, by przeżyć autentyczny, zimowy kulig i poznać lokalne tradycje w wyjątkowej atmosferze zakopiańskiej zimy.</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>[
@@ -6993,11 +7067,13 @@
       </c>
     </row>
     <row r="33">
+      <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
           <t>Dolina Chochołowska</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>Najdłuższa i jedna z najpiękniejszych dolin w polskich Tatrach, popularna zarówno wśród turystów pieszych, jak i rowerzystów.</t>
@@ -7013,6 +7089,7 @@
           <t>To miejsce obowiązkowe dla miłośników przyrody, fotografów i osób szukających spokojnych wędrówek z dala od tłumów popularnych szlaków. Dolina Chochołowska oferuje niepowtarzalne widoki o każdej porze roku.</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>[
@@ -7084,6 +7161,8 @@
       <c r="Q33" t="n">
         <v>19.8333333</v>
       </c>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -7204,11 +7283,13 @@
       </c>
     </row>
     <row r="34">
+      <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
           <t>Dolina Kościeliska</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>Jedna z najpiękniejszych tatrzańskich dolin, słynąca z malowniczych krajobrazów, jaskiń i górskich szlaków.</t>
@@ -7224,6 +7305,7 @@
           <t>To jedno z must-see Tatr – niesamowite widoki, łatwy dostęp i ciekawe formacje skalne sprawiają, że wizyta w Dolinie Kościeliskiej dostarcza niezapomnianych wrażeń każdemu, bez względu na wiek czy doświadczenie górskie.</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>[
@@ -7296,6 +7378,8 @@
       <c r="Q34" t="n">
         <v>19.8666667</v>
       </c>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -7416,11 +7500,13 @@
       </c>
     </row>
     <row r="35">
+      <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
           <t>Rusinowa Polana</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>Malownicza polana w Tatrach, oferująca piękne widoki na okoliczne szczyty.</t>
@@ -7436,6 +7522,7 @@
           <t>Warto odwiedzić Rusinową Polanę dla spektakularnych panoram Tatr, unikalnego klimatu regionu i tradycyjnego pasterstwa.</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>[
@@ -7508,6 +7595,8 @@
       <c r="Q35" t="n">
         <v>20.0895038</v>
       </c>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -7628,11 +7717,13 @@
       </c>
     </row>
     <row r="36">
+      <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr">
         <is>
           <t>Morskie Oko</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>Największe i jedno z najpiękniejszych jezior w Tatrach, otoczone spektakularnymi szczytami górskimi.</t>
@@ -7648,6 +7739,7 @@
           <t>Morskie Oko zachwyca spektakularnymi krajobrazami i doskonałymi możliwościami do fotografii. Szlak do jeziora to popularna górska trasa, idealna dla osób szukających kontaktu z przyrodą i pięknymi widokami.</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>[
@@ -7720,6 +7812,8 @@
       <c r="Q36" t="n">
         <v>20.070087</v>
       </c>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -7840,11 +7934,13 @@
       </c>
     </row>
     <row r="37">
+      <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
           <t>Gubałówka</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
           <t>Gubałówka to jedna z największych atrakcji Zakopanegp. Na górze czekają piękne widoki na Tatry z Giewontem.</t>
@@ -7860,6 +7956,7 @@
           <t>Znajdziesz tu jedne najpiękniejszych widoków na Tatry i panoramę Zakopanego. Na górze czekają rodzinne atrakcje, regionalne przysmaki i wyjątkowy, góralski klimat.</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>{
@@ -7908,6 +8005,8 @@
       <c r="Q37" t="n">
         <v>19.9454830120256</v>
       </c>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -8028,11 +8127,13 @@
       </c>
     </row>
     <row r="38">
+      <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
           <t>Snowdoo Adventure</t>
         </is>
       </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
           <t>Ośrodek oferujący wyprawy skuterami śnieżnymi i atrakcje zimowe.</t>
@@ -8048,6 +8149,7 @@
           <t>To wyjątkowa propozycja dla miłośników adrenaliny i aktywnego spędzania czasu na świeżym powietrzu w otoczeniu tatrzańskich krajobrazów.</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t xml:space="preserve">{
@@ -8097,6 +8199,8 @@
       <c r="Q38" t="n">
         <v>19.9128467</v>
       </c>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -8217,11 +8321,13 @@
       </c>
     </row>
     <row r="39">
+      <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
           <t xml:space="preserve">Kolejka linowa na Kasprowy Wierch </t>
         </is>
       </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>Kolejka linowa prowadzącej na szczyt Kasprowego Wierchu.</t>
@@ -8237,6 +8343,7 @@
           <t>To idealne miejsce, by rozpocząć podróż na jeden z najpopularniejszych szczytów Tatr, zarówno zimą, jak i latem. Wjazd kolejką pozwala podziwiać wyjątkowe widoki i uniknąć mozolnej wędrówki na szczyt.</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>{
@@ -8459,11 +8566,13 @@
       </c>
     </row>
     <row r="40">
+      <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
           <t>Droga pod Reglami</t>
         </is>
       </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
           <t>Malowniczy szlak pieszy biegnący wzdłuż północnych zboczy Tatr, idealny na spacer i podziwianie przyrody.</t>
@@ -8479,6 +8588,7 @@
           <t>Idealna propozycja dla osób szukających łatwej trasy w Tatrach, z pięknymi widokami i możliwością odpoczynku z dala od tłumu. Droga pod Reglami pozwala odkrywać uroki tatrzańskich dolin bez konieczności intensywnego wspinania.</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>{
@@ -8538,6 +8648,8 @@
       <c r="Q40" t="n">
         <v>19.9813526</v>
       </c>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -8658,11 +8770,13 @@
       </c>
     </row>
     <row r="41">
+      <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
           <t>Dolina Strążyska</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>Malownicza dolina tatrzańska prowadząca u stóp Giewontu, popularna wśród turystów pieszych.</t>
@@ -8678,6 +8792,7 @@
           <t>To jedno z najładniejszych i najłatwiejszych do przejścia miejsc w Tatrach, idealne zarówno dla rodzin z dziećmi, jak i osób ceniących spokojną przyrodę, a także fotografów krajobrazowych.</t>
         </is>
       </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>{
@@ -8737,6 +8852,8 @@
       <c r="Q41" t="n">
         <v>19.9333087</v>
       </c>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -8857,11 +8974,13 @@
       </c>
     </row>
     <row r="42">
+      <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
           <t>Dolina ku Dziurze</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>Mała, malownicza dolina tatrzańska znana z naturalnej jaskini Dziura.</t>
@@ -8877,6 +8996,7 @@
           <t>To łatwo dostępna dolinka, oferująca piękne widoki i unikalną jaskinię. Jest idealna na krótki wypad, szczególnie dla osób, które chcą szybko poczuć klimat Tatr bez długich, męczących wędrówek.</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>{
@@ -8936,6 +9056,8 @@
       <c r="Q42" t="n">
         <v>19.9411407</v>
       </c>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -9056,11 +9178,13 @@
       </c>
     </row>
     <row r="43">
+      <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
           <t>Polana Kalatówki</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>Malownicza polana położona w Tatrach, otoczona lasami i górami, popularna wśród turystów oraz miłośników wypoczynku na łonie natury.</t>
@@ -9076,6 +9200,7 @@
           <t>Warto odwiedzić to miejsce ze względu na wspaniałe widoki, atmosferę spokoju i możliwość łatwego kontaktu z tatrzańską przyrodą. Polana Kalatówki to jedno z najbardziej dostępnych i malowniczych miejsc w okolicach Zakopanego.</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>{
@@ -9135,6 +9260,8 @@
       <c r="Q43" t="n">
         <v>19.9683412</v>
       </c>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -9255,11 +9382,13 @@
       </c>
     </row>
     <row r="44">
+      <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
           <t>Punkt widokowy na Tatry</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>Punkt widokowy oferujący panoramę Tatr.</t>
@@ -9275,6 +9404,7 @@
           <t>To doskonałe miejsce, by zobaczyć piękno Tatr z innej perspektywy oraz zrobić wyjątkowe zdjęcia krajobrazowe.</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>{
@@ -9334,6 +9464,8 @@
       <c r="Q44" t="n">
         <v>20.0107764</v>
       </c>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -9454,11 +9586,13 @@
       </c>
     </row>
     <row r="45">
+      <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
           <t>Wodospad Siklawica</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>Malowniczy wodospad położony u podnóża Giewontu w Tatrach Zachodnich.</t>
@@ -9474,6 +9608,7 @@
           <t>To jedno z piękniejszych naturalnych miejsc w okolicy Zakopanego, idealne na krótki spacer z zachwycającymi widokami i możliwością kontaktu z naturą.</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>{
@@ -9533,6 +9668,8 @@
       <c r="Q45" t="n">
         <v>19.9302071</v>
       </c>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -9653,11 +9790,13 @@
       </c>
     </row>
     <row r="46">
+      <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr">
         <is>
           <t>Olczyska Polana</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
           <t>Malownicza polana położona na terenie Tatrzańskiego Parku Narodowego, idealna do pieszych wycieczek i wypoczynku na łonie natury.</t>
@@ -9673,6 +9812,7 @@
           <t>To świetne miejsce, aby odpocząć od tłoku Zakopanego i podziwiać naturalne piękno Tatr. Spacer na Olczyską Polanę to łagodna i dostępna trasa nawet dla rodzin z dziećmi.</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>{
@@ -9732,6 +9872,8 @@
       <c r="Q46" t="n">
         <v>20.0005687</v>
       </c>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -9852,11 +9994,13 @@
       </c>
     </row>
     <row r="47">
+      <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
           <t>Polana Jaworzynka</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>Malownicza polana w Tatrach, popularna wśród spacerowiczów i miłośników przyrody.</t>
@@ -9872,6 +10016,7 @@
           <t>Warto odwiedzić Polanę Jaworzynka, by wypocząć na łonie natury, podziwiać malownicze panoramy oraz poczuć niepowtarzalny klimat tatrzańskiej doliny.</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>{
@@ -9931,6 +10076,8 @@
       <c r="Q47" t="n">
         <v>19.9846641</v>
       </c>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -10051,11 +10198,13 @@
       </c>
     </row>
     <row r="48">
+      <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr">
         <is>
           <t>Sarni Wodospad</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
           <t>Malowniczy, niewielki wodospad położony na obrzeżach Zakopanego, wśród tatrzańskiej przyrody.</t>
@@ -10071,6 +10220,7 @@
           <t>To doskonałe miejsce, aby zrelaksować się w otoczeniu przyrody, z dala od tłumów i miejskiego zgiełku. Idealny punkt na krótki postój podczas wycieczek poza centrum Zakopanego.</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>{
@@ -10130,6 +10280,8 @@
       <c r="Q48" t="n">
         <v>19.9544844</v>
       </c>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -10250,11 +10402,13 @@
       </c>
     </row>
     <row r="49">
+      <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
           <t>Wielka Polana Małołącka</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
           <t>Szeroka polana górska położona w Dolinie Małej Łąki, otoczona malowniczymi szczytami Tatr Zachodnich.</t>
@@ -10270,6 +10424,7 @@
           <t>To idealne miejsce na relaks wśród natury, podziwianie tatrzańskich krajobrazów i piknik w górskim otoczeniu. Polana zachwyca ciszą i przestrzenią, a jednocześnie jest łatwo dostępna nawet dla osób mniej doświadczonych w górach.</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>{
@@ -10329,6 +10484,8 @@
       <c r="Q49" t="n">
         <v>19.9043787</v>
       </c>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -10449,11 +10606,13 @@
       </c>
     </row>
     <row r="50">
+      <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr">
         <is>
           <t>Dolina Za Bramką</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
           <t>Malownicza dolina tatrzańska idealna na spokojne spacery.</t>
@@ -10469,6 +10628,7 @@
           <t>Warto odwiedzić tę dolinę, by odpocząć od tłumów, podziwiać dziewiczą przyrodę i zrelaksować się na łonie Tatr.</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>{
@@ -10528,6 +10688,8 @@
       <c r="Q50" t="n">
         <v>19.9171668</v>
       </c>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -10648,11 +10810,13 @@
       </c>
     </row>
     <row r="51">
+      <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr">
         <is>
           <t>Dolina Suchej Wody</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>Malownicza dolina tatrzańska znajdująca się w rejonie Zakopanego.</t>
@@ -10668,6 +10832,7 @@
           <t>Jest to idealne miejsce na rozpoczęcie wędrówki w wyższe partie Tatr i podziwianie wyjątkowych widoków oraz alpejskiej przyrody.</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>{
@@ -10727,6 +10892,8 @@
       <c r="Q51" t="n">
         <v>20.0359096</v>
       </c>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -10847,11 +11014,13 @@
       </c>
     </row>
     <row r="52">
+      <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr">
         <is>
           <t>Dolina Gąsienicowa</t>
         </is>
       </c>
+      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
           <t>Malownicza dolina tatrzańska, popularna wśród turystów i miłośników górskich wędrówek.</t>
@@ -10867,6 +11036,7 @@
           <t>To miejsce obowiązkowe dla każdego miłośnika Tatr – urzeka nie tylko widokami, lecz również bogactwem górskiej przyrody i atmosferą schroniska. Stanowi początek wielu fascynujących tras trekkingowych.</t>
         </is>
       </c>
+      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
           <t>{
@@ -10926,6 +11096,8 @@
       <c r="Q52" t="n">
         <v>20.0063853</v>
       </c>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -11046,11 +11218,13 @@
       </c>
     </row>
     <row r="53">
+      <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr">
         <is>
           <t>Park Miejski im. Marszałka Józefa Piłsudskiego</t>
         </is>
       </c>
+      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
           <t>Zielona oaza w centrum Zakopanego z alejkami spacerowymi, placem zabaw i miejscami do odpoczynku.</t>
@@ -11066,6 +11240,7 @@
           <t>Warto odwiedzić park, aby odpocząć od zgiełku Zakopanego, nacieszyć się przyrodą i skorzystać z licznych atrakcji na świeżym powietrzu.</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>{
@@ -11125,6 +11300,8 @@
       <c r="Q53" t="n">
         <v>19.95507</v>
       </c>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -11245,11 +11422,13 @@
       </c>
     </row>
     <row r="54">
+      <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr">
         <is>
           <t>Chałupa Sabały</t>
         </is>
       </c>
+      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
           <t>Zabytkowa, drewniana chałupa rodem z XIX wieku, będąca dawnym domem góralskiego muzyka Jana Krzeptowskiego Sabały.</t>
@@ -11265,6 +11444,7 @@
           <t>Warto odwiedzić to miejsce, aby poczuć ducha dawnego Zakopanego, zobaczyć tradycyjną góralską izbę oraz poznać historię jednej z najbardziej barwnych postaci Tatr. Chałupa pozwala lepiej zrozumieć historię i kulturę regionu podhalańskiego.</t>
         </is>
       </c>
+      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>{
@@ -11313,6 +11493,8 @@
       <c r="Q54" t="n">
         <v>19.9193173</v>
       </c>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
       <c r="T54" t="inlineStr">
         <is>
           <t>mixed</t>
@@ -11433,11 +11615,13 @@
       </c>
     </row>
     <row r="55">
+      <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr">
         <is>
           <t>Quady Adventure Zakopane Wypożyczalnia</t>
         </is>
       </c>
+      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
           <t>Wypożyczalnia quadów i buggy oferująca wycieczki terenowe w okolicach Poronina.</t>
@@ -11453,6 +11637,7 @@
           <t>To doskonały sposób na aktywne spędzenie czasu, podziwianie górskich krajobrazów i przeżycie motoryzacyjnej przygody, dostępny zarówno dla początkujących, jak i zaawansowanych.</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>{
@@ -11501,6 +11686,8 @@
       <c r="Q55" t="n">
         <v>19.9937334</v>
       </c>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
       <c r="T55" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -11621,11 +11808,13 @@
       </c>
     </row>
     <row r="56">
+      <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr">
         <is>
           <t>Cudakowa Polana</t>
         </is>
       </c>
+      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>Malownicza polana położona przy czarnym szlaku turystycznym w Tatrach.</t>
@@ -11641,6 +11830,7 @@
           <t>Warto odwiedzić Cudakową Polanę, aby nacieszyć się wspaniałymi widokami oraz doświadczyć klimatu górskiej przyrody z dala od miejskiego zgiełku.</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>{
@@ -11684,6 +11874,7 @@
       <c r="M56" t="n">
         <v>5.5</v>
       </c>
+      <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr">
         <is>
           <t>Małopolska</t>
@@ -11695,6 +11886,8 @@
       <c r="Q56" t="n">
         <v>19.8693207</v>
       </c>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -11815,11 +12008,13 @@
       </c>
     </row>
     <row r="57">
+      <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr">
         <is>
           <t xml:space="preserve"> Beernarium Piwne Spa</t>
         </is>
       </c>
+      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>Relaksacyjne spa oferujące kąpiele piwne i zabiegi wellness.</t>
@@ -11835,6 +12030,7 @@
           <t>Wizyta w Beernarium Piwnym Spa to szansa na relaks i regenerację w niepowtarzalnej, piwnej atmosferze, jakiej nie znajdziemy w typowych spa. Kąpiele w piwie mają korzystny wpływ na skórę i samopoczucie.</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>{
@@ -11883,6 +12079,8 @@
       <c r="Q57" t="n">
         <v>19.9623495</v>
       </c>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
       <c r="T57" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -12003,11 +12201,13 @@
       </c>
     </row>
     <row r="58">
+      <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr">
         <is>
           <t>Iria Spa</t>
         </is>
       </c>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
           <t>Nowoczesne spa oferujące szeroki zakres zabiegów relaksacyjnych i pielęgnacyjnych.</t>
@@ -12023,6 +12223,7 @@
           <t>To doskonałe miejsce, aby zatroszczyć się o swoje zdrowie i dobre samopoczucie, odprężyć się oraz skorzystać z wysokiej jakości zabiegów w przyjaznej atmosferze.</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>{
@@ -12201,11 +12402,13 @@
       </c>
     </row>
     <row r="59">
+      <c r="A59" t="inlineStr"/>
       <c r="B59" t="inlineStr">
         <is>
           <t>Polana Głodówka</t>
         </is>
       </c>
+      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
           <t>Malownicza polana z panoramicznym widokiem na Tatry.</t>
@@ -12221,6 +12424,7 @@
           <t>To idealne miejsce, aby podziwiać panoramę Tatr, zrobić zdjęcia oraz odpocząć na łonie przyrody, z dala od gwaru kurortów.</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>{
@@ -12280,6 +12484,8 @@
       <c r="Q59" t="n">
         <v>20.1174987</v>
       </c>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr"/>
       <c r="T59" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -12400,11 +12606,13 @@
       </c>
     </row>
     <row r="60">
+      <c r="A60" t="inlineStr"/>
       <c r="B60" t="inlineStr">
         <is>
           <t>Park Przygody Gubałówka</t>
         </is>
       </c>
+      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
           <t>Park linowy na Gubałówce oferujący trasy o różnym stopniu trudności.</t>
@@ -12420,6 +12628,7 @@
           <t>To świetna propozycja dla osób żądnych aktywności i lubiących wyzwania, a także dla rodzin z dziećmi. Ropes Gold Ridge łączy sportową zabawę ze wspaniałymi widokami na Tatry.</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>{
@@ -12468,6 +12677,7 @@
       <c r="Q60" t="n">
         <v>19.9310972</v>
       </c>
+      <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr">
         <is>
           <t>https://park-przygody-gubalowka.pl/cennik/</t>
@@ -12593,11 +12803,13 @@
       </c>
     </row>
     <row r="61">
+      <c r="A61" t="inlineStr"/>
       <c r="B61" t="inlineStr">
         <is>
           <t>Cmentarz Zasłużonych na Pęksowym Brzyzku</t>
         </is>
       </c>
+      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
           <t>Historyczny cmentarz, miejsce pochówku znanych osób zasłużonych dla regionu Tatr i Zakopanego.</t>
@@ -12613,6 +12825,7 @@
           <t>Warto odwiedzić to miejsce, aby poznać historię regionu, oddać hołd wybitnym postaciom i podziwiać unikalne nagrobki będące dziełami lokalnych rzemieślników.</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>{
@@ -12661,6 +12874,8 @@
       <c r="Q61" t="n">
         <v>19.9470409</v>
       </c>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -12781,11 +12996,13 @@
       </c>
     </row>
     <row r="62">
+      <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr">
         <is>
           <t>Dwór Tetmajerów</t>
         </is>
       </c>
+      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
           <t>Zabytkowy dwór szlachecki będący filią Muzeum Tatrzańskiego, prezentujący kulturę regionu i historię rodu Tetmajerów.</t>
@@ -12801,6 +13018,7 @@
           <t>To miejsce łączy historię, tradycję i piękno architektury regionu, pozwalając lepiej zrozumieć bogatą kulturę Podhala oraz losy słynnej rodziny Tetmajerów.</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>{
@@ -12849,6 +13067,8 @@
       <c r="Q62" t="n">
         <v>20.1277911</v>
       </c>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr">
         <is>
           <t>mixed</t>
@@ -12969,11 +13189,13 @@
       </c>
     </row>
     <row r="63">
+      <c r="A63" t="inlineStr"/>
       <c r="B63" t="inlineStr">
         <is>
           <t>Sanktuarium Wiktorówki</t>
         </is>
       </c>
+      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
           <t>Sanktuarium Matki Bożej Królowej Tatr, popularne miejsce pielgrzymkowe i turystyczne w Tatrach.</t>
@@ -12989,6 +13211,7 @@
           <t>To wyjątkowe miejsce, gdzie można połączyć kontakt z przyrodą ze spokojem i duchowym wytchnieniem. Kaplica na Wiktorówkach to nie tylko cel religijny, ale także doskonały punkt na trasie wędrówek po Tatrach.</t>
         </is>
       </c>
+      <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
           <t>{
@@ -13037,6 +13260,8 @@
       <c r="Q63" t="n">
         <v>20.086447</v>
       </c>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr"/>
       <c r="T63" t="inlineStr">
         <is>
           <t>mixed</t>
@@ -13157,11 +13382,13 @@
       </c>
     </row>
     <row r="64">
+      <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr">
         <is>
           <t>Snow Zabawa – zimowe atrakcje</t>
         </is>
       </c>
+      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
           <t>Miejsce oferujące różnorodne zimowe atrakcje i zabawy na śniegu dla całych rodzin.</t>
@@ -13177,6 +13404,7 @@
           <t>To świetna okazja, aby aktywnie spędzić czas zimą, korzystając z bogatej oferty atrakcji na świeżym powietrzu, ciesząc się pięknymi widokami Tatr oraz lokalnym klimatem.</t>
         </is>
       </c>
+      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>{
@@ -13198,6 +13426,7 @@
       <c r="J64" t="n">
         <v>180</v>
       </c>
+      <c r="K64" t="inlineStr"/>
       <c r="L64" t="n">
         <v>30</v>
       </c>
@@ -13221,6 +13450,8 @@
       <c r="Q64" t="n">
         <v>19.9045138</v>
       </c>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -13341,11 +13572,13 @@
       </c>
     </row>
     <row r="65">
+      <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr">
         <is>
           <t>Krupówki</t>
         </is>
       </c>
+      <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
           <t>Główna ulica spacerowa i handlowa w Zakopanem, pełna sklepów, restauracji oraz atrakcji kulturalnych.</t>
@@ -13361,6 +13594,7 @@
           <t>Krupówki to prawdziwe serce Zakopanego; miejsce, gdzie można poczuć góralską atmosferę, skosztować regionalnej kuchni, kupić pamiątki, a także obserwować codzienne życie mieszkańców i turystów.</t>
         </is>
       </c>
+      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
           <t>{
@@ -13543,11 +13777,13 @@
       </c>
     </row>
     <row r="66">
+      <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr">
         <is>
           <t>Dolna Rówień Krupowa</t>
         </is>
       </c>
+      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
           <t>Rozległy, zielony park w centrum Zakopanego, popularny na spacery oraz rekreację.</t>
@@ -13563,6 +13799,7 @@
           <t>To idealne miejsce na relaks po zwiedzaniu Zakopanego lub szlakach górskich. Można tu odpocząć, podziwiać panoramę gór, aktywnie spędzić czas z rodziną lub spotkać się na piknik.</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>{
@@ -13622,6 +13859,8 @@
       <c r="Q66" t="n">
         <v>19.9559261</v>
       </c>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
       <c r="T66" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -13746,11 +13985,13 @@
       </c>
     </row>
     <row r="67">
+      <c r="A67" t="inlineStr"/>
       <c r="B67" t="inlineStr">
         <is>
           <t>Muzeum Jana Kasprowicza</t>
         </is>
       </c>
+      <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
           <t>Muzeum poświęcone życiu i twórczości poety Jana Kasprowicza.</t>
@@ -13766,6 +14007,7 @@
           <t>To wyjątkowa okazja, by poznać historię życia Jana Kasprowicza – jednego z najwybitniejszych polskich poetów, a także zobaczyć wnętrza willi z początku XX wieku.</t>
         </is>
       </c>
+      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
           <t>{
@@ -13944,11 +14186,13 @@
       </c>
     </row>
     <row r="68">
+      <c r="A68" t="inlineStr"/>
       <c r="B68" t="inlineStr">
         <is>
           <t>Willa Koliba</t>
         </is>
       </c>
+      <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
           <t>Pierwszy dom w stylu zakopiańskim, mieszczący muzeum poświęcone temu unikalnemu nurtowi architektonicznemu.</t>
@@ -13964,6 +14208,7 @@
           <t>To obowiązkowe miejsce dla miłośników sztuki, architektury i historii regionu. Możesz poczuć klimat dawnego Zakopanego i odkryć źródła stylu zakopiańskiego.</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
           <t>{
@@ -14142,11 +14387,13 @@
       </c>
     </row>
     <row r="69">
+      <c r="A69" t="inlineStr"/>
       <c r="B69" t="inlineStr">
         <is>
           <t>Kaplica Gąsieniców na Pęksowym Brzyzku pw. św. Andrzeja i św. Benedykta</t>
         </is>
       </c>
+      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
           <t>Drewniana kaplica z XIX wieku, najstarszy obiekt sakralny Zakopanego, położona na zabytkowym cmentarzu Pęksowym Brzyzku.</t>
@@ -14162,6 +14409,7 @@
           <t>To miejsce o wyjątkowym znaczeniu historycznym i kulturalnym, idealne dla osób chcących poznać początki Zakopanego i tradycje regionu. Cicha, klimatyczna kaplica i zabytkowy cmentarz tworzą niezwykłą przestrzeń do zadumy oraz spotkania z dziedzictwem Podhala.</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
           <t>{
@@ -14221,6 +14469,8 @@
       <c r="Q69" t="n">
         <v>19.9464968</v>
       </c>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr"/>
       <c r="T69" t="inlineStr">
         <is>
           <t>mixed</t>
@@ -14341,11 +14591,13 @@
       </c>
     </row>
     <row r="70">
+      <c r="A70" t="inlineStr"/>
       <c r="B70" t="inlineStr">
         <is>
           <t>Galeria Władysława Hasiora</t>
         </is>
       </c>
+      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
           <t>Galeria poświęcona twórczości Władysława Hasiora, wybitnego artysty i rzeźbiarza, będąca filią Muzeum Tatrzańskiego.</t>
@@ -14361,6 +14613,7 @@
           <t>To obowiązkowy punkt dla miłośników sztuki współczesnej oraz osób pragnących bliżej poznać sylwetkę i twórczość Władysława Hasiora, który w oryginalny sposób łączył kulturę ludową z nowoczesnością.</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>{
@@ -14539,11 +14792,13 @@
       </c>
     </row>
     <row r="71">
+      <c r="A71" t="inlineStr"/>
       <c r="B71" t="inlineStr">
         <is>
           <t>SkyWalk Serce Poronina</t>
         </is>
       </c>
+      <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
           <t>Platforma widokowa z panoramicznym widokiem na Tatry i okolice.</t>
@@ -14559,6 +14814,7 @@
           <t>Warto odwiedzić SkyWalk Serce Poronina, aby doświadczyć spektakularnych górskich widoków i zrobić pamiątkowe zdjęcia w wyjątkowym miejscu, które łączy nowoczesność z pięknem tatrzańskiej przyrody.</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>{
@@ -14770,11 +15026,13 @@
       </c>
     </row>
     <row r="72">
+      <c r="A72" t="inlineStr"/>
       <c r="B72" t="inlineStr">
         <is>
           <t>BeHappy Muzeum Zakopane</t>
         </is>
       </c>
+      <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
           <t>Interaktywne muzeum z kolorowymi instalacjami do zdjęć.</t>
@@ -14790,6 +15048,7 @@
           <t>Atrakcja oferuje mnóstwo radości, kreatywnych inspiracji i okazji do zrobienia unikalnych, wesołych zdjęć w ciekawie zaaranżowanych przestrzeniach.</t>
         </is>
       </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>{
@@ -14968,11 +15227,13 @@
       </c>
     </row>
     <row r="73">
+      <c r="A73" t="inlineStr"/>
       <c r="B73" t="inlineStr">
         <is>
           <t>Polana Szymoszkowa</t>
         </is>
       </c>
+      <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
           <t>Popularna stacja narciarska i rekreacyjna z pięknym widokiem na Tatry.</t>
@@ -14988,6 +15249,7 @@
           <t>To świetne miejsce zarówno dla miłośników sportów zimowych, jak i dla osób szukających relaksu w górach. Różnorodność atrakcji oraz piękne widoki sprawiają, że każdy znajdzie tu coś dla siebie.</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>{
@@ -15047,6 +15309,7 @@
       <c r="Q73" t="n">
         <v>19.9296709</v>
       </c>
+      <c r="R73" t="inlineStr"/>
       <c r="S73" t="inlineStr">
         <is>
           <t>https://szymoszkowa.pl/cennik-przejazdow-turystycznych/</t>
@@ -15172,11 +15435,13 @@
       </c>
     </row>
     <row r="74">
+      <c r="A74" t="inlineStr"/>
       <c r="B74" t="inlineStr">
         <is>
           <t>Królikarnia Zakopane</t>
         </is>
       </c>
+      <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
           <t>Małe prywatne mini-zoo w Zakopanem, w którym można zobaczyć króliki oraz inne drobne zwierzęta.</t>
@@ -15192,6 +15457,7 @@
           <t>To świetna opcja na relaksującą wizytę dla rodzin z dziećmi oraz miłośników zwierząt. Pozwala na bliski kontakt ze zwierzętami oraz odpoczynek w otoczeniu natury.</t>
         </is>
       </c>
+      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
           <t>{
@@ -15240,6 +15506,8 @@
       <c r="Q74" t="n">
         <v>19.9532834</v>
       </c>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr"/>
       <c r="T74" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -15360,11 +15628,13 @@
       </c>
     </row>
     <row r="75">
+      <c r="A75" t="inlineStr"/>
       <c r="B75" t="inlineStr">
         <is>
           <t>Kąpielisko na Polanie Szymoszkowej</t>
         </is>
       </c>
+      <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
           <t>Unikalny basen geotermalny z widokiem na Tatry.</t>
@@ -15380,6 +15650,7 @@
           <t>To idealne miejsce na odpoczynek po górskich wędrówkach, a przy tym świetna rozrywka dla całej rodziny w sercu Tatr.</t>
         </is>
       </c>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
           <t>{
@@ -15428,6 +15699,7 @@
       <c r="Q75" t="n">
         <v>19.9324219</v>
       </c>
+      <c r="R75" t="inlineStr"/>
       <c r="S75" t="inlineStr">
         <is>
           <t>https://szymoszkowa.pl/cennik-kapieliska/</t>
@@ -15553,11 +15825,13 @@
       </c>
     </row>
     <row r="76">
+      <c r="A76" t="inlineStr"/>
       <c r="B76" t="inlineStr">
         <is>
           <t>Bacówka zakopiańczyk</t>
         </is>
       </c>
+      <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr">
         <is>
           <t>Tradycyjna bacówka oferująca regionalne sery i produkty góralskie.</t>
@@ -15573,6 +15847,7 @@
           <t>Warto odwiedzić Bacówkę Zakopiańczyk, aby spróbować autentycznych serów z mleka owczego i doświadczyć żywej tradycji góralskiej. To idealne miejsce na zakup lokalnych przysmaków i oryginalnych pamiątek z regionu.</t>
         </is>
       </c>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>{
@@ -15621,6 +15896,8 @@
       <c r="Q76" t="n">
         <v>19.958669</v>
       </c>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr"/>
       <c r="T76" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -15662,6 +15939,7 @@
           <t>couples, seniors friends</t>
         </is>
       </c>
+      <c r="AC76" t="inlineStr"/>
       <c r="AD76" t="inlineStr">
         <is>
           <t>local_food_experience</t>
@@ -15736,11 +16014,13 @@
       </c>
     </row>
     <row r="77">
+      <c r="A77" t="inlineStr"/>
       <c r="B77" t="inlineStr">
         <is>
           <t>Dom Oscypka w Zakopanem</t>
         </is>
       </c>
+      <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr">
         <is>
           <t>Miejsce, gdzie można poznać tradycję wyrobu oscypka i wziąć udział w warsztatach na żywo.</t>
@@ -15756,6 +16036,7 @@
           <t>To idealne miejsce, aby lepiej poznać kulturę Podhala, spróbować tradycyjnych serów i zabrać do domu własnoręcznie zrobionego oscypka.</t>
         </is>
       </c>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
           <t>{
@@ -15804,6 +16085,8 @@
       <c r="Q77" t="n">
         <v>19.9549909</v>
       </c>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr"/>
       <c r="T77" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -15924,11 +16207,13 @@
       </c>
     </row>
     <row r="78">
+      <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr">
         <is>
           <t>Targowisko pod Gubałówką</t>
         </is>
       </c>
+      <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
           <t>Popularny bazar zlokalizowany u stóp Gubałówki w Zakopanem, oferujący lokalne produkty, pamiątki oraz wyroby regionalne.</t>
@@ -15944,6 +16229,7 @@
           <t>To idealne miejsce, by poczuć klimat Zakopanego, kupić regionalne przysmaki i oryginalne pamiątki oraz spotkać autentycznych producentów z Podhala.</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
           <t>{
@@ -15992,6 +16278,8 @@
       <c r="Q78" t="n">
         <v>19.9464494</v>
       </c>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
       <c r="T78" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -16033,6 +16321,7 @@
           <t>couples, seniors</t>
         </is>
       </c>
+      <c r="AC78" t="inlineStr"/>
       <c r="AD78" t="inlineStr">
         <is>
           <t>food_market</t>
@@ -16107,11 +16396,13 @@
       </c>
     </row>
     <row r="79">
+      <c r="A79" t="inlineStr"/>
       <c r="B79" t="inlineStr">
         <is>
           <t>Bachledówka</t>
         </is>
       </c>
+      <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
           <t>Bachledówka to malownicze wzniesienie niedaleko Zakopanego. Na szczycie znajduje się sanktuarium, a z okolicy można podziwiać piękne panoramy Tatr i Podhala.</t>
@@ -16127,6 +16418,7 @@
           <t>To idealne miejsce na chwilę odpoczynku i podziwianie górskich krajobrazów.</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
           <t>{
@@ -16175,6 +16467,8 @@
       <c r="Q79" t="n">
         <v>19.9192039620706</v>
       </c>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr"/>
       <c r="T79" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -16216,6 +16510,7 @@
           <t>seniors, couples</t>
         </is>
       </c>
+      <c r="AC79" t="inlineStr"/>
       <c r="AD79" t="inlineStr">
         <is>
           <t>nature_landscape</t>
@@ -16290,11 +16585,13 @@
       </c>
     </row>
     <row r="80">
+      <c r="A80" t="inlineStr"/>
       <c r="B80" t="inlineStr">
         <is>
           <t>Punkt widokowy na Antałówce</t>
         </is>
       </c>
+      <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
           <t>Punkt widokowy na Antałówce to spokojne miejsce w centrum Zakopanego z piękną panoramą Tatr. Idealne na krótki odpoczynek, zdjęcia lub piknik przy zachodzie słońca.</t>
@@ -16310,6 +16607,7 @@
           <t>Warto odwiedzić Antałówkę, by podziwiać piękne widoki na Tatry oraz miasto Zakopane.</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
           <t>{
@@ -16358,6 +16656,8 @@
       <c r="Q80" t="n">
         <v>19.9724934</v>
       </c>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr"/>
       <c r="T80" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -16484,11 +16784,13 @@
       </c>
     </row>
     <row r="81">
+      <c r="A81" t="inlineStr"/>
       <c r="B81" t="inlineStr">
         <is>
           <t>Tatrzańskie Archiwum Planety Ziemia</t>
         </is>
       </c>
+      <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
           <t>Nowoczesne centrum edukacyjne przybliżające faunę, florę i geologię Tatr.</t>
@@ -16504,6 +16806,7 @@
           <t>Miejsce idealne dla rodzin z dziećmi i osób zainteresowanych przyrodą Tatr. Pozwala w atrakcyjny sposób poznać unikatowy świat tatrzańskiej przyrody i przygotować się do wycieczek terenowych.</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
           <t>[
@@ -16565,6 +16868,8 @@
       <c r="Q81" t="n">
         <v>19.868302</v>
       </c>
+      <c r="R81" t="inlineStr"/>
+      <c r="S81" t="inlineStr"/>
       <c r="T81" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -16690,11 +16995,13 @@
       </c>
     </row>
     <row r="82">
+      <c r="A82" t="inlineStr"/>
       <c r="B82" t="inlineStr">
         <is>
           <t>Bachledzki Wierch</t>
         </is>
       </c>
+      <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
           <t>Bachledzki Wierch to widokowe wzniesienie położone w Zakopanem, popularne wśród spacerowiczów oraz turystów ceniących spokojne trasy i panoramę Tatr.</t>
@@ -16710,6 +17017,7 @@
           <t>Ze względu na rozległe widoki i mniej uczęszczane ścieżki, Bachledzki Wierch to doskonałe miejsce na spokojny spacer z dala od tłumów oraz na podziwianie panoramy Tatr i Zakopanego.</t>
         </is>
       </c>
+      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
           <t>{
@@ -16758,6 +17066,8 @@
       <c r="Q82" t="n">
         <v>19.9718091</v>
       </c>
+      <c r="R82" t="inlineStr"/>
+      <c r="S82" t="inlineStr"/>
       <c r="T82" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -16884,11 +17194,13 @@
       </c>
     </row>
     <row r="83">
+      <c r="A83" t="inlineStr"/>
       <c r="B83" t="inlineStr">
         <is>
           <t>Centrum Kultury Rodzimej w willi Czerwony Dwór</t>
         </is>
       </c>
+      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
           <t>Zabytkowa willa prezentująca sztukę i kulturę regionu Podhala.</t>
@@ -16904,6 +17216,7 @@
           <t>To wyjątkowe miejsce pozwalające poznać podhalańską sztukę, kulturę i architekturę w autentycznym otoczeniu historycznej willi.</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
           <t>{
@@ -16952,6 +17265,8 @@
       <c r="Q83" t="n">
         <v>19.9484177</v>
       </c>
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr"/>
       <c r="T83" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -16993,6 +17308,7 @@
           <t>seniors, solo</t>
         </is>
       </c>
+      <c r="AC83" t="inlineStr"/>
       <c r="AD83" t="inlineStr">
         <is>
           <t>museum_heritage</t>
@@ -17073,11 +17389,13 @@
       </c>
     </row>
     <row r="84">
+      <c r="A84" t="inlineStr"/>
       <c r="B84" t="inlineStr">
         <is>
           <t>Spływy Dunajcem tratwami flisackimi</t>
         </is>
       </c>
+      <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
           <t>Tradycyjne spływy tratwami przełomem Dunajca.</t>
@@ -17093,6 +17411,7 @@
           <t>Wyjątkowa okazja, by przeżyć tradycyjny, historyczny spływ z flisakami pośród spektakularnych krajobrazów Pienin. Biuro to punkt startowy dla tej niezapomnianej przygody.</t>
         </is>
       </c>
+      <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
           <t>[
@@ -17176,6 +17495,8 @@
       <c r="Q84" t="n">
         <v>20.368371</v>
       </c>
+      <c r="R84" t="inlineStr"/>
+      <c r="S84" t="inlineStr"/>
       <c r="T84" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -17286,7 +17607,7 @@
       </c>
       <c r="AR84" t="inlineStr">
         <is>
-          <t>history_mystery, legend_story, local_tradition, scenic_view, outdoor, family_friendly, rafting</t>
+          <t>river, rafting, sightseeing, scenic_views, family_friendly, outdoor, local_tradition</t>
         </is>
       </c>
       <c r="AS84" t="inlineStr">
@@ -17296,11 +17617,13 @@
       </c>
     </row>
     <row r="85">
+      <c r="A85" t="inlineStr"/>
       <c r="B85" t="inlineStr">
         <is>
           <t>Zamek w Niedzicy</t>
         </is>
       </c>
+      <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
           <t>Malowniczo położony średniowieczny zamek nad Jeziorem Czorsztyńskim.</t>
@@ -17316,6 +17639,7 @@
           <t>Zamek Dunajec to jeden z najważniejszych zabytków regionu, oferujący fascynującą podróż przez historię, piękne widoki i unikalną atmosferę średniowiecznej twierdzy.</t>
         </is>
       </c>
+      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t xml:space="preserve">
@@ -17379,6 +17703,8 @@
       <c r="Q85" t="n">
         <v>20.3196436</v>
       </c>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="inlineStr"/>
       <c r="T85" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -17489,7 +17815,7 @@
       </c>
       <c r="AR85" t="inlineStr">
         <is>
-          <t>history_mystery, local_history, legends, historic_building, regional_heritage, architecture_heritage, panoramic_view, sightseeing</t>
+          <t>castle, history, legends, architecture, panoramic_views, sightseeing</t>
         </is>
       </c>
       <c r="AS85" t="inlineStr">
@@ -17499,11 +17825,13 @@
       </c>
     </row>
     <row r="86">
+      <c r="A86" t="inlineStr"/>
       <c r="B86" t="inlineStr">
         <is>
           <t>Rejs statkiem po jeziorze Czorsztyńskim</t>
         </is>
       </c>
+      <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
           <t>Rejsy turystyczne po malowniczym jeziorze Czorsztyńskim ze wspaniałymi widokami na okoliczne zamki i Tatry.</t>
@@ -17519,6 +17847,7 @@
           <t>To wyjątkowa okazja, aby podziwiać naturę i zabytki regionu z pokładu statku oraz poczuć klimat górskiej przygody na wodzie.</t>
         </is>
       </c>
+      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>{
@@ -17567,6 +17896,8 @@
       <c r="Q86" t="n">
         <v>20.317104</v>
       </c>
+      <c r="R86" t="inlineStr"/>
+      <c r="S86" t="inlineStr"/>
       <c r="T86" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -17677,7 +18008,7 @@
       </c>
       <c r="AR86" t="inlineStr">
         <is>
-          <t>history_mystery, scenic_view, relaxation, sightseeing, family_friendly, boat_trip</t>
+          <t>boat_trip, lake, scenic_views, relaxation, sightseeing, family_friendly</t>
         </is>
       </c>
       <c r="AS86" t="inlineStr">
@@ -17687,11 +18018,13 @@
       </c>
     </row>
     <row r="87">
+      <c r="A87" t="inlineStr"/>
       <c r="B87" t="inlineStr">
         <is>
           <t>Zamek w Czorsztynie</t>
         </is>
       </c>
+      <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
           <t>Malownicze ruiny średniowiecznego zamku położone nad Jeziorem Czorsztyńskim.</t>
@@ -17707,6 +18040,7 @@
           <t>Zamek Czorsztyn to doskonałe miejsce zarówno dla miłośników historii, jak i osób spragnionych pięknych krajobrazów. Zwiedzanie ruin pozwala przenieść się w czasie, a rozciągające się wokół widoki pozostają na długo w pamięci.</t>
         </is>
       </c>
+      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
           <t>[
@@ -17768,6 +18102,8 @@
       <c r="Q87" t="n">
         <v>20.3132003</v>
       </c>
+      <c r="R87" t="inlineStr"/>
+      <c r="S87" t="inlineStr"/>
       <c r="T87" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -17878,7 +18214,7 @@
       </c>
       <c r="AR87" t="inlineStr">
         <is>
-          <t>history_mystery, historic_ruins, legends, local_history, historic_building, regional_heritage, architecture_heritage, panoramic_view</t>
+          <t>castle_ruins, history, legends, architecture, panoramic_views, sightseeing</t>
         </is>
       </c>
       <c r="AS87" t="inlineStr">
@@ -17888,11 +18224,13 @@
       </c>
     </row>
     <row r="88">
+      <c r="A88" t="inlineStr"/>
       <c r="B88" t="inlineStr">
         <is>
           <t>Wąwóz Homole</t>
         </is>
       </c>
+      <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
           <t>Malowniczy wąwóz skalny z krystalicznym potokiem i licznymi trasami spacerowymi.</t>
@@ -17908,6 +18246,7 @@
           <t>Wąwóz Homole zapewnia unikalne wrażenia krajobrazowe i bliskość natury, jest łatwo dostępny zarówno dla rodzin z dziećmi, jak i miłośników górskich wędrówek. Spacer przez wąwóz pozwala odpocząć od miejskiego zgiełku i odkryć bogatą faunę oraz florę regionu.</t>
         </is>
       </c>
+      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>{
@@ -17956,6 +18295,8 @@
       <c r="Q88" t="n">
         <v>20.548795</v>
       </c>
+      <c r="R88" t="inlineStr"/>
+      <c r="S88" t="inlineStr"/>
       <c r="T88" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -18066,7 +18407,7 @@
       </c>
       <c r="AR88" t="inlineStr">
         <is>
-          <t>hiking, nature_trail, scenic_view, mountains, outdoor, nature_landscape</t>
+          <t>gorge, hiking, nature, scenic_views, mountains, outdoor</t>
         </is>
       </c>
       <c r="AS88" t="inlineStr">
@@ -18076,11 +18417,13 @@
       </c>
     </row>
     <row r="89">
+      <c r="A89" t="inlineStr"/>
       <c r="B89" t="inlineStr">
         <is>
           <t>Bachledka Ski &amp; Sun</t>
         </is>
       </c>
+      <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
           <t>Nowoczesny ośrodek narciarski i całoroczny kompleks rekreacyjny u podnóża Tatr.</t>
@@ -18096,6 +18439,7 @@
           <t>To idealne miejsce na aktywny wypoczynek zarówno zimą, jak i latem. Oprócz sportów zimowych można tu spacerować w koronach drzew, podziwiać panoramę Tatr oraz korzystać z uroków lokalnej kuchni.</t>
         </is>
       </c>
+      <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
           <t>{
@@ -18144,6 +18488,8 @@
       <c r="Q89" t="n">
         <v>20.3099199</v>
       </c>
+      <c r="R89" t="inlineStr"/>
+      <c r="S89" t="inlineStr"/>
       <c r="T89" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -18254,7 +18600,7 @@
       </c>
       <c r="AR89" t="inlineStr">
         <is>
-          <t>cable_car, scenic_view, mountains, viewpoint, family_friendly, outdoor</t>
+          <t>viewpoint, cable_car, mountains, family_friendly, outdoor, scenic_views</t>
         </is>
       </c>
       <c r="AS89" t="inlineStr">
@@ -18264,11 +18610,13 @@
       </c>
     </row>
     <row r="90">
+      <c r="A90" t="inlineStr"/>
       <c r="B90" t="inlineStr">
         <is>
           <t>Jaskinia Bielańska</t>
         </is>
       </c>
+      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
           <t>Jedna z najpiękniejszych jaskiń Słowacji, znana z bogatej szaty naciekowej i podziemnych jezior.</t>
@@ -18284,6 +18632,7 @@
           <t>Odwiedź, by zobaczyć wyjątkowe formacje skalne i piękno podziemnego świata Tatr, a także poczuć niezwykły mikroklimat jaskini.</t>
         </is>
       </c>
+      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>{
@@ -18332,6 +18681,8 @@
       <c r="Q90" t="n">
         <v>20.3113339</v>
       </c>
+      <c r="R90" t="inlineStr"/>
+      <c r="S90" t="inlineStr"/>
       <c r="T90" t="inlineStr">
         <is>
           <t>indoor</t>
@@ -18442,7 +18793,7 @@
       </c>
       <c r="AR90" t="inlineStr">
         <is>
-          <t>history_mystery, underground_tour, cave, geology, educational_route, sightseeing, family_friendly</t>
+          <t>cave, underground, geology, nature, sightseeing, family_friendly</t>
         </is>
       </c>
       <c r="AS90" t="inlineStr">
@@ -18452,11 +18803,13 @@
       </c>
     </row>
     <row r="91">
+      <c r="A91" t="inlineStr"/>
       <c r="B91" t="inlineStr">
         <is>
           <t>Kolej Linowa na Palenicę</t>
         </is>
       </c>
+      <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
           <t>Kolej linowa prowadząca na szczyt Palenicy w Szczawnicy.</t>
@@ -18472,6 +18825,7 @@
           <t>To świetny sposób, aby w prosty sposób dostać się na szczyt Palenicy, skąd roztacza się panorama Pienin i okolic Szczawnicy. Atrakcja jest wygodna dla rodzin z dziećmi i osób mniej sprawnych.</t>
         </is>
       </c>
+      <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
           <t>{
@@ -18520,6 +18874,8 @@
       <c r="Q91" t="n">
         <v>20.480353</v>
       </c>
+      <c r="R91" t="inlineStr"/>
+      <c r="S91" t="inlineStr"/>
       <c r="T91" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -18630,7 +18986,7 @@
       </c>
       <c r="AR91" t="inlineStr">
         <is>
-          <t>cable_car, scenic_view, mountains, viewpoint, family_friendly, outdoor</t>
+          <t>cable_car, viewpoint, mountains, scenic_views, family_friendly</t>
         </is>
       </c>
       <c r="AS91" t="inlineStr">
@@ -18640,11 +18996,13 @@
       </c>
     </row>
     <row r="92">
+      <c r="A92" t="inlineStr"/>
       <c r="B92" t="inlineStr">
         <is>
           <t>Promenada nad Grajcarkiem</t>
         </is>
       </c>
+      <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
           <t>Malownicza promenada spacerowa wzdłuż rzeki Grajcarek w Szczawnicy.</t>
@@ -18660,6 +19018,7 @@
           <t>Warto się tu wybrać, aby podziwiać piękne widoki na Pieniny, zrelaksować się nad rzeką lub skorzystać z licznych ścieżek pieszych i rowerowych. To idealne miejsce na spokojny spacer lub rodzinny wypad na świeżym powietrzu.</t>
         </is>
       </c>
+      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>{
@@ -18708,6 +19067,8 @@
       <c r="Q92" t="n">
         <v>20.4744818</v>
       </c>
+      <c r="R92" t="inlineStr"/>
+      <c r="S92" t="inlineStr"/>
       <c r="T92" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -18818,7 +19179,7 @@
       </c>
       <c r="AR92" t="inlineStr">
         <is>
-          <t>walking, scenic_view, relaxation, riverside, family_friendly</t>
+          <t>walking, riverside, relaxation, scenic_views, family_friendly</t>
         </is>
       </c>
       <c r="AS92" t="inlineStr">
@@ -18828,11 +19189,13 @@
       </c>
     </row>
     <row r="93">
+      <c r="A93" t="inlineStr"/>
       <c r="B93" t="inlineStr">
         <is>
           <t>Plac Dietla</t>
         </is>
       </c>
+      <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
           <t>Historyczny plac będący centralnym punktem Szczawnicy.</t>
@@ -18848,6 +19211,7 @@
           <t>Odwiedź Plac Dietla, by poczuć klimat uzdrowiskowej Szczawnicy, podziwiać zabytkową architekturę i odpocząć wśród malowniczych scenerii. To idealne miejsce na spacer i relaks.</t>
         </is>
       </c>
+      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>{
@@ -18896,6 +19260,8 @@
       <c r="Q93" t="n">
         <v>20.4877223</v>
       </c>
+      <c r="R93" t="inlineStr"/>
+      <c r="S93" t="inlineStr"/>
       <c r="T93" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -18937,6 +19303,7 @@
           <t>couples, seniors, solo</t>
         </is>
       </c>
+      <c r="AC93" t="inlineStr"/>
       <c r="AD93" t="inlineStr">
         <is>
           <t>relaxation</t>
@@ -19001,7 +19368,7 @@
       </c>
       <c r="AR93" t="inlineStr">
         <is>
-          <t>history_mystery, historic_market_square, architecture_heritage, regional_heritage, relaxation, sightseeing</t>
+          <t>historic_center, architecture, spa_town, relaxation, sightseeing</t>
         </is>
       </c>
       <c r="AS93" t="inlineStr">
@@ -19011,11 +19378,13 @@
       </c>
     </row>
     <row r="94">
+      <c r="A94" t="inlineStr"/>
       <c r="B94" t="inlineStr">
         <is>
           <t>Zapora w Niedzicy</t>
         </is>
       </c>
+      <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
           <t>Potężna zapora wodna regulująca poziom wód Zbiornika Czorsztyńskiego.</t>
@@ -19031,6 +19400,7 @@
           <t>Warto odwiedzić zaporę, aby zobaczyć imponującą infrastrukturę hydrotechniczną, podziwiać malownicze krajobrazy i poznać znaczenie tego miejsca dla bezpieczeństwa regionu. To też świetne miejsce do spacerów i fotografii.</t>
         </is>
       </c>
+      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>{
@@ -19079,6 +19449,8 @@
       <c r="Q94" t="n">
         <v>20.3209667</v>
       </c>
+      <c r="R94" t="inlineStr"/>
+      <c r="S94" t="inlineStr"/>
       <c r="T94" t="inlineStr">
         <is>
           <t>outdoor</t>
@@ -19189,12 +19561,374 @@
       </c>
       <c r="AR94" t="inlineStr">
         <is>
-          <t>history_mystery, local_history, industrial_heritage, scenic_view, sightseeing, engineering</t>
+          <t>dam, engineering, lake, scenic_views, sightseeing, history</t>
         </is>
       </c>
       <c r="AS94" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr"/>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Jaskinia Mroźna</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Popularna jaskinia udostępniona do zwiedzania w Tatrach Zachodnich.</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Jaskinia Mroźna to jedna z najbardziej znanych jaskiń tatrzańskich dostępnych dla turystów. Znajduje się w Dolinie Kościeliskiej w Tatrach Zachodnich. Całkowita długość trasy udostępnionej do zwiedzania wynosi około 560 metrów. Jaskinia słynie ze specyficznego, chłodnego mikroklimatu oraz licznych nacieków i form skalnych. Zwiedza się ją z przewodnikiem, a trasa jest oświetlona elektrycznie.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>To wyjątkowa okazja, aby zobaczyć wnętrze tatrzańskiej jaskini i poczuć panujący tam chłód, nawet w środku lata. Jaskinia zachwyca licznymi formami naciekowymi i malowniczym położeniem w Dolinie Kościeliskiej.</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>{
+  "date_from": "04-26",
+  "date_to": "10-31",
+  "mon": "09:00-17:00",
+  "tue": "09:00-17:00",
+  "wed": "09:00-17:00",
+  "thu": "09:00-17:00",
+  "fri": "09:00-17:00",
+  "sat": "09:00-17:00",
+  "sun": "09:00-17:00"
+}</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>40</v>
+      </c>
+      <c r="J95" t="n">
+        <v>60</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Bilet wstępu: 11,00 zł</t>
+        </is>
+      </c>
+      <c r="L95" t="n">
+        <v>11</v>
+      </c>
+      <c r="M95" t="n">
+        <v>11</v>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>Kiry 26, 34-511 Kościelisko, Poland</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>Małopolska</t>
+        </is>
+      </c>
+      <c r="P95" t="n">
+        <v>49.2523126</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>19.8702975</v>
+      </c>
+      <c r="R95" t="inlineStr"/>
+      <c r="S95" t="inlineStr"/>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>indoor</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>good_weather_only</t>
+        </is>
+      </c>
+      <c r="W95" t="n">
+        <v>8</v>
+      </c>
+      <c r="X95" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>12:00-16:00</t>
+        </is>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>morning, midday, afternoon,</t>
+        </is>
+      </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>Kościelisko</t>
+        </is>
+      </c>
+      <c r="AB95" t="inlineStr"/>
+      <c r="AC95" t="inlineStr"/>
+      <c r="AD95" t="inlineStr">
+        <is>
+          <t>underground, nature_landscape</t>
+        </is>
+      </c>
+      <c r="AE95" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AF95" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AG95" t="inlineStr"/>
+      <c r="AH95" t="inlineStr">
+        <is>
+          <t>spring,summer,autumn</t>
+        </is>
+      </c>
+      <c r="AI95" t="inlineStr">
+        <is>
+          <t>Nawet latem weź ze sobą cieplejszą odzież – temperatura w jaskini wynosi około 6°C przez cały rok.</t>
+        </is>
+      </c>
+      <c r="AJ95" t="inlineStr">
+        <is>
+          <t>Parking Kościelisko</t>
+        </is>
+      </c>
+      <c r="AK95" t="inlineStr">
+        <is>
+          <t>Strzelców Podhalańskich 58, 43-229 Kościelisko</t>
+        </is>
+      </c>
+      <c r="AL95" t="n">
+        <v>49.27558803722384</v>
+      </c>
+      <c r="AM95" t="n">
+        <v>19.86921141644109</v>
+      </c>
+      <c r="AN95" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="AO95" t="n">
+        <v>43</v>
+      </c>
+      <c r="AP95" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="AQ95" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR95" t="inlineStr">
+        <is>
+          <t>cave, underground, karst-cave, nature, geology, mountain-adventure, hiking, tatra-mountains, exploration, sightseeing</t>
+        </is>
+      </c>
+      <c r="AS95" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr"/>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Jaskinia Raptawicka</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Jaskinia Raptawicka to jedna z bardziej znanych jaskiń w Tatrach, dostępna dla turystów o podstawowym przygotowaniu.</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Jaskinia Raptawicka, położona niedaleko Doliny Kościeliskiej w Tatrach, to popularne miejsce eksploracji dla miłośników przygód i natury. Długość jaskini to około 150 metrów, a jej zwiedzanie wymaga posiadania latarki oraz podstawowego przygotowania kondycyjnego, gdyż niektóre przejścia są wąskie i strome. Jaskinia zachwyca różnorodnością form krasowych, a także nietypowym mikroklimatem. Wejście do jaskini możliwe jest po pokonaniu kilkudziesięciu metrów podejścia ze ścieżki prowadzącej Doliną Kościeliską.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>To atrakcja dla osób poszukujących lekkiej dawki adrenaliny i bliskiego kontaktu z tatrzańską przyrodą. Oferuje wyjątkowe przeżycia oraz ciekawy sposób na poznawanie geologii Tatr.</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>{
+  "date_from": "04-26",
+  "date_to": "10-31",
+  "mon": "09:00-17:00",
+  "tue": "09:00-17:00",
+  "wed": "09:00-17:00",
+  "thu": "09:00-17:00",
+  "fri": "09:00-17:00",
+  "sat": "09:00-17:00",
+  "sun": "09:00-17:00"
+}</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>40</v>
+      </c>
+      <c r="J96" t="n">
+        <v>60</v>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Bilet wstępu: 11,00 zł</t>
+        </is>
+      </c>
+      <c r="L96" t="n">
+        <v>11</v>
+      </c>
+      <c r="M96" t="n">
+        <v>11</v>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>34-511 Kościelisko, Poland</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>Małopolska</t>
+        </is>
+      </c>
+      <c r="P96" t="n">
+        <v>49.2398334</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>19.8619837</v>
+      </c>
+      <c r="R96" t="inlineStr"/>
+      <c r="S96" t="inlineStr"/>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>outdoor,indoor</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>good_weather_only</t>
+        </is>
+      </c>
+      <c r="W96" t="n">
+        <v>6</v>
+      </c>
+      <c r="X96" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>12:00-16:00</t>
+        </is>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>morning, midday, afternoon,</t>
+        </is>
+      </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>Kościelisko</t>
+        </is>
+      </c>
+      <c r="AB96" t="inlineStr"/>
+      <c r="AC96" t="inlineStr"/>
+      <c r="AD96" t="inlineStr">
+        <is>
+          <t>underground, nature_landscape</t>
+        </is>
+      </c>
+      <c r="AE96" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AF96" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AG96" t="inlineStr"/>
+      <c r="AH96" t="inlineStr">
+        <is>
+          <t>spring,summer,autumn</t>
+        </is>
+      </c>
+      <c r="AI96" t="inlineStr">
+        <is>
+          <t>Zabierz ze sobą latarkę czołową i odpowiednie obuwie – wewnątrz bywa ślisko i ciemno.</t>
+        </is>
+      </c>
+      <c r="AJ96" t="inlineStr">
+        <is>
+          <t>Parking Kościelisko</t>
+        </is>
+      </c>
+      <c r="AK96" t="inlineStr">
+        <is>
+          <t>Strzelców Podhalańskich 58, 43-229 Kościelisko</t>
+        </is>
+      </c>
+      <c r="AL96" t="n">
+        <v>49.27558803722384</v>
+      </c>
+      <c r="AM96" t="n">
+        <v>19.86921141644109</v>
+      </c>
+      <c r="AN96" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="AO96" t="n">
+        <v>64</v>
+      </c>
+      <c r="AP96" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="AQ96" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR96" t="inlineStr">
+        <is>
+          <t>cave, underground, nature, geology, mountain-adventure, hiking, viewpoint, tatra-mountains, exploration, sightseeing</t>
+        </is>
+      </c>
+      <c r="AS96" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FIX #189: Zone A/B/C dla wszystkich miast, import atrakcje6 z Hub
Import Planer miasta atrakcje6 (721 POI, kolumna Zone). Filtr po City lub Hub umozliwia day-tripsy Zone C. Poprawki City przy imporcie i skrypt _import_atrakcje6.py.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/zakopane.xlsx
+++ b/data/zakopane.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS96"/>
+  <dimension ref="A1:AU96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -656,6 +656,16 @@
       <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Zone</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
         </is>
       </c>
     </row>
@@ -865,7 +875,7 @@
 </t>
         </is>
       </c>
-      <c r="AQ2" t="b">
+      <c r="AQ2" t="n">
         <v>0</v>
       </c>
       <c r="AR2" t="inlineStr">
@@ -876,6 +886,16 @@
       <c r="AS2" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>Muzeum Oscypka Zakopane</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1094,7 @@
 </t>
         </is>
       </c>
-      <c r="AQ3" t="b">
+      <c r="AQ3" t="n">
         <v>0</v>
       </c>
       <c r="AR3" t="inlineStr">
@@ -1085,6 +1105,16 @@
       <c r="AS3" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>Tatrzańskie Mini Zoo</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1312,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ4" t="b">
+      <c r="AQ4" t="n">
         <v>0</v>
       </c>
       <c r="AR4" t="inlineStr">
@@ -1293,6 +1323,16 @@
       <c r="AS4" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>Myszogród</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1531,7 @@
 secondary</t>
         </is>
       </c>
-      <c r="AQ5" t="b">
+      <c r="AQ5" t="n">
         <v>0</v>
       </c>
       <c r="AR5" t="inlineStr">
@@ -1502,6 +1542,16 @@
       <c r="AS5" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>Iluzja Park</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1749,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ6" t="b">
+      <c r="AQ6" t="n">
         <v>0</v>
       </c>
       <c r="AR6" t="inlineStr">
@@ -1710,6 +1760,16 @@
       <c r="AS6" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>Papugarnia Egzotyczne Zakopane</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1967,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ7" t="b">
+      <c r="AQ7" t="n">
         <v>0</v>
       </c>
       <c r="AR7" t="inlineStr">
@@ -1918,6 +1978,16 @@
       <c r="AS7" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>Podwodny Świat</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2185,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ8" t="b">
+      <c r="AQ8" t="n">
         <v>0</v>
       </c>
       <c r="AR8" t="inlineStr">
@@ -2126,6 +2196,16 @@
       <c r="AS8" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>Zjazd pontonem ze skoczni narciarskiej Wielka Krokiew</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2406,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ9" t="b">
+      <c r="AQ9" t="n">
         <v>0</v>
       </c>
       <c r="AR9" t="inlineStr">
@@ -2337,6 +2417,16 @@
       <c r="AS9" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>Góralski Ślizg</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2624,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ10" t="b">
+      <c r="AQ10" t="n">
         <v>0</v>
       </c>
       <c r="AR10" t="inlineStr">
@@ -2545,6 +2635,16 @@
       <c r="AS10" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>Tatra Family</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2841,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ11" t="b">
+      <c r="AQ11" t="n">
         <v>0</v>
       </c>
       <c r="AR11" t="inlineStr">
@@ -2752,6 +2852,16 @@
       <c r="AS11" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>Park Harnasia</t>
         </is>
       </c>
     </row>
@@ -2945,7 +3055,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ12" t="b">
+      <c r="AQ12" t="n">
         <v>0</v>
       </c>
       <c r="AR12" t="inlineStr">
@@ -2956,6 +3066,16 @@
       <c r="AS12" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>DINO PARK</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3272,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ13" t="b">
+      <c r="AQ13" t="n">
         <v>0</v>
       </c>
       <c r="AR13" t="inlineStr">
@@ -3163,6 +3283,16 @@
       <c r="AS13" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>Illusion House</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3489,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ14" t="b">
+      <c r="AQ14" t="n">
         <v>0</v>
       </c>
       <c r="AR14" t="inlineStr">
@@ -3370,6 +3500,16 @@
       <c r="AS14" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>Dom do góry nogami</t>
         </is>
       </c>
     </row>
@@ -3562,7 +3702,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ15" t="b">
+      <c r="AQ15" t="n">
         <v>1</v>
       </c>
       <c r="AR15" t="inlineStr">
@@ -3573,6 +3713,16 @@
       <c r="AS15" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>Plac zabaw na Górnej Równi Krupowej</t>
         </is>
       </c>
     </row>
@@ -3770,7 +3920,7 @@
 secondary</t>
         </is>
       </c>
-      <c r="AQ16" t="b">
+      <c r="AQ16" t="n">
         <v>0</v>
       </c>
       <c r="AR16" t="inlineStr">
@@ -3781,6 +3931,16 @@
       <c r="AS16" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>Termy Zakopiańskie</t>
         </is>
       </c>
     </row>
@@ -3978,7 +4138,7 @@
 secondary</t>
         </is>
       </c>
-      <c r="AQ17" t="b">
+      <c r="AQ17" t="n">
         <v>0</v>
       </c>
       <c r="AR17" t="inlineStr">
@@ -3989,6 +4149,16 @@
       <c r="AS17" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU17" t="inlineStr">
+        <is>
+          <t>Termy Gorący Potok</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4356,7 @@
 secondary</t>
         </is>
       </c>
-      <c r="AQ18" t="b">
+      <c r="AQ18" t="n">
         <v>0</v>
       </c>
       <c r="AR18" t="inlineStr">
@@ -4197,6 +4367,16 @@
       <c r="AS18" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>Chochołowskie Termy</t>
         </is>
       </c>
     </row>
@@ -4393,7 +4573,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ19" t="b">
+      <c r="AQ19" t="n">
         <v>0</v>
       </c>
       <c r="AR19" t="inlineStr">
@@ -4404,6 +4584,16 @@
       <c r="AS19" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU19" t="inlineStr">
+        <is>
+          <t>Terma Bania</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4791,7 @@
 secondary</t>
         </is>
       </c>
-      <c r="AQ20" t="b">
+      <c r="AQ20" t="n">
         <v>0</v>
       </c>
       <c r="AR20" t="inlineStr">
@@ -4612,6 +4802,16 @@
       <c r="AS20" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>Termy Bukovina</t>
         </is>
       </c>
     </row>
@@ -4808,7 +5008,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ21" t="b">
+      <c r="AQ21" t="n">
         <v>0</v>
       </c>
       <c r="AR21" t="inlineStr">
@@ -4819,6 +5019,16 @@
       <c r="AS21" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU21" t="inlineStr">
+        <is>
+          <t>Wielka Krokiew</t>
         </is>
       </c>
     </row>
@@ -5015,7 +5225,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ22" t="b">
+      <c r="AQ22" t="n">
         <v>0</v>
       </c>
       <c r="AR22" t="inlineStr">
@@ -5026,6 +5236,16 @@
       <c r="AS22" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU22" t="inlineStr">
+        <is>
+          <t>Centrum Edukacji Przyrodniczej Tatrzańskiego Parku Narodowego</t>
         </is>
       </c>
     </row>
@@ -5218,7 +5438,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ23" t="b">
+      <c r="AQ23" t="n">
         <v>0</v>
       </c>
       <c r="AR23" t="inlineStr">
@@ -5229,6 +5449,16 @@
       <c r="AS23" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU23" t="inlineStr">
+        <is>
+          <t>Wystawa Figur Woskowych EXPO Krupówki</t>
         </is>
       </c>
     </row>
@@ -5421,7 +5651,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ24" t="b">
+      <c r="AQ24" t="n">
         <v>0</v>
       </c>
       <c r="AR24" t="inlineStr">
@@ -5432,6 +5662,16 @@
       <c r="AS24" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU24" t="inlineStr">
+        <is>
+          <t>Wielka Wystawa Klocków LEGO</t>
         </is>
       </c>
     </row>
@@ -5623,7 +5863,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ25" t="b">
+      <c r="AQ25" t="n">
         <v>0</v>
       </c>
       <c r="AR25" t="inlineStr">
@@ -5634,6 +5874,16 @@
       <c r="AS25" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU25" t="inlineStr">
+        <is>
+          <t>Muzeum Tatrzańskie</t>
         </is>
       </c>
     </row>
@@ -5825,7 +6075,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ26" t="b">
+      <c r="AQ26" t="n">
         <v>0</v>
       </c>
       <c r="AR26" t="inlineStr">
@@ -5836,6 +6086,16 @@
       <c r="AS26" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU26" t="inlineStr">
+        <is>
+          <t>Muzeum Kornela Makuszyńskiego</t>
         </is>
       </c>
     </row>
@@ -6027,7 +6287,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ27" t="b">
+      <c r="AQ27" t="n">
         <v>0</v>
       </c>
       <c r="AR27" t="inlineStr">
@@ -6038,6 +6298,16 @@
       <c r="AS27" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU27" t="inlineStr">
+        <is>
+          <t>Muzeum Stylu Zakopiańskiego im. S. Witkiewicza</t>
         </is>
       </c>
     </row>
@@ -6229,7 +6499,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ28" t="b">
+      <c r="AQ28" t="n">
         <v>0</v>
       </c>
       <c r="AR28" t="inlineStr">
@@ -6240,6 +6510,16 @@
       <c r="AS28" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU28" t="inlineStr">
+        <is>
+          <t>Galeria sztuki w willi Oksza</t>
         </is>
       </c>
     </row>
@@ -6430,7 +6710,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ29" t="b">
+      <c r="AQ29" t="n">
         <v>0</v>
       </c>
       <c r="AR29" t="inlineStr">
@@ -6441,6 +6721,16 @@
       <c r="AS29" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU29" t="inlineStr">
+        <is>
+          <t>Muzeum Karola Szymanowskiego w willi "Atma"</t>
         </is>
       </c>
     </row>
@@ -6635,7 +6925,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ30" t="b">
+      <c r="AQ30" t="n">
         <v>0</v>
       </c>
       <c r="AR30" t="inlineStr">
@@ -6646,6 +6936,16 @@
       <c r="AS30" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU30" t="inlineStr">
+        <is>
+          <t>Tatrzański Park Edukacyjny</t>
         </is>
       </c>
     </row>
@@ -6838,7 +7138,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ31" t="b">
+      <c r="AQ31" t="n">
         <v>0</v>
       </c>
       <c r="AR31" t="inlineStr">
@@ -6849,6 +7149,16 @@
       <c r="AS31" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU31" t="inlineStr">
+        <is>
+          <t>Kaplica Najświętszego Serca Pana Jezusa w Jaszczurówce</t>
         </is>
       </c>
     </row>
@@ -7052,7 +7362,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ32" t="b">
+      <c r="AQ32" t="n">
         <v>0</v>
       </c>
       <c r="AR32" t="inlineStr">
@@ -7063,6 +7373,16 @@
       <c r="AS32" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU32" t="inlineStr">
+        <is>
+          <t>KULIGI w Zakopanem</t>
         </is>
       </c>
     </row>
@@ -7268,7 +7588,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ33" t="b">
+      <c r="AQ33" t="n">
         <v>0</v>
       </c>
       <c r="AR33" t="inlineStr">
@@ -7279,6 +7599,16 @@
       <c r="AS33" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU33" t="inlineStr">
+        <is>
+          <t>Dolina Chochołowska</t>
         </is>
       </c>
     </row>
@@ -7485,7 +7815,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ34" t="b">
+      <c r="AQ34" t="n">
         <v>0</v>
       </c>
       <c r="AR34" t="inlineStr">
@@ -7496,6 +7826,16 @@
       <c r="AS34" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU34" t="inlineStr">
+        <is>
+          <t>Dolina Kościeliska</t>
         </is>
       </c>
     </row>
@@ -7702,7 +8042,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ35" t="b">
+      <c r="AQ35" t="n">
         <v>0</v>
       </c>
       <c r="AR35" t="inlineStr">
@@ -7713,6 +8053,16 @@
       <c r="AS35" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU35" t="inlineStr">
+        <is>
+          <t>Rusinowa Polana</t>
         </is>
       </c>
     </row>
@@ -7919,7 +8269,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ36" t="b">
+      <c r="AQ36" t="n">
         <v>0</v>
       </c>
       <c r="AR36" t="inlineStr">
@@ -7930,6 +8280,16 @@
       <c r="AS36" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT36" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU36" t="inlineStr">
+        <is>
+          <t>Morskie Oko</t>
         </is>
       </c>
     </row>
@@ -8112,7 +8472,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ37" t="b">
+      <c r="AQ37" t="n">
         <v>0</v>
       </c>
       <c r="AR37" t="inlineStr">
@@ -8123,6 +8483,16 @@
       <c r="AS37" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU37" t="inlineStr">
+        <is>
+          <t>Gubałówka</t>
         </is>
       </c>
     </row>
@@ -8306,7 +8676,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ38" t="b">
+      <c r="AQ38" t="n">
         <v>0</v>
       </c>
       <c r="AR38" t="inlineStr">
@@ -8317,6 +8687,16 @@
       <c r="AS38" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT38" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU38" t="inlineStr">
+        <is>
+          <t>Snowdoo Adventure</t>
         </is>
       </c>
     </row>
@@ -8551,7 +8931,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ39" t="b">
+      <c r="AQ39" t="n">
         <v>0</v>
       </c>
       <c r="AR39" t="inlineStr">
@@ -8562,6 +8942,16 @@
       <c r="AS39" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT39" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kolejka linowa na Kasprowy Wierch </t>
         </is>
       </c>
     </row>
@@ -8755,7 +9145,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ40" t="b">
+      <c r="AQ40" t="n">
         <v>0</v>
       </c>
       <c r="AR40" t="inlineStr">
@@ -8766,6 +9156,16 @@
       <c r="AS40" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT40" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU40" t="inlineStr">
+        <is>
+          <t>Droga pod Reglami</t>
         </is>
       </c>
     </row>
@@ -8959,7 +9359,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ41" t="b">
+      <c r="AQ41" t="n">
         <v>0</v>
       </c>
       <c r="AR41" t="inlineStr">
@@ -8970,6 +9370,16 @@
       <c r="AS41" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT41" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU41" t="inlineStr">
+        <is>
+          <t>Dolina Strążyska</t>
         </is>
       </c>
     </row>
@@ -9163,7 +9573,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ42" t="b">
+      <c r="AQ42" t="n">
         <v>0</v>
       </c>
       <c r="AR42" t="inlineStr">
@@ -9174,6 +9584,16 @@
       <c r="AS42" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT42" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU42" t="inlineStr">
+        <is>
+          <t>Dolina ku Dziurze</t>
         </is>
       </c>
     </row>
@@ -9367,7 +9787,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ43" t="b">
+      <c r="AQ43" t="n">
         <v>0</v>
       </c>
       <c r="AR43" t="inlineStr">
@@ -9378,6 +9798,16 @@
       <c r="AS43" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT43" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU43" t="inlineStr">
+        <is>
+          <t>Polana Kalatówki</t>
         </is>
       </c>
     </row>
@@ -9571,7 +10001,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ44" t="b">
+      <c r="AQ44" t="n">
         <v>0</v>
       </c>
       <c r="AR44" t="inlineStr">
@@ -9582,6 +10012,16 @@
       <c r="AS44" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT44" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU44" t="inlineStr">
+        <is>
+          <t>Punkt widokowy na Tatry</t>
         </is>
       </c>
     </row>
@@ -9775,7 +10215,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ45" t="b">
+      <c r="AQ45" t="n">
         <v>0</v>
       </c>
       <c r="AR45" t="inlineStr">
@@ -9786,6 +10226,16 @@
       <c r="AS45" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT45" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU45" t="inlineStr">
+        <is>
+          <t>Wodospad Siklawica</t>
         </is>
       </c>
     </row>
@@ -9979,7 +10429,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ46" t="b">
+      <c r="AQ46" t="n">
         <v>0</v>
       </c>
       <c r="AR46" t="inlineStr">
@@ -9990,6 +10440,16 @@
       <c r="AS46" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT46" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU46" t="inlineStr">
+        <is>
+          <t>Olczyska Polana</t>
         </is>
       </c>
     </row>
@@ -10183,7 +10643,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ47" t="b">
+      <c r="AQ47" t="n">
         <v>0</v>
       </c>
       <c r="AR47" t="inlineStr">
@@ -10194,6 +10654,16 @@
       <c r="AS47" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT47" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU47" t="inlineStr">
+        <is>
+          <t>Polana Jaworzynka</t>
         </is>
       </c>
     </row>
@@ -10387,7 +10857,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ48" t="b">
+      <c r="AQ48" t="n">
         <v>0</v>
       </c>
       <c r="AR48" t="inlineStr">
@@ -10398,6 +10868,16 @@
       <c r="AS48" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT48" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU48" t="inlineStr">
+        <is>
+          <t>Sarni Wodospad</t>
         </is>
       </c>
     </row>
@@ -10591,7 +11071,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ49" t="b">
+      <c r="AQ49" t="n">
         <v>0</v>
       </c>
       <c r="AR49" t="inlineStr">
@@ -10602,6 +11082,16 @@
       <c r="AS49" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT49" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU49" t="inlineStr">
+        <is>
+          <t>Wielka Polana Małołącka</t>
         </is>
       </c>
     </row>
@@ -10795,7 +11285,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ50" t="b">
+      <c r="AQ50" t="n">
         <v>0</v>
       </c>
       <c r="AR50" t="inlineStr">
@@ -10806,6 +11296,16 @@
       <c r="AS50" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT50" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU50" t="inlineStr">
+        <is>
+          <t>Dolina Za Bramką</t>
         </is>
       </c>
     </row>
@@ -10999,7 +11499,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ51" t="b">
+      <c r="AQ51" t="n">
         <v>0</v>
       </c>
       <c r="AR51" t="inlineStr">
@@ -11010,6 +11510,16 @@
       <c r="AS51" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT51" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU51" t="inlineStr">
+        <is>
+          <t>Dolina Suchej Wody</t>
         </is>
       </c>
     </row>
@@ -11203,7 +11713,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ52" t="b">
+      <c r="AQ52" t="n">
         <v>0</v>
       </c>
       <c r="AR52" t="inlineStr">
@@ -11214,6 +11724,16 @@
       <c r="AS52" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT52" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU52" t="inlineStr">
+        <is>
+          <t>Dolina Gąsienicowa</t>
         </is>
       </c>
     </row>
@@ -11407,7 +11927,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ53" t="b">
+      <c r="AQ53" t="n">
         <v>0</v>
       </c>
       <c r="AR53" t="inlineStr">
@@ -11418,6 +11938,16 @@
       <c r="AS53" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT53" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU53" t="inlineStr">
+        <is>
+          <t>Park Miejski im. Marszałka Józefa Piłsudskiego</t>
         </is>
       </c>
     </row>
@@ -11600,7 +12130,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ54" t="b">
+      <c r="AQ54" t="n">
         <v>0</v>
       </c>
       <c r="AR54" t="inlineStr">
@@ -11611,6 +12141,16 @@
       <c r="AS54" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT54" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU54" t="inlineStr">
+        <is>
+          <t>Chałupa Sabały</t>
         </is>
       </c>
     </row>
@@ -11793,7 +12333,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ55" t="b">
+      <c r="AQ55" t="n">
         <v>0</v>
       </c>
       <c r="AR55" t="inlineStr">
@@ -11804,6 +12344,16 @@
       <c r="AS55" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT55" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU55" t="inlineStr">
+        <is>
+          <t>Quady Adventure Zakopane Wypożyczalnia</t>
         </is>
       </c>
     </row>
@@ -11993,7 +12543,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ56" t="b">
+      <c r="AQ56" t="n">
         <v>0</v>
       </c>
       <c r="AR56" t="inlineStr">
@@ -12004,6 +12554,16 @@
       <c r="AS56" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT56" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU56" t="inlineStr">
+        <is>
+          <t>Cudakowa Polana</t>
         </is>
       </c>
     </row>
@@ -12186,7 +12746,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ57" t="b">
+      <c r="AQ57" t="n">
         <v>0</v>
       </c>
       <c r="AR57" t="inlineStr">
@@ -12197,6 +12757,16 @@
       <c r="AS57" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT57" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Beernarium Piwne Spa</t>
         </is>
       </c>
     </row>
@@ -12387,7 +12957,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ58" t="b">
+      <c r="AQ58" t="n">
         <v>0</v>
       </c>
       <c r="AR58" t="inlineStr">
@@ -12398,6 +12968,16 @@
       <c r="AS58" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT58" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU58" t="inlineStr">
+        <is>
+          <t>Iria Spa</t>
         </is>
       </c>
     </row>
@@ -12591,7 +13171,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ59" t="b">
+      <c r="AQ59" t="n">
         <v>0</v>
       </c>
       <c r="AR59" t="inlineStr">
@@ -12602,6 +13182,16 @@
       <c r="AS59" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT59" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU59" t="inlineStr">
+        <is>
+          <t>Polana Głodówka</t>
         </is>
       </c>
     </row>
@@ -12788,7 +13378,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ60" t="b">
+      <c r="AQ60" t="n">
         <v>0</v>
       </c>
       <c r="AR60" t="inlineStr">
@@ -12799,6 +13389,16 @@
       <c r="AS60" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT60" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU60" t="inlineStr">
+        <is>
+          <t>Park Przygody Gubałówka</t>
         </is>
       </c>
     </row>
@@ -12981,7 +13581,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ61" t="b">
+      <c r="AQ61" t="n">
         <v>0</v>
       </c>
       <c r="AR61" t="inlineStr">
@@ -12992,6 +13592,16 @@
       <c r="AS61" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT61" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU61" t="inlineStr">
+        <is>
+          <t>Cmentarz Zasłużonych na Pęksowym Brzyzku</t>
         </is>
       </c>
     </row>
@@ -13174,7 +13784,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ62" t="b">
+      <c r="AQ62" t="n">
         <v>0</v>
       </c>
       <c r="AR62" t="inlineStr">
@@ -13185,6 +13795,16 @@
       <c r="AS62" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT62" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU62" t="inlineStr">
+        <is>
+          <t>Dwór Tetmajerów</t>
         </is>
       </c>
     </row>
@@ -13367,7 +13987,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ63" t="b">
+      <c r="AQ63" t="n">
         <v>0</v>
       </c>
       <c r="AR63" t="inlineStr">
@@ -13378,6 +13998,16 @@
       <c r="AS63" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT63" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU63" t="inlineStr">
+        <is>
+          <t>Sanktuarium Wiktorówki</t>
         </is>
       </c>
     </row>
@@ -13557,7 +14187,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ64" t="b">
+      <c r="AQ64" t="n">
         <v>1</v>
       </c>
       <c r="AR64" t="inlineStr">
@@ -13568,6 +14198,16 @@
       <c r="AS64" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT64" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU64" t="inlineStr">
+        <is>
+          <t>Snow Zabawa – zimowe atrakcje</t>
         </is>
       </c>
     </row>
@@ -13758,7 +14398,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ65" t="b">
+      <c r="AQ65" t="n">
         <v>0</v>
       </c>
       <c r="AR65" t="inlineStr">
@@ -13773,6 +14413,16 @@
       <c r="AS65" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT65" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU65" t="inlineStr">
+        <is>
+          <t>Krupówki</t>
         </is>
       </c>
     </row>
@@ -13966,7 +14616,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ66" t="b">
+      <c r="AQ66" t="n">
         <v>0</v>
       </c>
       <c r="AR66" t="inlineStr">
@@ -13981,6 +14631,16 @@
       <c r="AS66" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT66" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU66" t="inlineStr">
+        <is>
+          <t>Dolna Rówień Krupowa</t>
         </is>
       </c>
     </row>
@@ -14171,7 +14831,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ67" t="b">
+      <c r="AQ67" t="n">
         <v>0</v>
       </c>
       <c r="AR67" t="inlineStr">
@@ -14182,6 +14842,16 @@
       <c r="AS67" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT67" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU67" t="inlineStr">
+        <is>
+          <t>Muzeum Jana Kasprowicza</t>
         </is>
       </c>
     </row>
@@ -14372,7 +15042,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ68" t="b">
+      <c r="AQ68" t="n">
         <v>0</v>
       </c>
       <c r="AR68" t="inlineStr">
@@ -14383,6 +15053,16 @@
       <c r="AS68" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT68" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU68" t="inlineStr">
+        <is>
+          <t>Willa Koliba</t>
         </is>
       </c>
     </row>
@@ -14576,7 +15256,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ69" t="b">
+      <c r="AQ69" t="n">
         <v>0</v>
       </c>
       <c r="AR69" t="inlineStr">
@@ -14587,6 +15267,16 @@
       <c r="AS69" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT69" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU69" t="inlineStr">
+        <is>
+          <t>Kaplica Gąsieniców na Pęksowym Brzyzku pw. św. Andrzeja i św. Benedykta</t>
         </is>
       </c>
     </row>
@@ -14777,7 +15467,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ70" t="b">
+      <c r="AQ70" t="n">
         <v>0</v>
       </c>
       <c r="AR70" t="inlineStr">
@@ -14788,6 +15478,16 @@
       <c r="AS70" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT70" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU70" t="inlineStr">
+        <is>
+          <t>Galeria Władysława Hasiora</t>
         </is>
       </c>
     </row>
@@ -15011,7 +15711,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ71" t="b">
+      <c r="AQ71" t="n">
         <v>0</v>
       </c>
       <c r="AR71" t="inlineStr">
@@ -15022,6 +15722,16 @@
       <c r="AS71" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT71" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU71" t="inlineStr">
+        <is>
+          <t>SkyWalk Serce Poronina</t>
         </is>
       </c>
     </row>
@@ -15212,7 +15922,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ72" t="b">
+      <c r="AQ72" t="n">
         <v>0</v>
       </c>
       <c r="AR72" t="inlineStr">
@@ -15223,6 +15933,16 @@
       <c r="AS72" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT72" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU72" t="inlineStr">
+        <is>
+          <t>BeHappy Muzeum Zakopane</t>
         </is>
       </c>
     </row>
@@ -15420,7 +16140,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ73" t="b">
+      <c r="AQ73" t="n">
         <v>0</v>
       </c>
       <c r="AR73" t="inlineStr">
@@ -15431,6 +16151,16 @@
       <c r="AS73" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT73" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU73" t="inlineStr">
+        <is>
+          <t>Polana Szymoszkowa</t>
         </is>
       </c>
     </row>
@@ -15613,7 +16343,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ74" t="b">
+      <c r="AQ74" t="n">
         <v>0</v>
       </c>
       <c r="AR74" t="inlineStr">
@@ -15624,6 +16354,16 @@
       <c r="AS74" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT74" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU74" t="inlineStr">
+        <is>
+          <t>Królikarnia Zakopane</t>
         </is>
       </c>
     </row>
@@ -15810,7 +16550,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ75" t="b">
+      <c r="AQ75" t="n">
         <v>0</v>
       </c>
       <c r="AR75" t="inlineStr">
@@ -15821,6 +16561,16 @@
       <c r="AS75" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT75" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU75" t="inlineStr">
+        <is>
+          <t>Kąpielisko na Polanie Szymoszkowej</t>
         </is>
       </c>
     </row>
@@ -15999,7 +16749,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ76" t="b">
+      <c r="AQ76" t="n">
         <v>0</v>
       </c>
       <c r="AR76" t="inlineStr">
@@ -16010,6 +16760,16 @@
       <c r="AS76" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT76" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU76" t="inlineStr">
+        <is>
+          <t>Bacówka zakopiańczyk</t>
         </is>
       </c>
     </row>
@@ -16192,7 +16952,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ77" t="b">
+      <c r="AQ77" t="n">
         <v>0</v>
       </c>
       <c r="AR77" t="inlineStr">
@@ -16203,6 +16963,16 @@
       <c r="AS77" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT77" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU77" t="inlineStr">
+        <is>
+          <t>Dom Oscypka w Zakopanem</t>
         </is>
       </c>
     </row>
@@ -16381,7 +17151,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ78" t="b">
+      <c r="AQ78" t="n">
         <v>0</v>
       </c>
       <c r="AR78" t="inlineStr">
@@ -16392,6 +17162,16 @@
       <c r="AS78" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT78" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU78" t="inlineStr">
+        <is>
+          <t>Targowisko pod Gubałówką</t>
         </is>
       </c>
     </row>
@@ -16570,7 +17350,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ79" t="b">
+      <c r="AQ79" t="n">
         <v>0</v>
       </c>
       <c r="AR79" t="inlineStr">
@@ -16581,6 +17361,16 @@
       <c r="AS79" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT79" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU79" t="inlineStr">
+        <is>
+          <t>Bachledówka</t>
         </is>
       </c>
     </row>
@@ -16763,7 +17553,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ80" t="b">
+      <c r="AQ80" t="n">
         <v>0</v>
       </c>
       <c r="AR80" t="inlineStr">
@@ -16780,6 +17570,16 @@
       <c r="AS80" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT80" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU80" t="inlineStr">
+        <is>
+          <t>Punkt widokowy na Antałówce</t>
         </is>
       </c>
     </row>
@@ -16975,7 +17775,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ81" t="b">
+      <c r="AQ81" t="n">
         <v>0</v>
       </c>
       <c r="AR81" t="inlineStr">
@@ -16991,6 +17791,16 @@
       <c r="AS81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT81" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU81" t="inlineStr">
+        <is>
+          <t>Tatrzańskie Archiwum Planety Ziemia</t>
         </is>
       </c>
     </row>
@@ -17173,7 +17983,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ82" t="b">
+      <c r="AQ82" t="n">
         <v>0</v>
       </c>
       <c r="AR82" t="inlineStr">
@@ -17190,6 +18000,16 @@
       <c r="AS82" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="AT82" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU82" t="inlineStr">
+        <is>
+          <t>Bachledzki Wierch</t>
         </is>
       </c>
     </row>
@@ -17368,7 +18188,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ83" t="b">
+      <c r="AQ83" t="n">
         <v>0</v>
       </c>
       <c r="AR83" t="inlineStr">
@@ -17385,6 +18205,16 @@
       <c r="AS83" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT83" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU83" t="inlineStr">
+        <is>
+          <t>Centrum Kultury Rodzimej w willi Czerwony Dwór</t>
         </is>
       </c>
     </row>
@@ -17602,7 +18432,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ84" t="b">
+      <c r="AQ84" t="n">
         <v>0</v>
       </c>
       <c r="AR84" t="inlineStr">
@@ -17613,6 +18443,16 @@
       <c r="AS84" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT84" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU84" t="inlineStr">
+        <is>
+          <t>Spływy Dunajcem tratwami flisackimi</t>
         </is>
       </c>
     </row>
@@ -17810,7 +18650,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ85" t="b">
+      <c r="AQ85" t="n">
         <v>0</v>
       </c>
       <c r="AR85" t="inlineStr">
@@ -17821,6 +18661,16 @@
       <c r="AS85" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT85" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU85" t="inlineStr">
+        <is>
+          <t>Zamek w Niedzicy</t>
         </is>
       </c>
     </row>
@@ -18003,7 +18853,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ86" t="b">
+      <c r="AQ86" t="n">
         <v>0</v>
       </c>
       <c r="AR86" t="inlineStr">
@@ -18014,6 +18864,16 @@
       <c r="AS86" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT86" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU86" t="inlineStr">
+        <is>
+          <t>Rejs statkiem po jeziorze Czorsztyńskim</t>
         </is>
       </c>
     </row>
@@ -18209,7 +19069,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ87" t="b">
+      <c r="AQ87" t="n">
         <v>0</v>
       </c>
       <c r="AR87" t="inlineStr">
@@ -18220,6 +19080,16 @@
       <c r="AS87" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT87" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU87" t="inlineStr">
+        <is>
+          <t>Zamek w Czorsztynie</t>
         </is>
       </c>
     </row>
@@ -18402,7 +19272,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ88" t="b">
+      <c r="AQ88" t="n">
         <v>0</v>
       </c>
       <c r="AR88" t="inlineStr">
@@ -18413,6 +19283,16 @@
       <c r="AS88" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT88" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU88" t="inlineStr">
+        <is>
+          <t>Wąwóz Homole</t>
         </is>
       </c>
     </row>
@@ -18595,7 +19475,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ89" t="b">
+      <c r="AQ89" t="n">
         <v>0</v>
       </c>
       <c r="AR89" t="inlineStr">
@@ -18606,6 +19486,16 @@
       <c r="AS89" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT89" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU89" t="inlineStr">
+        <is>
+          <t>Bachledka Ski &amp; Sun</t>
         </is>
       </c>
     </row>
@@ -18788,7 +19678,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ90" t="b">
+      <c r="AQ90" t="n">
         <v>0</v>
       </c>
       <c r="AR90" t="inlineStr">
@@ -18799,6 +19689,16 @@
       <c r="AS90" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT90" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU90" t="inlineStr">
+        <is>
+          <t>Jaskinia Bielańska</t>
         </is>
       </c>
     </row>
@@ -18981,7 +19881,7 @@
           <t>core</t>
         </is>
       </c>
-      <c r="AQ91" t="b">
+      <c r="AQ91" t="n">
         <v>0</v>
       </c>
       <c r="AR91" t="inlineStr">
@@ -18992,6 +19892,16 @@
       <c r="AS91" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT91" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU91" t="inlineStr">
+        <is>
+          <t>Kolej Linowa na Palenicę</t>
         </is>
       </c>
     </row>
@@ -19174,7 +20084,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ92" t="b">
+      <c r="AQ92" t="n">
         <v>0</v>
       </c>
       <c r="AR92" t="inlineStr">
@@ -19185,6 +20095,16 @@
       <c r="AS92" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT92" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU92" t="inlineStr">
+        <is>
+          <t>Promenada nad Grajcarkiem</t>
         </is>
       </c>
     </row>
@@ -19363,7 +20283,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="AQ93" t="b">
+      <c r="AQ93" t="n">
         <v>0</v>
       </c>
       <c r="AR93" t="inlineStr">
@@ -19374,6 +20294,16 @@
       <c r="AS93" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT93" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU93" t="inlineStr">
+        <is>
+          <t>Plac Dietla</t>
         </is>
       </c>
     </row>
@@ -19556,7 +20486,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ94" t="b">
+      <c r="AQ94" t="n">
         <v>0</v>
       </c>
       <c r="AR94" t="inlineStr">
@@ -19567,6 +20497,16 @@
       <c r="AS94" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="AT94" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU94" t="inlineStr">
+        <is>
+          <t>Zapora w Niedzicy</t>
         </is>
       </c>
     </row>
@@ -19680,8 +20620,16 @@
           <t>Kościelisko</t>
         </is>
       </c>
-      <c r="AB95" t="inlineStr"/>
-      <c r="AC95" t="inlineStr"/>
+      <c r="AB95" t="inlineStr">
+        <is>
+          <t>couples, friends, family_kids, solo</t>
+        </is>
+      </c>
+      <c r="AC95" t="inlineStr">
+        <is>
+          <t>6-10, 10-14</t>
+        </is>
+      </c>
       <c r="AD95" t="inlineStr">
         <is>
           <t>underground, nature_landscape</t>
@@ -19697,7 +20645,11 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="AG95" t="inlineStr"/>
+      <c r="AG95" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
       <c r="AH95" t="inlineStr">
         <is>
           <t>spring,summer,autumn</t>
@@ -19737,7 +20689,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ95" t="b">
+      <c r="AQ95" t="n">
         <v>0</v>
       </c>
       <c r="AR95" t="inlineStr">
@@ -19748,6 +20700,16 @@
       <c r="AS95" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT95" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU95" t="inlineStr">
+        <is>
+          <t>Jaskinia Mroźna</t>
         </is>
       </c>
     </row>
@@ -19861,8 +20823,16 @@
           <t>Kościelisko</t>
         </is>
       </c>
-      <c r="AB96" t="inlineStr"/>
-      <c r="AC96" t="inlineStr"/>
+      <c r="AB96" t="inlineStr">
+        <is>
+          <t>couples, friends, solo</t>
+        </is>
+      </c>
+      <c r="AC96" t="inlineStr">
+        <is>
+          <t>6-10, 10-14</t>
+        </is>
+      </c>
       <c r="AD96" t="inlineStr">
         <is>
           <t>underground, nature_landscape</t>
@@ -19878,7 +20848,11 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="AG96" t="inlineStr"/>
+      <c r="AG96" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
       <c r="AH96" t="inlineStr">
         <is>
           <t>spring,summer,autumn</t>
@@ -19918,7 +20892,7 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="AQ96" t="b">
+      <c r="AQ96" t="n">
         <v>0</v>
       </c>
       <c r="AR96" t="inlineStr">
@@ -19929,6 +20903,16 @@
       <c r="AS96" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="AT96" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AU96" t="inlineStr">
+        <is>
+          <t>Jaskinia Raptawicka</t>
         </is>
       </c>
     </row>

</xml_diff>